<commit_message>
Atualização de dados — 29/09/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -98,12 +98,12 @@
     <t>Munhoz De Melo</t>
   </si>
   <si>
+    <t>Astorga</t>
+  </si>
+  <si>
     <t>Lobato</t>
   </si>
   <si>
-    <t>Astorga</t>
-  </si>
-  <si>
     <t>Floresta</t>
   </si>
   <si>
@@ -143,12 +143,12 @@
     <t>Obesidade</t>
   </si>
   <si>
+    <t>Diabetes</t>
+  </si>
+  <si>
     <t>Cardiopatia</t>
   </si>
   <si>
-    <t>Diabetes</t>
-  </si>
-  <si>
     <t>Imunodepressão</t>
   </si>
   <si>
@@ -257,10 +257,10 @@
     <t>Laboratorial</t>
   </si>
   <si>
+    <t>Clínico-Imagem</t>
+  </si>
+  <si>
     <t>Não informado</t>
-  </si>
-  <si>
-    <t>Clínico-Imagem</t>
   </si>
   <si>
     <t>antiviral_label</t>
@@ -658,7 +658,7 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C2">
         <v>9</v>
@@ -667,16 +667,16 @@
         <v>4</v>
       </c>
       <c r="E2">
-        <v>372.1</v>
+        <v>386.9</v>
       </c>
       <c r="F2">
         <v>33.2</v>
       </c>
       <c r="G2">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -866,25 +866,25 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>907</v>
+        <v>931</v>
       </c>
       <c r="C10">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D10">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="E10">
-        <v>211.1</v>
+        <v>216.7</v>
       </c>
       <c r="F10">
-        <v>16.8</v>
+        <v>17.2</v>
       </c>
       <c r="G10">
         <v>7.9</v>
       </c>
       <c r="H10">
-        <v>28.8</v>
+        <v>28.9</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -892,7 +892,7 @@
         <v>17</v>
       </c>
       <c r="B11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -901,7 +901,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>185.7</v>
+        <v>201.1</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>16.7</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -996,25 +996,25 @@
         <v>21</v>
       </c>
       <c r="B15">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
       <c r="D15">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E15">
-        <v>138.6</v>
+        <v>143</v>
       </c>
       <c r="F15">
         <v>4.5</v>
       </c>
       <c r="G15">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="H15">
-        <v>46.8</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1048,25 +1048,25 @@
         <v>23</v>
       </c>
       <c r="B17">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C17">
         <v>8</v>
       </c>
       <c r="D17">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E17">
-        <v>95.2</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F17">
         <v>6.2</v>
       </c>
       <c r="G17">
-        <v>6.6</v>
+        <v>6.3</v>
       </c>
       <c r="H17">
-        <v>39.3</v>
+        <v>39.7</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1100,16 +1100,16 @@
         <v>25</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E19">
-        <v>63.7</v>
+        <v>68.7</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1118,7 +1118,7 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>33.3</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1126,16 +1126,16 @@
         <v>26</v>
       </c>
       <c r="B20">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E20">
-        <v>57.2</v>
+        <v>63.7</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -1311,7 +1311,7 @@
         <v>14</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27">
         <v>11</v>
@@ -1320,10 +1320,10 @@
         <v>36.5</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>7.1</v>
       </c>
       <c r="H27">
         <v>78.59999999999999</v>
@@ -1407,10 +1407,10 @@
         <v>39</v>
       </c>
       <c r="B2">
-        <v>61.2</v>
+        <v>60.7</v>
       </c>
       <c r="C2">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1418,10 +1418,10 @@
         <v>40</v>
       </c>
       <c r="B3">
-        <v>61.7</v>
+        <v>61.2</v>
       </c>
       <c r="C3">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1429,10 +1429,10 @@
         <v>41</v>
       </c>
       <c r="B4">
-        <v>61.7</v>
+        <v>61.3</v>
       </c>
       <c r="C4">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1440,10 +1440,10 @@
         <v>42</v>
       </c>
       <c r="B5">
-        <v>61.7</v>
+        <v>61.3</v>
       </c>
       <c r="C5">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1451,10 +1451,10 @@
         <v>43</v>
       </c>
       <c r="B6">
-        <v>88.7</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="C6">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1462,10 +1462,10 @@
         <v>44</v>
       </c>
       <c r="B7">
-        <v>95</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="C7">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1476,7 +1476,7 @@
         <v>98.59999999999999</v>
       </c>
       <c r="C8">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1484,10 +1484,10 @@
         <v>46</v>
       </c>
       <c r="B9">
-        <v>98.59999999999999</v>
+        <v>98.8</v>
       </c>
       <c r="C9">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1498,7 +1498,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="C10">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1509,7 +1509,7 @@
         <v>99.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1520,7 +1520,7 @@
         <v>100</v>
       </c>
       <c r="C12">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1531,7 +1531,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1542,7 +1542,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1553,7 +1553,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1424</v>
+        <v>1462</v>
       </c>
     </row>
   </sheetData>
@@ -1579,24 +1579,24 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="C2">
-        <v>30.5</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B3">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C3">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1604,10 +1604,10 @@
         <v>56</v>
       </c>
       <c r="B4">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="C4">
-        <v>12.4</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1615,7 +1615,7 @@
         <v>57</v>
       </c>
       <c r="B5">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C5">
         <v>12</v>
@@ -1626,10 +1626,10 @@
         <v>58</v>
       </c>
       <c r="B6">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1637,7 +1637,7 @@
         <v>59</v>
       </c>
       <c r="B7">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C7">
         <v>3.6</v>
@@ -1651,7 +1651,7 @@
         <v>37</v>
       </c>
       <c r="C8">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1662,7 +1662,7 @@
         <v>27</v>
       </c>
       <c r="C9">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1716,13 +1716,13 @@
         <v>64</v>
       </c>
       <c r="B2">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1730,7 +1730,7 @@
         <v>65</v>
       </c>
       <c r="B3">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1744,7 +1744,7 @@
         <v>66</v>
       </c>
       <c r="B4">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1758,13 +1758,13 @@
         <v>67</v>
       </c>
       <c r="B5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>2</v>
       </c>
       <c r="D5">
-        <v>25</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1786,13 +1786,13 @@
         <v>69</v>
       </c>
       <c r="B7">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1800,7 +1800,7 @@
         <v>70</v>
       </c>
       <c r="B8">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -1814,13 +1814,13 @@
         <v>71</v>
       </c>
       <c r="B9">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1828,13 +1828,13 @@
         <v>72</v>
       </c>
       <c r="B10">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D10">
-        <v>4.9</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -1842,7 +1842,7 @@
         <v>73</v>
       </c>
       <c r="B11">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1856,13 +1856,13 @@
         <v>74</v>
       </c>
       <c r="B12">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="C12">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D12">
-        <v>13</v>
+        <v>13.1</v>
       </c>
     </row>
   </sheetData>
@@ -1894,13 +1894,13 @@
         <v>64</v>
       </c>
       <c r="B2">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="C2">
         <v>62</v>
       </c>
       <c r="D2">
-        <v>47</v>
+        <v>44.9</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1908,13 +1908,13 @@
         <v>65</v>
       </c>
       <c r="B3">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="C3">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3">
-        <v>21.3</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -1922,13 +1922,13 @@
         <v>66</v>
       </c>
       <c r="B4">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>15.6</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1936,13 +1936,13 @@
         <v>67</v>
       </c>
       <c r="B5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5">
-        <v>37.5</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1964,13 +1964,13 @@
         <v>69</v>
       </c>
       <c r="B7">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C7">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7">
-        <v>34.3</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1978,13 +1978,13 @@
         <v>70</v>
       </c>
       <c r="B8">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C8">
         <v>17</v>
       </c>
       <c r="D8">
-        <v>36.2</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1992,13 +1992,13 @@
         <v>71</v>
       </c>
       <c r="B9">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C9">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9">
-        <v>24.4</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2006,13 +2006,13 @@
         <v>72</v>
       </c>
       <c r="B10">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C10">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10">
-        <v>34.6</v>
+        <v>35.4</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2020,10 +2020,10 @@
         <v>73</v>
       </c>
       <c r="B11">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C11">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11">
         <v>25.2</v>
@@ -2034,13 +2034,13 @@
         <v>74</v>
       </c>
       <c r="B12">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="C12">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D12">
-        <v>27.8</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -2069,10 +2069,10 @@
         <v>77</v>
       </c>
       <c r="B2">
-        <v>822</v>
+        <v>849</v>
       </c>
       <c r="C2">
-        <v>98.90000000000001</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2080,10 +2080,10 @@
         <v>78</v>
       </c>
       <c r="B3">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2091,10 +2091,10 @@
         <v>79</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -2123,10 +2123,10 @@
         <v>81</v>
       </c>
       <c r="B2">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C2">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2134,10 +2134,10 @@
         <v>82</v>
       </c>
       <c r="B3">
-        <v>1031</v>
+        <v>1071</v>
       </c>
       <c r="C3">
-        <v>72.40000000000001</v>
+        <v>73.3</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2145,10 +2145,10 @@
         <v>83</v>
       </c>
       <c r="B4">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C4">
-        <v>26.2</v>
+        <v>25.6</v>
       </c>
     </row>
   </sheetData>
@@ -2188,10 +2188,10 @@
         <v>85</v>
       </c>
       <c r="B3">
-        <v>568</v>
+        <v>588</v>
       </c>
       <c r="C3">
-        <v>39.9</v>
+        <v>40.2</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2199,10 +2199,10 @@
         <v>86</v>
       </c>
       <c r="B4">
-        <v>854</v>
+        <v>872</v>
       </c>
       <c r="C4">
-        <v>60</v>
+        <v>59.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de dados — 03/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="88">
   <si>
     <t>municipio</t>
   </si>
@@ -29,6 +29,9 @@
     <t>casos</t>
   </si>
   <si>
+    <t>encerrados</t>
+  </si>
+  <si>
     <t>obitos_srag</t>
   </si>
   <si>
@@ -59,33 +62,33 @@
     <t>Ourizona</t>
   </si>
   <si>
+    <t>Atalaia</t>
+  </si>
+  <si>
+    <t>Itaguaje</t>
+  </si>
+  <si>
     <t>Sao Jorge Do Ivai</t>
   </si>
   <si>
-    <t>Atalaia</t>
-  </si>
-  <si>
-    <t>Itaguaje</t>
+    <t>Maringa</t>
   </si>
   <si>
     <t>Nossa Senhora Das Gracas</t>
   </si>
   <si>
-    <t>Maringa</t>
-  </si>
-  <si>
     <t>Santo Inacio</t>
   </si>
   <si>
     <t>Colorado</t>
   </si>
   <si>
+    <t>Itambe</t>
+  </si>
+  <si>
     <t>Florai</t>
   </si>
   <si>
-    <t>Itambe</t>
-  </si>
-  <si>
     <t>Marialva</t>
   </si>
   <si>
@@ -110,12 +113,12 @@
     <t>Paicandu</t>
   </si>
   <si>
+    <t>Presidente Castelo Branco</t>
+  </si>
+  <si>
     <t>Mandaguacu</t>
   </si>
   <si>
-    <t>Presidente Castelo Branco</t>
-  </si>
-  <si>
     <t>Santa Fe</t>
   </si>
   <si>
@@ -176,7 +179,7 @@
     <t>Idade</t>
   </si>
   <si>
-    <t>Semana Epidemiológica</t>
+    <t>Semana de início dos sintomas</t>
   </si>
   <si>
     <t>Data Início Sintomas</t>
@@ -624,10 +627,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1">
+    <row r="1" spans="1:9" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -652,634 +655,709 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>101</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E2">
-        <v>386.9</v>
+        <v>6</v>
       </c>
       <c r="F2">
-        <v>33.2</v>
+        <v>420</v>
       </c>
       <c r="G2">
-        <v>8.6</v>
+        <v>36.8</v>
       </c>
       <c r="H2">
-        <v>3.8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>9.9</v>
+      </c>
+      <c r="I2">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <v>5</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
         <v>286.5</v>
       </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:8">
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>6</v>
       </c>
       <c r="C4">
+        <v>6</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
       <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
         <v>284.9</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>47.5</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>16.7</v>
       </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>8</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
         <v>3</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>250.5</v>
       </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
         <v>37.5</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <v>9</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>247.2</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>242.8</v>
+      </c>
+      <c r="G7">
+        <v>22.1</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
         <v>12</v>
       </c>
-      <c r="B6">
+      <c r="C8">
         <v>12</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
         <v>3</v>
       </c>
-      <c r="E6">
+      <c r="F8">
         <v>232.1</v>
       </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7">
-        <v>9</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>222.4</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9">
+        <v>970</v>
+      </c>
+      <c r="C9">
+        <v>862</v>
+      </c>
+      <c r="D9">
+        <v>81</v>
+      </c>
+      <c r="E9">
+        <v>287</v>
+      </c>
+      <c r="F9">
+        <v>225.8</v>
+      </c>
+      <c r="G9">
+        <v>18.9</v>
+      </c>
+      <c r="H9">
+        <v>9.4</v>
+      </c>
+      <c r="I9">
+        <v>29.6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10">
+        <v>218</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>37.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11">
         <v>14</v>
       </c>
-      <c r="B8">
-        <v>10</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>220.8</v>
-      </c>
-      <c r="F8">
-        <v>22.1</v>
-      </c>
-      <c r="G8">
-        <v>10</v>
-      </c>
-      <c r="H8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9">
-        <v>8</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
+      <c r="C11">
+        <v>12</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
         <v>3</v>
       </c>
-      <c r="E9">
-        <v>218</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>37.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10">
-        <v>931</v>
-      </c>
-      <c r="C10">
-        <v>74</v>
-      </c>
-      <c r="D10">
-        <v>269</v>
-      </c>
-      <c r="E10">
-        <v>216.7</v>
-      </c>
-      <c r="F10">
-        <v>17.2</v>
-      </c>
-      <c r="G10">
-        <v>7.9</v>
-      </c>
-      <c r="H10">
-        <v>28.9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11">
-        <v>13</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>2</v>
-      </c>
-      <c r="E11">
-        <v>201.1</v>
-      </c>
       <c r="F11">
-        <v>0</v>
+        <v>216.6</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11">
-        <v>15.4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B12">
         <v>42</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
         <v>2</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>180.2</v>
       </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
       <c r="G12">
         <v>0</v>
       </c>
       <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
         <v>4.8</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B13">
+        <v>10</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13">
+        <v>160.6</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14">
         <v>7</v>
       </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
+      <c r="C14">
+        <v>7</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
         <v>2</v>
       </c>
-      <c r="E13">
+      <c r="F14">
         <v>145.7</v>
       </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
         <v>28.6</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14">
-        <v>9</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15">
+        <v>65</v>
+      </c>
+      <c r="C15">
+        <v>64</v>
+      </c>
+      <c r="D15">
         <v>2</v>
       </c>
-      <c r="E14">
-        <v>144.5</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>22.2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15">
-        <v>64</v>
-      </c>
-      <c r="C15">
-        <v>2</v>
-      </c>
-      <c r="D15">
-        <v>30</v>
-      </c>
       <c r="E15">
-        <v>143</v>
+        <v>31</v>
       </c>
       <c r="F15">
+        <v>145.3</v>
+      </c>
+      <c r="G15">
         <v>4.5</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>3.1</v>
       </c>
-      <c r="H15">
-        <v>46.9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
+      <c r="I15">
+        <v>47.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B16">
         <v>10</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
         <v>2</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <v>104.7</v>
       </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
       <c r="G16">
         <v>0</v>
       </c>
       <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B17">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C17">
-        <v>8</v>
+        <v>129</v>
       </c>
       <c r="D17">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="E17">
-        <v>98.40000000000001</v>
+        <v>52</v>
       </c>
       <c r="F17">
-        <v>6.2</v>
+        <v>103</v>
       </c>
       <c r="G17">
-        <v>6.3</v>
+        <v>7</v>
       </c>
       <c r="H17">
-        <v>39.7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
+        <v>7</v>
+      </c>
+      <c r="I17">
+        <v>39.4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B18">
         <v>3</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
         <v>1</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <v>73.90000000000001</v>
       </c>
-      <c r="F18">
-        <v>0</v>
-      </c>
       <c r="G18">
         <v>0</v>
       </c>
       <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
         <v>33.3</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B19">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
         <v>5</v>
       </c>
-      <c r="E19">
-        <v>68.7</v>
-      </c>
       <c r="F19">
-        <v>0</v>
+        <v>72.5</v>
       </c>
       <c r="G19">
         <v>0</v>
       </c>
       <c r="H19">
-        <v>27.8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>26.3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B20">
         <v>3</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
         <v>1</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <v>63.7</v>
       </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
       <c r="G20">
         <v>0</v>
       </c>
       <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
         <v>33.3</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>52.1</v>
+        <v>2</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>60.8</v>
       </c>
       <c r="G21">
         <v>0</v>
       </c>
       <c r="H21">
-        <v>16.7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B22">
         <v>24</v>
       </c>
       <c r="C22">
+        <v>24</v>
+      </c>
+      <c r="D22">
         <v>1</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>15</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <v>49.3</v>
       </c>
-      <c r="F22">
+      <c r="G22">
         <v>2.1</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>4.2</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>62.5</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B23">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>46.5</v>
+      </c>
+      <c r="G23">
+        <v>23.2</v>
+      </c>
+      <c r="H23">
+        <v>50</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24">
+        <v>16</v>
+      </c>
+      <c r="C24">
+        <v>15</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
         <v>7</v>
       </c>
-      <c r="E23">
-        <v>49.2</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
-      <c r="H23">
-        <v>41.2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24">
-        <v>2</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24">
-        <v>0</v>
-      </c>
-      <c r="E24">
-        <v>46.5</v>
-      </c>
       <c r="F24">
-        <v>23.2</v>
+        <v>46.3</v>
       </c>
       <c r="G24">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="H24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:8">
+      <c r="I24">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B25">
         <v>5</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
         <v>4</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>42.6</v>
       </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
       <c r="G25">
         <v>0</v>
       </c>
       <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B26">
         <v>1</v>
@@ -1288,96 +1366,105 @@
         <v>0</v>
       </c>
       <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
         <v>1</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <v>36.9</v>
       </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
       <c r="G26">
         <v>0</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B27">
         <v>14</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
         <v>11</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <v>36.5</v>
       </c>
-      <c r="F27">
-        <v>2.6</v>
-      </c>
       <c r="G27">
-        <v>7.1</v>
+        <v>0</v>
       </c>
       <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
         <v>78.59999999999999</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D28">
+        <v>0</v>
+      </c>
+      <c r="E28">
         <v>1</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <v>35.1</v>
       </c>
-      <c r="F28">
-        <v>0</v>
-      </c>
       <c r="G28">
         <v>0</v>
       </c>
       <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B29">
         <v>2</v>
       </c>
       <c r="C29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
         <v>1</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>30.7</v>
       </c>
-      <c r="F29">
-        <v>0</v>
-      </c>
       <c r="G29">
         <v>0</v>
       </c>
       <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29">
         <v>50</v>
       </c>
     </row>
@@ -1393,167 +1480,167 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2">
-        <v>60.7</v>
+        <v>60.9</v>
       </c>
       <c r="C2">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3">
-        <v>61.2</v>
+        <v>61.3</v>
       </c>
       <c r="C3">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4">
-        <v>61.3</v>
+        <v>61.4</v>
       </c>
       <c r="C4">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B5">
-        <v>61.3</v>
+        <v>61.4</v>
       </c>
       <c r="C5">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6">
-        <v>89.90000000000001</v>
+        <v>90.5</v>
       </c>
       <c r="C6">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7">
-        <v>96.09999999999999</v>
+        <v>95.7</v>
       </c>
       <c r="C7">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B8">
-        <v>98.59999999999999</v>
+        <v>98.7</v>
       </c>
       <c r="C8">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9">
-        <v>98.8</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="C9">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10">
-        <v>98.90000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="C10">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11">
         <v>99.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B12">
         <v>100</v>
       </c>
       <c r="C12">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B13">
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B14">
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B15">
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1462</v>
+        <v>1522</v>
       </c>
     </row>
   </sheetData>
@@ -1568,87 +1655,87 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2">
-        <v>442</v>
+        <v>461</v>
       </c>
       <c r="C2">
-        <v>30.2</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3">
-        <v>223</v>
+        <v>232</v>
       </c>
       <c r="C3">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B4">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C4">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B5">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C5">
-        <v>12</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B6">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="C6">
-        <v>10.7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B7">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C7">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C8">
         <v>2.5</v>
@@ -1656,29 +1743,29 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C9">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B10">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C10">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -1694,175 +1781,211 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1">
+    <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+        <v>64</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="C2">
+        <v>129</v>
+      </c>
+      <c r="D2">
         <v>4</v>
       </c>
-      <c r="D2">
-        <v>2.9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B3">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B4">
         <v>33</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B5">
         <v>9</v>
       </c>
       <c r="C5">
+        <v>9</v>
+      </c>
+      <c r="D5">
         <v>2</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>22.2</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B6">
         <v>21</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B7">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="D7">
-        <v>5.6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B8">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B9">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C9">
+        <v>86</v>
+      </c>
+      <c r="D9">
         <v>1</v>
       </c>
-      <c r="D9">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B10">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C10">
+        <v>79</v>
+      </c>
+      <c r="D10">
         <v>5</v>
       </c>
-      <c r="D10">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B11">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12">
-        <v>643</v>
+        <v>668</v>
       </c>
       <c r="C12">
-        <v>84</v>
+        <v>601</v>
       </c>
       <c r="D12">
-        <v>13.1</v>
+        <v>93</v>
+      </c>
+      <c r="E12">
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>
@@ -1877,49 +2000,49 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2">
+        <v>146</v>
+      </c>
+      <c r="C2">
         <v>64</v>
       </c>
-      <c r="B2">
-        <v>138</v>
-      </c>
-      <c r="C2">
-        <v>62</v>
-      </c>
       <c r="D2">
-        <v>44.9</v>
+        <v>43.8</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B3">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="C3">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D3">
-        <v>21.1</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B4">
         <v>33</v>
@@ -1933,7 +2056,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B5">
         <v>9</v>
@@ -1947,7 +2070,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B6">
         <v>21</v>
@@ -1961,86 +2084,86 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B7">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>13</v>
       </c>
       <c r="D7">
-        <v>36.1</v>
+        <v>39.4</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B8">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C8">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D8">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B9">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C9">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9">
-        <v>23.6</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B10">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C10">
         <v>29</v>
       </c>
       <c r="D10">
-        <v>35.4</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B11">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C11">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D11">
-        <v>25.2</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12">
-        <v>643</v>
+        <v>668</v>
       </c>
       <c r="C12">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="D12">
-        <v>28</v>
+        <v>28.9</v>
       </c>
     </row>
   </sheetData>
@@ -2055,46 +2178,46 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B2">
-        <v>849</v>
+        <v>871</v>
       </c>
       <c r="C2">
-        <v>99.40000000000001</v>
+        <v>98.90000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C4">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -2109,46 +2232,46 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B2">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B3">
-        <v>1071</v>
+        <v>1130</v>
       </c>
       <c r="C3">
-        <v>73.3</v>
+        <v>74.2</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B4">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C4">
-        <v>25.6</v>
+        <v>24.7</v>
       </c>
     </row>
   </sheetData>
@@ -2163,18 +2286,18 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -2185,24 +2308,24 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B3">
-        <v>588</v>
+        <v>619</v>
       </c>
       <c r="C3">
-        <v>40.2</v>
+        <v>40.7</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4">
-        <v>872</v>
+        <v>901</v>
       </c>
       <c r="C4">
-        <v>59.6</v>
+        <v>59.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização de layout/texto — 03/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -14,14 +14,15 @@
     <sheet name="uti_faixa" sheetId="5" r:id="rId5"/>
     <sheet name="criterio_conf" sheetId="6" r:id="rId6"/>
     <sheet name="antiviral" sheetId="7" r:id="rId7"/>
-    <sheet name="vacinal" sheetId="8" r:id="rId8"/>
+    <sheet name="antiviral_influenza" sheetId="8" r:id="rId8"/>
+    <sheet name="vacinal" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="88">
   <si>
     <t>municipio</t>
   </si>
@@ -2286,6 +2287,60 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3">
+        <v>112</v>
+      </c>
+      <c r="C3">
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4">
+        <v>278</v>
+      </c>
+      <c r="C4">
+        <v>70.90000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
         <v>85</v>
       </c>
       <c r="B1" s="1" t="s">

</xml_diff>

<commit_message>
Atualização de dados — 04/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -22,15 +22,19 @@
     <sheet name="digitacao_unidade" sheetId="13" r:id="rId13"/>
     <sheet name="digitacao_mes" sheetId="14" r:id="rId14"/>
     <sheet name="qualidade" sheetId="15" r:id="rId15"/>
-    <sheet name="vacina_influenza" sheetId="16" r:id="rId16"/>
-    <sheet name="vacinal" sheetId="17" r:id="rId17"/>
+    <sheet name="consistencia_regras" sheetId="16" r:id="rId16"/>
+    <sheet name="consistencia_unidade" sheetId="17" r:id="rId17"/>
+    <sheet name="representatividade_rip" sheetId="18" r:id="rId18"/>
+    <sheet name="internacao_fora" sheetId="19" r:id="rId19"/>
+    <sheet name="vacina_influenza" sheetId="20" r:id="rId20"/>
+    <sheet name="vacinal" sheetId="21" r:id="rId21"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="262">
   <si>
     <t>municipio</t>
   </si>
@@ -714,6 +718,90 @@
   </si>
   <si>
     <t>Satisfatório</t>
+  </si>
+  <si>
+    <t>regra</t>
+  </si>
+  <si>
+    <t>aplicaveis</t>
+  </si>
+  <si>
+    <t>inconsistentes</t>
+  </si>
+  <si>
+    <t>Classificação final informada sem data de encerramento</t>
+  </si>
+  <si>
+    <t>Antiviral informado sem data de início</t>
+  </si>
+  <si>
+    <t>Internação mais de 30 dias após o início dos sintomas</t>
+  </si>
+  <si>
+    <t>Internação em UTI informada sem data de entrada</t>
+  </si>
+  <si>
+    <t>Evolução (cura ou óbito) informada sem classificação final</t>
+  </si>
+  <si>
+    <t>Evolução mais de 120 dias após a internação</t>
+  </si>
+  <si>
+    <t>registros</t>
+  </si>
+  <si>
+    <t>com_inconsistencia</t>
+  </si>
+  <si>
+    <t>regra_mais_comum</t>
+  </si>
+  <si>
+    <t>codigo_ibge_6</t>
+  </si>
+  <si>
+    <t>esperados</t>
+  </si>
+  <si>
+    <t>observados</t>
+  </si>
+  <si>
+    <t>rip</t>
+  </si>
+  <si>
+    <t>li</t>
+  </si>
+  <si>
+    <t>ls</t>
+  </si>
+  <si>
+    <t>situacao</t>
+  </si>
+  <si>
+    <t>acima</t>
+  </si>
+  <si>
+    <t>compativel</t>
+  </si>
+  <si>
+    <t>abaixo</t>
+  </si>
+  <si>
+    <t>Angulo</t>
+  </si>
+  <si>
+    <t>Ivatuba</t>
+  </si>
+  <si>
+    <t>Internados em município da regional</t>
+  </si>
+  <si>
+    <t>Internados fora da regional, no Paraná</t>
+  </si>
+  <si>
+    <t>Internados fora do Paraná</t>
+  </si>
+  <si>
+    <t>Município de internação não informado</t>
   </si>
   <si>
     <t>grupo</t>
@@ -3775,10 +3863,10 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1">
+    <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>228</v>
       </c>
@@ -3786,115 +3874,94 @@
         <v>229</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>230</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B2" t="s">
         <v>231</v>
       </c>
+      <c r="B2">
+        <v>1487</v>
+      </c>
       <c r="C2">
-        <v>160</v>
+        <v>17</v>
       </c>
       <c r="D2">
-        <v>392</v>
-      </c>
-      <c r="E2">
-        <v>40.8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>230</v>
-      </c>
-      <c r="B3" t="s">
         <v>232</v>
       </c>
+      <c r="B3">
+        <v>387</v>
+      </c>
       <c r="C3">
-        <v>230</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>392</v>
-      </c>
-      <c r="E3">
-        <v>58.7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>230</v>
-      </c>
-      <c r="B4" t="s">
-        <v>82</v>
+        <v>233</v>
+      </c>
+      <c r="B4">
+        <v>1533</v>
       </c>
       <c r="C4">
+        <v>7</v>
+      </c>
+      <c r="D4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>234</v>
+      </c>
+      <c r="B5">
+        <v>473</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>235</v>
+      </c>
+      <c r="B6">
+        <v>1400</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B7">
+        <v>1389</v>
+      </c>
+      <c r="C7">
         <v>2</v>
       </c>
-      <c r="D4">
-        <v>392</v>
-      </c>
-      <c r="E4">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" t="s">
-        <v>231</v>
-      </c>
-      <c r="C5">
-        <v>30</v>
-      </c>
-      <c r="D5">
-        <v>56</v>
-      </c>
-      <c r="E5">
-        <v>53.6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" t="s">
-        <v>232</v>
-      </c>
-      <c r="C6">
-        <v>26</v>
-      </c>
-      <c r="D6">
-        <v>56</v>
-      </c>
-      <c r="E6">
-        <v>46.4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
       <c r="D7">
-        <v>56</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -3904,15 +3971,1314 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:6" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3">
+        <v>72</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>5.6</v>
+      </c>
+      <c r="F3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>98</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>5.1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>78</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>2.6</v>
+      </c>
+      <c r="F5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>198</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6">
+        <v>331</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>2.4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7">
+        <v>42</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>2.4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8">
+        <v>101</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9">
+        <v>63</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1.6</v>
+      </c>
+      <c r="F9" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>202</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>131</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>1.5</v>
+      </c>
+      <c r="F10" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>199</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>280</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>1.1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>205</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12">
+        <v>101</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>207</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13">
+        <v>154</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>204</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14">
+        <v>18</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>200</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15">
+        <v>15</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>211</v>
+      </c>
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16">
+        <v>14</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>212</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>196</v>
+      </c>
+      <c r="B18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18">
+        <v>9</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>213</v>
+      </c>
+      <c r="B19" t="s">
+        <v>214</v>
+      </c>
+      <c r="C19">
+        <v>6</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>16.7</v>
+      </c>
+      <c r="F19" t="s">
+        <v>233</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:9" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2">
+        <v>411690</v>
+      </c>
+      <c r="B2">
+        <v>47.59190958417413</v>
+      </c>
+      <c r="C2">
+        <v>27142</v>
+      </c>
+      <c r="D2">
+        <v>114</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2">
+        <v>2.395365115542847</v>
+      </c>
+      <c r="G2">
+        <v>1.975880837385551</v>
+      </c>
+      <c r="H2">
+        <v>2.87756521607562</v>
+      </c>
+      <c r="I2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3">
+        <v>412360</v>
+      </c>
+      <c r="B3">
+        <v>3.120055957676751</v>
+      </c>
+      <c r="C3">
+        <v>1745</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>1.60253536084753</v>
+      </c>
+      <c r="G3">
+        <v>0.5203388696038955</v>
+      </c>
+      <c r="H3">
+        <v>3.739782951845233</v>
+      </c>
+      <c r="I3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4">
+        <v>412830</v>
+      </c>
+      <c r="B4">
+        <v>3.820820242331692</v>
+      </c>
+      <c r="C4">
+        <v>2106</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4">
+        <v>1.570343439224045</v>
+      </c>
+      <c r="G4">
+        <v>0.5762883658057475</v>
+      </c>
+      <c r="H4">
+        <v>3.417976558496512</v>
+      </c>
+      <c r="I4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>410220</v>
+      </c>
+      <c r="B5">
+        <v>7.182495033139207</v>
+      </c>
+      <c r="C5">
+        <v>4046</v>
+      </c>
+      <c r="D5">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5">
+        <v>1.392273848274332</v>
+      </c>
+      <c r="G5">
+        <v>0.6676494273935535</v>
+      </c>
+      <c r="H5">
+        <v>2.56044117777552</v>
+      </c>
+      <c r="I5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6">
+        <v>411090</v>
+      </c>
+      <c r="B6">
+        <v>7.925565257205213</v>
+      </c>
+      <c r="C6">
+        <v>4530</v>
+      </c>
+      <c r="D6">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>1.387913624204884</v>
+      </c>
+      <c r="G6">
+        <v>0.6928414805801728</v>
+      </c>
+      <c r="H6">
+        <v>2.483360854976093</v>
+      </c>
+      <c r="I6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7">
+        <v>411520</v>
+      </c>
+      <c r="B7">
+        <v>708.618739424934</v>
+      </c>
+      <c r="C7">
+        <v>429660</v>
+      </c>
+      <c r="D7">
+        <v>970</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7">
+        <v>1.368860214996833</v>
+      </c>
+      <c r="G7">
+        <v>1.284061260184467</v>
+      </c>
+      <c r="H7">
+        <v>1.457787801171709</v>
+      </c>
+      <c r="I7" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8">
+        <v>411740</v>
+      </c>
+      <c r="B8">
+        <v>5.887620794244284</v>
+      </c>
+      <c r="C8">
+        <v>3193</v>
+      </c>
+      <c r="D8">
+        <v>8</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8">
+        <v>1.358783162091684</v>
+      </c>
+      <c r="G8">
+        <v>0.5866261258070417</v>
+      </c>
+      <c r="H8">
+        <v>2.677344511657977</v>
+      </c>
+      <c r="I8" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9">
+        <v>411640</v>
+      </c>
+      <c r="B9">
+        <v>6.05448539639124</v>
+      </c>
+      <c r="C9">
+        <v>3669</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9">
+        <v>1.321334428317951</v>
+      </c>
+      <c r="G9">
+        <v>0.5704584205962656</v>
+      </c>
+      <c r="H9">
+        <v>2.603555577091477</v>
+      </c>
+      <c r="I9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10">
+        <v>412530</v>
+      </c>
+      <c r="B10">
+        <v>9.881799363449487</v>
+      </c>
+      <c r="C10">
+        <v>5170</v>
+      </c>
+      <c r="D10">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10">
+        <v>1.214353738488686</v>
+      </c>
+      <c r="G10">
+        <v>0.627474297004726</v>
+      </c>
+      <c r="H10">
+        <v>2.121231597325185</v>
+      </c>
+      <c r="I10" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11">
+        <v>412450</v>
+      </c>
+      <c r="B11">
+        <v>11.61148021598628</v>
+      </c>
+      <c r="C11">
+        <v>6463</v>
+      </c>
+      <c r="D11">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11">
+        <v>1.205703298768515</v>
+      </c>
+      <c r="G11">
+        <v>0.6591692130485598</v>
+      </c>
+      <c r="H11">
+        <v>2.022965262387124</v>
+      </c>
+      <c r="I11" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12">
+        <v>410590</v>
+      </c>
+      <c r="B12">
+        <v>40.65070550415243</v>
+      </c>
+      <c r="C12">
+        <v>23313</v>
+      </c>
+      <c r="D12">
+        <v>42</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12">
+        <v>1.033192400454396</v>
+      </c>
+      <c r="G12">
+        <v>0.744634203934927</v>
+      </c>
+      <c r="H12">
+        <v>1.396575977572922</v>
+      </c>
+      <c r="I12" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13">
+        <v>411110</v>
+      </c>
+      <c r="B13">
+        <v>10.71960483015752</v>
+      </c>
+      <c r="C13">
+        <v>6228</v>
+      </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13">
+        <v>0.9328702091579858</v>
+      </c>
+      <c r="G13">
+        <v>0.4473475255954904</v>
+      </c>
+      <c r="H13">
+        <v>1.715581528740695</v>
+      </c>
+      <c r="I13" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14">
+        <v>411480</v>
+      </c>
+      <c r="B14">
+        <v>76.1402973292391</v>
+      </c>
+      <c r="C14">
+        <v>44749</v>
+      </c>
+      <c r="D14">
+        <v>65</v>
+      </c>
+      <c r="E14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14">
+        <v>0.8536872363255003</v>
+      </c>
+      <c r="G14">
+        <v>0.6588577860723676</v>
+      </c>
+      <c r="H14">
+        <v>1.088094461433849</v>
+      </c>
+      <c r="I14" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15">
+        <v>410780</v>
+      </c>
+      <c r="B15">
+        <v>9.655942925034168</v>
+      </c>
+      <c r="C15">
+        <v>4805</v>
+      </c>
+      <c r="D15">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15">
+        <v>0.7249421474780755</v>
+      </c>
+      <c r="G15">
+        <v>0.2914643420502517</v>
+      </c>
+      <c r="H15">
+        <v>1.493657892727379</v>
+      </c>
+      <c r="I15" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16">
+        <v>412625</v>
+      </c>
+      <c r="B16">
+        <v>202.9578045524855</v>
+      </c>
+      <c r="C16">
+        <v>128106</v>
+      </c>
+      <c r="D16">
+        <v>132</v>
+      </c>
+      <c r="E16" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16">
+        <v>0.6503814932914512</v>
+      </c>
+      <c r="G16">
+        <v>0.5441688170690743</v>
+      </c>
+      <c r="H16">
+        <v>0.7712694703079357</v>
+      </c>
+      <c r="I16" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17">
+        <v>411810</v>
+      </c>
+      <c r="B17">
+        <v>15.98585273920547</v>
+      </c>
+      <c r="C17">
+        <v>9549</v>
+      </c>
+      <c r="D17">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17">
+        <v>0.6255531164424465</v>
+      </c>
+      <c r="G17">
+        <v>0.2999770343418524</v>
+      </c>
+      <c r="H17">
+        <v>1.15041445345704</v>
+      </c>
+      <c r="I17" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18">
+        <v>410210</v>
+      </c>
+      <c r="B18">
+        <v>47.85677468621944</v>
+      </c>
+      <c r="C18">
+        <v>26203</v>
+      </c>
+      <c r="D18">
+        <v>19</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18">
+        <v>0.3970179796815921</v>
+      </c>
+      <c r="G18">
+        <v>0.2390307587456517</v>
+      </c>
+      <c r="H18">
+        <v>0.6199927547589087</v>
+      </c>
+      <c r="I18" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19">
+        <v>411360</v>
+      </c>
+      <c r="B19">
+        <v>7.671612549406151</v>
+      </c>
+      <c r="C19">
+        <v>4707</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19">
+        <v>0.3910520742125104</v>
+      </c>
+      <c r="G19">
+        <v>0.08064433897192734</v>
+      </c>
+      <c r="H19">
+        <v>1.142820106370073</v>
+      </c>
+      <c r="I19" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20">
+        <v>411630</v>
+      </c>
+      <c r="B20">
+        <v>7.932381828941635</v>
+      </c>
+      <c r="C20">
+        <v>4057</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20">
+        <v>0.3781966204720972</v>
+      </c>
+      <c r="G20">
+        <v>0.07799323535313815</v>
+      </c>
+      <c r="H20">
+        <v>1.105251015244192</v>
+      </c>
+      <c r="I20" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21">
+        <v>410790</v>
+      </c>
+      <c r="B21">
+        <v>19.89931648618882</v>
+      </c>
+      <c r="C21">
+        <v>11522</v>
+      </c>
+      <c r="D21">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21">
+        <v>0.3517708763945923</v>
+      </c>
+      <c r="G21">
+        <v>0.1414301367322432</v>
+      </c>
+      <c r="H21">
+        <v>0.7247824502772484</v>
+      </c>
+      <c r="I21" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22">
+        <v>411750</v>
+      </c>
+      <c r="B22">
+        <v>79.20952501920122</v>
+      </c>
+      <c r="C22">
+        <v>48695</v>
+      </c>
+      <c r="D22">
+        <v>24</v>
+      </c>
+      <c r="E22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22">
+        <v>0.3029938633539609</v>
+      </c>
+      <c r="G22">
+        <v>0.1941338854255072</v>
+      </c>
+      <c r="H22">
+        <v>0.4508308512782611</v>
+      </c>
+      <c r="I22" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23">
+        <v>412040</v>
+      </c>
+      <c r="B23">
+        <v>7.037976950852113</v>
+      </c>
+      <c r="C23">
+        <v>4304</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23">
+        <v>0.2841725703233303</v>
+      </c>
+      <c r="G23">
+        <v>0.03441461661999898</v>
+      </c>
+      <c r="H23">
+        <v>1.026529032160192</v>
+      </c>
+      <c r="I23" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24">
+        <v>411410</v>
+      </c>
+      <c r="B24">
+        <v>58.77064219403454</v>
+      </c>
+      <c r="C24">
+        <v>34521</v>
+      </c>
+      <c r="D24">
+        <v>16</v>
+      </c>
+      <c r="E24" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24">
+        <v>0.2722447705637639</v>
+      </c>
+      <c r="G24">
+        <v>0.1556114092380943</v>
+      </c>
+      <c r="H24">
+        <v>0.4421084512191757</v>
+      </c>
+      <c r="I24" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25">
+        <v>412340</v>
+      </c>
+      <c r="B25">
+        <v>20.57924830121171</v>
+      </c>
+      <c r="C25">
+        <v>11730</v>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+      <c r="E25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25">
+        <v>0.2429631989865053</v>
+      </c>
+      <c r="G25">
+        <v>0.07888948937084499</v>
+      </c>
+      <c r="H25">
+        <v>0.5669950577658192</v>
+      </c>
+      <c r="I25" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26">
+        <v>411000</v>
+      </c>
+      <c r="B26">
+        <v>9.383815600487981</v>
+      </c>
+      <c r="C26">
+        <v>5693</v>
+      </c>
+      <c r="D26">
+        <v>2</v>
+      </c>
+      <c r="E26" t="s">
+        <v>35</v>
+      </c>
+      <c r="F26">
+        <v>0.2131329179034587</v>
+      </c>
+      <c r="G26">
+        <v>0.02581138513968341</v>
+      </c>
+      <c r="H26">
+        <v>0.7699093817815704</v>
+      </c>
+      <c r="I26" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27">
+        <v>411420</v>
+      </c>
+      <c r="B27">
+        <v>67.28291493023241</v>
+      </c>
+      <c r="C27">
+        <v>38313</v>
+      </c>
+      <c r="D27">
+        <v>14</v>
+      </c>
+      <c r="E27" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27">
+        <v>0.208076597372706</v>
+      </c>
+      <c r="G27">
+        <v>0.1137574120300403</v>
+      </c>
+      <c r="H27">
+        <v>0.3491171740432566</v>
+      </c>
+      <c r="I27" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28">
+        <v>410810</v>
+      </c>
+      <c r="B28">
+        <v>4.925906682619705</v>
+      </c>
+      <c r="C28">
+        <v>2711</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28" t="s">
+        <v>33</v>
+      </c>
+      <c r="F28">
+        <v>0.2030083118562405</v>
+      </c>
+      <c r="G28">
+        <v>0.005139725458791134</v>
+      </c>
+      <c r="H28">
+        <v>1.131089919059485</v>
+      </c>
+      <c r="I28" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29">
+        <v>410730</v>
+      </c>
+      <c r="B29">
+        <v>12.69243639221791</v>
+      </c>
+      <c r="C29">
+        <v>6517</v>
+      </c>
+      <c r="D29">
+        <v>2</v>
+      </c>
+      <c r="E29" t="s">
+        <v>36</v>
+      </c>
+      <c r="F29">
+        <v>0.1575741597748921</v>
+      </c>
+      <c r="G29">
+        <v>0.01908296177812404</v>
+      </c>
+      <c r="H29">
+        <v>0.5692120444388139</v>
+      </c>
+      <c r="I29" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30">
+        <v>410115</v>
+      </c>
+      <c r="B30">
+        <v>6.072693210742867</v>
+      </c>
+      <c r="C30">
+        <v>3357</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>250</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>0.607453616722831</v>
+      </c>
+      <c r="I30" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31">
+        <v>411160</v>
+      </c>
+      <c r="B31">
+        <v>4.879576017837054</v>
+      </c>
+      <c r="C31">
+        <v>2685</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>251</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0.7559836019829214</v>
+      </c>
+      <c r="I31" t="s">
+        <v>249</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>56</v>
@@ -3920,35 +5286,46 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>252</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1477</v>
       </c>
       <c r="C2">
-        <v>0.1</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="B3">
-        <v>619</v>
+        <v>23</v>
       </c>
       <c r="C3">
-        <v>40.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>231</v>
+        <v>254</v>
       </c>
       <c r="B4">
-        <v>901</v>
+        <v>8</v>
       </c>
       <c r="C4">
-        <v>59.2</v>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>255</v>
+      </c>
+      <c r="B5">
+        <v>14</v>
+      </c>
+      <c r="C5">
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>
@@ -4131,6 +5508,189 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C2">
+        <v>160</v>
+      </c>
+      <c r="D2">
+        <v>392</v>
+      </c>
+      <c r="E2">
+        <v>40.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B3" t="s">
+        <v>260</v>
+      </c>
+      <c r="C3">
+        <v>230</v>
+      </c>
+      <c r="D3">
+        <v>392</v>
+      </c>
+      <c r="E3">
+        <v>58.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>392</v>
+      </c>
+      <c r="E4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" t="s">
+        <v>259</v>
+      </c>
+      <c r="C5">
+        <v>30</v>
+      </c>
+      <c r="D5">
+        <v>56</v>
+      </c>
+      <c r="E5">
+        <v>53.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6">
+        <v>26</v>
+      </c>
+      <c r="D6">
+        <v>56</v>
+      </c>
+      <c r="E6">
+        <v>46.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>56</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B3">
+        <v>619</v>
+      </c>
+      <c r="C3">
+        <v>40.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B4">
+        <v>901</v>
+      </c>
+      <c r="C4">
+        <v>59.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C11"/>

</xml_diff>

<commit_message>
Atualização de dados — 05/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="264">
   <si>
     <t>municipio</t>
   </si>
@@ -72,12 +72,12 @@
     <t>Uniflor</t>
   </si>
   <si>
+    <t>Atalaia</t>
+  </si>
+  <si>
     <t>Ourizona</t>
   </si>
   <si>
-    <t>Atalaia</t>
-  </si>
-  <si>
     <t>Itaguaje</t>
   </si>
   <si>
@@ -126,21 +126,21 @@
     <t>Paicandu</t>
   </si>
   <si>
+    <t>Mandaguacu</t>
+  </si>
+  <si>
     <t>Presidente Castelo Branco</t>
   </si>
   <si>
-    <t>Mandaguacu</t>
-  </si>
-  <si>
     <t>Santa Fe</t>
   </si>
   <si>
+    <t>Mandaguari</t>
+  </si>
+  <si>
     <t>Florida</t>
   </si>
   <si>
-    <t>Mandaguari</t>
-  </si>
-  <si>
     <t>Iguaracu</t>
   </si>
   <si>
@@ -399,66 +399,72 @@
     <t>100,0% (17)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 30,0% (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 80,0% (10)</t>
+    <t xml:space="preserve"> 27,3% (11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 72,7% (11)</t>
+  </si>
+  <si>
+    <t>100,0% (11)</t>
+  </si>
+  <si>
+    <t>100,0% (9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 28,6% (42)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 95,2% (42)</t>
+  </si>
+  <si>
+    <t>100,0% (41)</t>
+  </si>
+  <si>
+    <t>100,0% (40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 50,0% (2)</t>
+  </si>
+  <si>
+    <t>100,0% (2)</t>
+  </si>
+  <si>
+    <t>100,0% (1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 28,6% (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 85,7% (7)</t>
+  </si>
+  <si>
+    <t>100,0% (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 57,1% (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 66,7% (3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 71,4% (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  0,0% (1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  0,0% (2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 10,0% (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 90,0% (10)</t>
   </si>
   <si>
     <t>100,0% (10)</t>
   </si>
   <si>
-    <t>100,0% (9)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 26,8% (41)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 95,1% (41)</t>
-  </si>
-  <si>
-    <t>100,0% (40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 50,0% (2)</t>
-  </si>
-  <si>
-    <t>100,0% (2)</t>
-  </si>
-  <si>
-    <t>100,0% (1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 28,6% (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 85,7% (7)</t>
-  </si>
-  <si>
-    <t>100,0% (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 57,1% (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 66,7% (3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 71,4% (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  0,0% (1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  0,0% (2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 10,0% (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 90,0% (10)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 40,0% (10)</t>
   </si>
   <si>
@@ -471,114 +477,114 @@
     <t>100,0% (3)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 31,2% (16)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 62,5% (16)</t>
-  </si>
-  <si>
-    <t>100,0% (16)</t>
+    <t xml:space="preserve"> 29,4% (17)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 64,7% (17)</t>
   </si>
   <si>
     <t xml:space="preserve"> 81,2% (16)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 42,9% (14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 50,0% (14)</t>
+    <t xml:space="preserve"> 40,0% (15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 46,7% (15)</t>
+  </si>
+  <si>
+    <t>100,0% (15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,9% (14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 27,7% (65)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 55,4% (65)</t>
+  </si>
+  <si>
+    <t>100,0% (4)</t>
+  </si>
+  <si>
+    <t>100,0% (65)</t>
+  </si>
+  <si>
+    <t>100,0% (64)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 29,0% (972)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 77,0% (969)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 98,0% (350)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 99,7% (971)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,8% (934)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 25,0% (8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 87,5% (8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 26,3% (114)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,1% (114)</t>
+  </si>
+  <si>
+    <t>100,0% (112)</t>
+  </si>
+  <si>
+    <t>100,0% (106)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 37,5% (24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 75,0% (24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 95,8% (24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 82,6% (23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 50,0% (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 20,0% (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 60,0% (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 80,0% (5)</t>
+  </si>
+  <si>
+    <t>100,0% (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 25,0% (4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 14,3% (14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 85,7% (14)</t>
   </si>
   <si>
     <t>100,0% (14)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 92,9% (14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 27,7% (65)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 55,4% (65)</t>
-  </si>
-  <si>
-    <t>100,0% (4)</t>
-  </si>
-  <si>
-    <t>100,0% (65)</t>
-  </si>
-  <si>
-    <t>100,0% (64)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 29,0% (965)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 77,3% (962)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 98,0% (350)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 99,7% (964)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,8% (922)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 25,0% (8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 87,5% (8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 26,3% (114)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,1% (114)</t>
-  </si>
-  <si>
-    <t>100,0% (112)</t>
-  </si>
-  <si>
-    <t>100,0% (101)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 37,5% (24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 75,0% (24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 95,8% (24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 82,6% (23)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 50,0% (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 20,0% (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 60,0% (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 80,0% (5)</t>
-  </si>
-  <si>
-    <t>100,0% (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 25,0% (4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 14,3% (14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 85,7% (14)</t>
-  </si>
-  <si>
     <t>100,0% (12)</t>
   </si>
   <si>
@@ -588,16 +594,16 @@
     <t xml:space="preserve"> 83,3% (12)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 24,0% (129)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 69,0% (129)</t>
-  </si>
-  <si>
-    <t>100,0% (129)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 93,7% (127)</t>
+    <t xml:space="preserve"> 24,6% (130)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 68,5% (130)</t>
+  </si>
+  <si>
+    <t>100,0% (130)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 93,8% (128)</t>
   </si>
   <si>
     <t xml:space="preserve">  0,0% (6)</t>
@@ -1206,10 +1212,10 @@
         <v>114</v>
       </c>
       <c r="C2">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2">
         <v>6</v>
@@ -1218,10 +1224,10 @@
         <v>420</v>
       </c>
       <c r="G2">
-        <v>36.8</v>
+        <v>40.5</v>
       </c>
       <c r="H2">
-        <v>9.9</v>
+        <v>10.4</v>
       </c>
       <c r="I2">
         <v>5.3</v>
@@ -1290,19 +1296,19 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>250.5</v>
+        <v>271.9</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1311,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>37.5</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1319,19 +1325,19 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F6">
-        <v>247.2</v>
+        <v>250.5</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1340,7 +1346,7 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1406,25 +1412,25 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>970</v>
+        <v>977</v>
       </c>
       <c r="C9">
-        <v>862</v>
+        <v>883</v>
       </c>
       <c r="D9">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E9">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="F9">
-        <v>225.8</v>
+        <v>227.4</v>
       </c>
       <c r="G9">
-        <v>18.9</v>
+        <v>19.1</v>
       </c>
       <c r="H9">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I9">
         <v>29.6</v>
@@ -1493,7 +1499,7 @@
         <v>19</v>
       </c>
       <c r="B12">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12">
         <v>40</v>
@@ -1505,7 +1511,7 @@
         <v>2</v>
       </c>
       <c r="F12">
-        <v>180.2</v>
+        <v>184.4</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1514,7 +1520,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1638,10 +1644,10 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C17">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D17">
         <v>9</v>
@@ -1650,16 +1656,16 @@
         <v>52</v>
       </c>
       <c r="F17">
-        <v>103</v>
+        <v>104.6</v>
       </c>
       <c r="G17">
         <v>7</v>
       </c>
       <c r="H17">
-        <v>7</v>
+        <v>6.9</v>
       </c>
       <c r="I17">
-        <v>39.4</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1812,28 +1818,28 @@
         <v>30</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C23">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F23">
-        <v>46.5</v>
+        <v>49.2</v>
       </c>
       <c r="G23">
-        <v>23.2</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>41.2</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1841,28 +1847,28 @@
         <v>31</v>
       </c>
       <c r="B24">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C24">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F24">
-        <v>46.3</v>
+        <v>46.5</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>23.2</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I24">
-        <v>43.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1899,25 +1905,28 @@
         <v>33</v>
       </c>
       <c r="B26">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="D26">
         <v>0</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F26">
-        <v>36.9</v>
+        <v>39.2</v>
       </c>
       <c r="G26">
         <v>0</v>
       </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
       <c r="I26">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1925,28 +1934,25 @@
         <v>34</v>
       </c>
       <c r="B27">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C27">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="D27">
         <v>0</v>
       </c>
       <c r="E27">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F27">
-        <v>36.5</v>
+        <v>36.9</v>
       </c>
       <c r="G27">
         <v>0</v>
       </c>
-      <c r="H27">
-        <v>0</v>
-      </c>
       <c r="I27">
-        <v>78.59999999999999</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -2036,13 +2042,13 @@
         <v>96</v>
       </c>
       <c r="B2">
-        <v>1509</v>
+        <v>1521</v>
       </c>
       <c r="C2">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="D2">
-        <v>28.4</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2050,13 +2056,13 @@
         <v>97</v>
       </c>
       <c r="B3">
-        <v>1506</v>
+        <v>1518</v>
       </c>
       <c r="C3">
-        <v>1162</v>
+        <v>1166</v>
       </c>
       <c r="D3">
-        <v>77.2</v>
+        <v>76.8</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2078,10 +2084,10 @@
         <v>99</v>
       </c>
       <c r="B5">
-        <v>1504</v>
+        <v>1516</v>
       </c>
       <c r="C5">
-        <v>1497</v>
+        <v>1509</v>
       </c>
       <c r="D5">
         <v>99.5</v>
@@ -2092,10 +2098,10 @@
         <v>100</v>
       </c>
       <c r="B6">
-        <v>1434</v>
+        <v>1453</v>
       </c>
       <c r="C6">
-        <v>1351</v>
+        <v>1368</v>
       </c>
       <c r="D6">
         <v>94.2</v>
@@ -2142,7 +2148,7 @@
         <v>104</v>
       </c>
       <c r="B2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C2">
         <v>4</v>
@@ -2154,7 +2160,7 @@
         <v>10254</v>
       </c>
       <c r="F2">
-        <v>2672.1</v>
+        <v>2681.9</v>
       </c>
       <c r="G2">
         <v>39</v>
@@ -2168,25 +2174,25 @@
         <v>105</v>
       </c>
       <c r="B3">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E3">
         <v>42663</v>
       </c>
       <c r="F3">
-        <v>602.4</v>
+        <v>625.8</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>133.6</v>
+        <v>138.3</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2376,7 +2382,7 @@
         <v>113</v>
       </c>
       <c r="B11">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C11">
         <v>15</v>
@@ -2388,7 +2394,7 @@
         <v>91102</v>
       </c>
       <c r="F11">
-        <v>160.3</v>
+        <v>162.5</v>
       </c>
       <c r="G11">
         <v>16.5</v>
@@ -2408,7 +2414,7 @@
         <v>27</v>
       </c>
       <c r="D12">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E12">
         <v>53206</v>
@@ -2420,7 +2426,7 @@
         <v>50.7</v>
       </c>
       <c r="H12">
-        <v>105.3</v>
+        <v>107.1</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2431,10 +2437,10 @@
         <v>319</v>
       </c>
       <c r="C13">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D13">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E13">
         <v>23417</v>
@@ -2443,10 +2449,10 @@
         <v>1362.3</v>
       </c>
       <c r="G13">
-        <v>217.8</v>
+        <v>226.3</v>
       </c>
       <c r="H13">
-        <v>324.6</v>
+        <v>328.8</v>
       </c>
     </row>
   </sheetData>
@@ -2501,7 +2507,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>121</v>
@@ -2536,7 +2542,7 @@
         <v>127</v>
       </c>
       <c r="F4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2544,19 +2550,19 @@
         <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2564,19 +2570,19 @@
         <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D6" t="s">
         <v>118</v>
       </c>
       <c r="E6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2584,39 +2590,39 @@
         <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E8" t="s">
         <v>118</v>
       </c>
       <c r="F8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2624,19 +2630,19 @@
         <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D9" t="s">
+        <v>131</v>
+      </c>
+      <c r="E9" t="s">
         <v>130</v>
       </c>
-      <c r="E9" t="s">
-        <v>129</v>
-      </c>
       <c r="F9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2644,19 +2650,19 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D10" t="s">
         <v>118</v>
       </c>
       <c r="E10" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="F10" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2664,19 +2670,19 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C11" t="s">
+        <v>144</v>
+      </c>
+      <c r="D11" t="s">
+        <v>131</v>
+      </c>
+      <c r="E11" t="s">
         <v>142</v>
       </c>
-      <c r="D11" t="s">
-        <v>130</v>
-      </c>
-      <c r="E11" t="s">
-        <v>123</v>
-      </c>
       <c r="F11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2684,59 +2690,59 @@
         <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D12" t="s">
         <v>118</v>
       </c>
       <c r="E12" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F12" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C13" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E13" t="s">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="F13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C14" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2744,19 +2750,19 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C15" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2764,19 +2770,19 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D16" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E16" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2784,19 +2790,19 @@
         <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C17" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D17" t="s">
         <v>118</v>
       </c>
       <c r="E17" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2804,19 +2810,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D18" t="s">
         <v>118</v>
       </c>
       <c r="E18" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2824,39 +2830,39 @@
         <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E19" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D20" t="s">
         <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F20" t="s">
-        <v>133</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2864,19 +2870,19 @@
         <v>29</v>
       </c>
       <c r="B21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D21" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2884,39 +2890,39 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C22" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E22" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="F22" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D23" t="s">
         <v>118</v>
       </c>
       <c r="E23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2924,19 +2930,19 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D24" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E24" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F24" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2944,19 +2950,19 @@
         <v>10</v>
       </c>
       <c r="B25" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D25" t="s">
         <v>118</v>
       </c>
       <c r="E25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2964,19 +2970,19 @@
         <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C26" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D26" t="s">
         <v>118</v>
       </c>
       <c r="E26" t="s">
-        <v>151</v>
+        <v>182</v>
       </c>
       <c r="F26" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2984,19 +2990,19 @@
         <v>15</v>
       </c>
       <c r="B27" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C27" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D27" t="s">
         <v>118</v>
       </c>
       <c r="E27" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F27" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -3004,19 +3010,19 @@
         <v>24</v>
       </c>
       <c r="B28" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C28" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F28" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -3024,19 +3030,19 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D29" t="s">
         <v>118</v>
       </c>
       <c r="E29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F29" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -3051,7 +3057,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3060,24 +3066,24 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B2" t="s">
         <v>24</v>
@@ -3103,13 +3109,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -3118,7 +3124,7 @@
         <v>5</v>
       </c>
       <c r="F3">
-        <v>38</v>
+        <v>37.6</v>
       </c>
       <c r="G3">
         <v>97</v>
@@ -3129,13 +3135,13 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
       <c r="C4">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -3144,7 +3150,7 @@
         <v>5</v>
       </c>
       <c r="F4">
-        <v>38.7</v>
+        <v>38.5</v>
       </c>
       <c r="G4">
         <v>98.40000000000001</v>
@@ -3155,13 +3161,13 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
       </c>
       <c r="C5">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -3170,7 +3176,7 @@
         <v>5</v>
       </c>
       <c r="F5">
-        <v>41</v>
+        <v>40.9</v>
       </c>
       <c r="G5">
         <v>97.59999999999999</v>
@@ -3181,22 +3187,22 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F6">
-        <v>50</v>
+        <v>45.5</v>
       </c>
       <c r="G6">
         <v>100</v>
@@ -3207,7 +3213,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
@@ -3233,13 +3239,13 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
       <c r="C8">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -3248,7 +3254,7 @@
         <v>4</v>
       </c>
       <c r="F8">
-        <v>57</v>
+        <v>56.6</v>
       </c>
       <c r="G8">
         <v>99.2</v>
@@ -3259,13 +3265,13 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
       </c>
       <c r="C9">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -3274,10 +3280,10 @@
         <v>5</v>
       </c>
       <c r="F9">
-        <v>65.59999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="G9">
-        <v>96.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -3285,7 +3291,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B10" t="s">
         <v>16</v>
@@ -3311,7 +3317,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
@@ -3337,13 +3343,13 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
       </c>
       <c r="C12">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -3352,7 +3358,7 @@
         <v>4</v>
       </c>
       <c r="F12">
-        <v>80</v>
+        <v>80.2</v>
       </c>
       <c r="G12">
         <v>98.8</v>
@@ -3363,7 +3369,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
@@ -3389,7 +3395,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
@@ -3415,7 +3421,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -3441,13 +3447,13 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
       </c>
       <c r="C16">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -3467,7 +3473,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -3493,7 +3499,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
@@ -3519,10 +3525,10 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -3558,25 +3564,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3768,16 +3774,16 @@
         <v>46266</v>
       </c>
       <c r="B10">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E10">
-        <v>92.3</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="F10">
         <v>100</v>
@@ -3798,62 +3804,62 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
       <c r="C2">
-        <v>1515</v>
+        <v>1528</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B3">
-        <v>878</v>
+        <v>886</v>
       </c>
       <c r="C3">
-        <v>1522</v>
+        <v>1535</v>
       </c>
       <c r="D3">
         <v>57.7</v>
       </c>
       <c r="E3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3868,13 +3874,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>56</v>
@@ -3882,21 +3888,21 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B2">
-        <v>1487</v>
+        <v>1504</v>
       </c>
       <c r="C2">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B3">
         <v>387</v>
@@ -3910,10 +3916,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B4">
-        <v>1533</v>
+        <v>1545</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -3924,10 +3930,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B5">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -3938,10 +3944,10 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B6">
-        <v>1400</v>
+        <v>1428</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -3952,10 +3958,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B7">
-        <v>1389</v>
+        <v>1417</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -3976,27 +3982,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>56</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -4011,52 +4017,52 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D3">
         <v>4</v>
       </c>
       <c r="E3">
-        <v>5.6</v>
+        <v>5.3</v>
       </c>
       <c r="F3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D4">
         <v>5</v>
       </c>
       <c r="E4">
-        <v>5.1</v>
+        <v>5</v>
       </c>
       <c r="F4" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
@@ -4071,12 +4077,12 @@
         <v>2.6</v>
       </c>
       <c r="F5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B6" t="s">
         <v>24</v>
@@ -4091,138 +4097,138 @@
         <v>2.4</v>
       </c>
       <c r="F6" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="C7">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="F7" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
       </c>
       <c r="C8">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="F8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C9">
-        <v>63</v>
+        <v>131</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="F9" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C10">
-        <v>131</v>
+        <v>284</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>1.5</v>
+        <v>1.1</v>
       </c>
       <c r="F10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C11">
-        <v>280</v>
+        <v>102</v>
       </c>
       <c r="D11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C12">
-        <v>101</v>
+        <v>155</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>231</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
       </c>
       <c r="C13">
-        <v>154</v>
+        <v>101</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -4236,7 +4242,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
@@ -4256,7 +4262,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
@@ -4276,7 +4282,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
@@ -4296,7 +4302,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -4316,7 +4322,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B18" t="s">
         <v>24</v>
@@ -4336,10 +4342,10 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -4351,7 +4357,7 @@
         <v>16.7</v>
       </c>
       <c r="F19" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -4366,31 +4372,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>102</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -4398,7 +4404,7 @@
         <v>411690</v>
       </c>
       <c r="B2">
-        <v>47.59190958417413</v>
+        <v>47.96421738600731</v>
       </c>
       <c r="C2">
         <v>27142</v>
@@ -4410,16 +4416,16 @@
         <v>9</v>
       </c>
       <c r="F2">
-        <v>2.395365115542847</v>
+        <v>2.376771814758254</v>
       </c>
       <c r="G2">
-        <v>1.975880837385551</v>
+        <v>1.960543657059412</v>
       </c>
       <c r="H2">
-        <v>2.87756521607562</v>
+        <v>2.855228982136748</v>
       </c>
       <c r="I2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -4427,7 +4433,7 @@
         <v>412360</v>
       </c>
       <c r="B3">
-        <v>3.120055957676751</v>
+        <v>3.144135478454948</v>
       </c>
       <c r="C3">
         <v>1745</v>
@@ -4439,16 +4445,16 @@
         <v>10</v>
       </c>
       <c r="F3">
-        <v>1.60253536084753</v>
+        <v>1.590262262635399</v>
       </c>
       <c r="G3">
-        <v>0.5203388696038955</v>
+        <v>0.5163538280214993</v>
       </c>
       <c r="H3">
-        <v>3.739782951845233</v>
+        <v>3.711141634728976</v>
       </c>
       <c r="I3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -4456,7 +4462,7 @@
         <v>412830</v>
       </c>
       <c r="B4">
-        <v>3.820820242331692</v>
+        <v>3.846634840978511</v>
       </c>
       <c r="C4">
         <v>2106</v>
@@ -4468,16 +4474,16 @@
         <v>11</v>
       </c>
       <c r="F4">
-        <v>1.570343439224045</v>
+        <v>1.559804932893946</v>
       </c>
       <c r="G4">
-        <v>0.5762883658057475</v>
+        <v>0.5724209197176435</v>
       </c>
       <c r="H4">
-        <v>3.417976558496512</v>
+        <v>3.395038666887498</v>
       </c>
       <c r="I4" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -4485,28 +4491,28 @@
         <v>410220</v>
       </c>
       <c r="B5">
-        <v>7.182495033139207</v>
+        <v>7.229864258194739</v>
       </c>
       <c r="C5">
         <v>4046</v>
       </c>
       <c r="D5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F5">
-        <v>1.392273848274332</v>
+        <v>1.521467016138232</v>
       </c>
       <c r="G5">
-        <v>0.6676494273935535</v>
+        <v>0.7595108526433044</v>
       </c>
       <c r="H5">
-        <v>2.56044117777552</v>
+        <v>2.722324764395571</v>
       </c>
       <c r="I5" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -4514,7 +4520,7 @@
         <v>411090</v>
       </c>
       <c r="B6">
-        <v>7.925565257205213</v>
+        <v>7.99422861813144</v>
       </c>
       <c r="C6">
         <v>4530</v>
@@ -4526,16 +4532,16 @@
         <v>14</v>
       </c>
       <c r="F6">
-        <v>1.387913624204884</v>
+        <v>1.375992672395091</v>
       </c>
       <c r="G6">
-        <v>0.6928414805801728</v>
+        <v>0.6868905843876572</v>
       </c>
       <c r="H6">
-        <v>2.483360854976093</v>
+        <v>2.462030979281952</v>
       </c>
       <c r="I6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -4543,28 +4549,28 @@
         <v>411520</v>
       </c>
       <c r="B7">
-        <v>708.618739424934</v>
+        <v>714.2098872198766</v>
       </c>
       <c r="C7">
         <v>429660</v>
       </c>
       <c r="D7">
-        <v>970</v>
+        <v>977</v>
       </c>
       <c r="E7" t="s">
         <v>16</v>
       </c>
       <c r="F7">
-        <v>1.368860214996833</v>
+        <v>1.36794521818097</v>
       </c>
       <c r="G7">
-        <v>1.284061260184467</v>
+        <v>1.283502241155937</v>
       </c>
       <c r="H7">
-        <v>1.457787801171709</v>
+        <v>1.456484349211052</v>
       </c>
       <c r="I7" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -4572,7 +4578,7 @@
         <v>411740</v>
       </c>
       <c r="B8">
-        <v>5.887620794244284</v>
+        <v>5.9266473822138</v>
       </c>
       <c r="C8">
         <v>3193</v>
@@ -4581,19 +4587,19 @@
         <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>1.358783162091684</v>
+        <v>1.34983566324672</v>
       </c>
       <c r="G8">
-        <v>0.5866261258070417</v>
+        <v>0.5827632308805218</v>
       </c>
       <c r="H8">
-        <v>2.677344511657977</v>
+        <v>2.659714371990398</v>
       </c>
       <c r="I8" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -4601,7 +4607,7 @@
         <v>411640</v>
       </c>
       <c r="B9">
-        <v>6.05448539639124</v>
+        <v>6.106002803986375</v>
       </c>
       <c r="C9">
         <v>3669</v>
@@ -4613,16 +4619,16 @@
         <v>17</v>
       </c>
       <c r="F9">
-        <v>1.321334428317951</v>
+        <v>1.310186099943667</v>
       </c>
       <c r="G9">
-        <v>0.5704584205962656</v>
+        <v>0.5656453636892579</v>
       </c>
       <c r="H9">
-        <v>2.603555577091477</v>
+        <v>2.581588925884891</v>
       </c>
       <c r="I9" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -4630,7 +4636,7 @@
         <v>412530</v>
       </c>
       <c r="B10">
-        <v>9.881799363449487</v>
+        <v>9.943131633395389</v>
       </c>
       <c r="C10">
         <v>5170</v>
@@ -4642,16 +4648,16 @@
         <v>15</v>
       </c>
       <c r="F10">
-        <v>1.214353738488686</v>
+        <v>1.20686323408375</v>
       </c>
       <c r="G10">
-        <v>0.627474297004726</v>
+        <v>0.6236038440743078</v>
       </c>
       <c r="H10">
-        <v>2.121231597325185</v>
+        <v>2.108147193563702</v>
       </c>
       <c r="I10" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -4659,7 +4665,7 @@
         <v>412450</v>
       </c>
       <c r="B11">
-        <v>11.61148021598628</v>
+        <v>11.71986363210249</v>
       </c>
       <c r="C11">
         <v>6463</v>
@@ -4671,16 +4677,16 @@
         <v>18</v>
       </c>
       <c r="F11">
-        <v>1.205703298768515</v>
+        <v>1.194553148353354</v>
       </c>
       <c r="G11">
-        <v>0.6591692130485598</v>
+        <v>0.6530733220594237</v>
       </c>
       <c r="H11">
-        <v>2.022965262387124</v>
+        <v>2.00425720462258</v>
       </c>
       <c r="I11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -4688,28 +4694,28 @@
         <v>410590</v>
       </c>
       <c r="B12">
-        <v>40.65070550415243</v>
+        <v>40.96748889977696</v>
       </c>
       <c r="C12">
         <v>23313</v>
       </c>
       <c r="D12">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E12" t="s">
         <v>19</v>
       </c>
       <c r="F12">
-        <v>1.033192400454396</v>
+        <v>1.049612782106206</v>
       </c>
       <c r="G12">
-        <v>0.744634203934927</v>
+        <v>0.7596099748290065</v>
       </c>
       <c r="H12">
-        <v>1.396575977572922</v>
+        <v>1.413821529361517</v>
       </c>
       <c r="I12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -4717,7 +4723,7 @@
         <v>411110</v>
       </c>
       <c r="B13">
-        <v>10.71960483015752</v>
+        <v>10.79983434460729</v>
       </c>
       <c r="C13">
         <v>6228</v>
@@ -4729,16 +4735,16 @@
         <v>20</v>
       </c>
       <c r="F13">
-        <v>0.9328702091579858</v>
+        <v>0.9259401284236665</v>
       </c>
       <c r="G13">
-        <v>0.4473475255954904</v>
+        <v>0.4440242825138264</v>
       </c>
       <c r="H13">
-        <v>1.715581528740695</v>
+        <v>1.702836863530289</v>
       </c>
       <c r="I13" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -4746,7 +4752,7 @@
         <v>411480</v>
       </c>
       <c r="B14">
-        <v>76.1402973292391</v>
+        <v>76.80636875810966</v>
       </c>
       <c r="C14">
         <v>44749</v>
@@ -4758,16 +4764,16 @@
         <v>22</v>
       </c>
       <c r="F14">
-        <v>0.8536872363255003</v>
+        <v>0.8462839872655342</v>
       </c>
       <c r="G14">
-        <v>0.6588577860723676</v>
+        <v>0.6531441147442282</v>
       </c>
       <c r="H14">
-        <v>1.088094461433849</v>
+        <v>1.078658412778094</v>
       </c>
       <c r="I14" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -4775,7 +4781,7 @@
         <v>410780</v>
       </c>
       <c r="B15">
-        <v>9.655942925034168</v>
+        <v>9.716834185999264</v>
       </c>
       <c r="C15">
         <v>4805</v>
@@ -4787,16 +4793,16 @@
         <v>21</v>
       </c>
       <c r="F15">
-        <v>0.7249421474780755</v>
+        <v>0.7203992438284189</v>
       </c>
       <c r="G15">
-        <v>0.2914643420502517</v>
+        <v>0.2896378591676504</v>
       </c>
       <c r="H15">
-        <v>1.493657892727379</v>
+        <v>1.484297774936166</v>
       </c>
       <c r="I15" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -4804,28 +4810,28 @@
         <v>412625</v>
       </c>
       <c r="B16">
-        <v>202.9578045524855</v>
+        <v>205.1262256501793</v>
       </c>
       <c r="C16">
         <v>128106</v>
       </c>
       <c r="D16">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E16" t="s">
         <v>24</v>
       </c>
       <c r="F16">
-        <v>0.6503814932914512</v>
+        <v>0.6532563038941817</v>
       </c>
       <c r="G16">
-        <v>0.5441688170690743</v>
+        <v>0.5473373897687619</v>
       </c>
       <c r="H16">
-        <v>0.7712694703079357</v>
+        <v>0.7736923554173603</v>
       </c>
       <c r="I16" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -4833,7 +4839,7 @@
         <v>411810</v>
       </c>
       <c r="B17">
-        <v>15.98585273920547</v>
+        <v>16.11760058906637</v>
       </c>
       <c r="C17">
         <v>9549</v>
@@ -4845,16 +4851,16 @@
         <v>23</v>
       </c>
       <c r="F17">
-        <v>0.6255531164424465</v>
+        <v>0.6204397450315068</v>
       </c>
       <c r="G17">
-        <v>0.2999770343418524</v>
+        <v>0.2975249739955377</v>
       </c>
       <c r="H17">
-        <v>1.15041445345704</v>
+        <v>1.141010781374814</v>
       </c>
       <c r="I17" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -4862,7 +4868,7 @@
         <v>410210</v>
       </c>
       <c r="B18">
-        <v>47.85677468621944</v>
+        <v>48.22934288769908</v>
       </c>
       <c r="C18">
         <v>26203</v>
@@ -4874,16 +4880,16 @@
         <v>26</v>
       </c>
       <c r="F18">
-        <v>0.3970179796815921</v>
+        <v>0.3939510443723247</v>
       </c>
       <c r="G18">
-        <v>0.2390307587456517</v>
+        <v>0.2371842633436401</v>
       </c>
       <c r="H18">
-        <v>0.6199927547589087</v>
+        <v>0.6152033553654982</v>
       </c>
       <c r="I18" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -4891,7 +4897,7 @@
         <v>411360</v>
       </c>
       <c r="B19">
-        <v>7.671612549406151</v>
+        <v>7.730903745984839</v>
       </c>
       <c r="C19">
         <v>4707</v>
@@ -4903,16 +4909,16 @@
         <v>27</v>
       </c>
       <c r="F19">
-        <v>0.3910520742125104</v>
+        <v>0.3880529493797016</v>
       </c>
       <c r="G19">
-        <v>0.08064433897192734</v>
+        <v>0.08002584732954644</v>
       </c>
       <c r="H19">
-        <v>1.142820106370073</v>
+        <v>1.134055390910246</v>
       </c>
       <c r="I19" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -4920,7 +4926,7 @@
         <v>411630</v>
       </c>
       <c r="B20">
-        <v>7.932381828941635</v>
+        <v>7.99254170451731</v>
       </c>
       <c r="C20">
         <v>4057</v>
@@ -4932,16 +4938,16 @@
         <v>25</v>
       </c>
       <c r="F20">
-        <v>0.3781966204720972</v>
+        <v>0.3753499338394979</v>
       </c>
       <c r="G20">
-        <v>0.07799323535313815</v>
+        <v>0.07740618013240189</v>
       </c>
       <c r="H20">
-        <v>1.105251015244192</v>
+        <v>1.096931788893531</v>
       </c>
       <c r="I20" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -4949,7 +4955,7 @@
         <v>410790</v>
       </c>
       <c r="B21">
-        <v>19.89931648618882</v>
+        <v>20.09957764655562</v>
       </c>
       <c r="C21">
         <v>11522</v>
@@ -4961,16 +4967,16 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>0.3517708763945923</v>
+        <v>0.3482660244455216</v>
       </c>
       <c r="G21">
-        <v>0.1414301367322432</v>
+        <v>0.140021004471313</v>
       </c>
       <c r="H21">
-        <v>0.7247824502772484</v>
+        <v>0.7175611157269233</v>
       </c>
       <c r="I21" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -4978,7 +4984,7 @@
         <v>411750</v>
       </c>
       <c r="B22">
-        <v>79.20952501920122</v>
+        <v>80.00855318129641</v>
       </c>
       <c r="C22">
         <v>48695</v>
@@ -4990,74 +4996,74 @@
         <v>29</v>
       </c>
       <c r="F22">
-        <v>0.3029938633539609</v>
+        <v>0.299967928999002</v>
       </c>
       <c r="G22">
-        <v>0.1941338854255072</v>
+        <v>0.1921951121880954</v>
       </c>
       <c r="H22">
-        <v>0.4508308512782611</v>
+        <v>0.4463285008145998</v>
       </c>
       <c r="I22" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23">
-        <v>412040</v>
+        <v>411410</v>
       </c>
       <c r="B23">
-        <v>7.037976950852113</v>
+        <v>59.38056063714926</v>
       </c>
       <c r="C23">
-        <v>4304</v>
+        <v>34521</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="E23" t="s">
         <v>30</v>
       </c>
       <c r="F23">
-        <v>0.2841725703233303</v>
+        <v>0.2862889776989505</v>
       </c>
       <c r="G23">
-        <v>0.03441461661999898</v>
+        <v>0.1667738795886639</v>
       </c>
       <c r="H23">
-        <v>1.026529032160192</v>
+        <v>0.4583763865455704</v>
       </c>
       <c r="I23" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24">
-        <v>411410</v>
+        <v>412040</v>
       </c>
       <c r="B24">
-        <v>58.77064219403454</v>
+        <v>7.100523496262464</v>
       </c>
       <c r="C24">
-        <v>34521</v>
+        <v>4304</v>
       </c>
       <c r="D24">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E24" t="s">
         <v>31</v>
       </c>
       <c r="F24">
-        <v>0.2722447705637639</v>
+        <v>0.2816693728360662</v>
       </c>
       <c r="G24">
-        <v>0.1556114092380943</v>
+        <v>0.03411146779127732</v>
       </c>
       <c r="H24">
-        <v>0.4421084512191757</v>
+        <v>1.017486622152134</v>
       </c>
       <c r="I24" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -5065,7 +5071,7 @@
         <v>412340</v>
       </c>
       <c r="B25">
-        <v>20.57924830121171</v>
+        <v>20.73664061668979</v>
       </c>
       <c r="C25">
         <v>11730</v>
@@ -5077,74 +5083,74 @@
         <v>32</v>
       </c>
       <c r="F25">
-        <v>0.2429631989865053</v>
+        <v>0.2411190940916328</v>
       </c>
       <c r="G25">
-        <v>0.07888948937084499</v>
+        <v>0.07829071353108977</v>
       </c>
       <c r="H25">
-        <v>0.5669950577658192</v>
+        <v>0.562691532105324</v>
       </c>
       <c r="I25" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26">
-        <v>411000</v>
+        <v>411420</v>
       </c>
       <c r="B26">
-        <v>9.383815600487981</v>
+        <v>67.84653078949061</v>
       </c>
       <c r="C26">
-        <v>5693</v>
+        <v>38313</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F26">
-        <v>0.2131329179034587</v>
+        <v>0.2210872070458685</v>
       </c>
       <c r="G26">
-        <v>0.02581138513968341</v>
+        <v>0.1237408314779118</v>
       </c>
       <c r="H26">
-        <v>0.7699093817815704</v>
+        <v>0.3646497261333528</v>
       </c>
       <c r="I26" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27">
-        <v>411420</v>
+        <v>411000</v>
       </c>
       <c r="B27">
-        <v>67.28291493023241</v>
+        <v>9.470975222399511</v>
       </c>
       <c r="C27">
-        <v>38313</v>
+        <v>5693</v>
       </c>
       <c r="D27">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E27" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F27">
-        <v>0.208076597372706</v>
+        <v>0.2111714953355449</v>
       </c>
       <c r="G27">
-        <v>0.1137574120300403</v>
+        <v>0.02557384776713629</v>
       </c>
       <c r="H27">
-        <v>0.3491171740432566</v>
+        <v>0.7628240490627693</v>
       </c>
       <c r="I27" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -5152,7 +5158,7 @@
         <v>410810</v>
       </c>
       <c r="B28">
-        <v>4.925906682619705</v>
+        <v>4.967466015473944</v>
       </c>
       <c r="C28">
         <v>2711</v>
@@ -5161,19 +5167,19 @@
         <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F28">
-        <v>0.2030083118562405</v>
+        <v>0.2013098825205733</v>
       </c>
       <c r="G28">
-        <v>0.005139725458791134</v>
+        <v>0.005096724950995828</v>
       </c>
       <c r="H28">
-        <v>1.131089919059485</v>
+        <v>1.121626876476438</v>
       </c>
       <c r="I28" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -5181,7 +5187,7 @@
         <v>410730</v>
       </c>
       <c r="B29">
-        <v>12.69243639221791</v>
+        <v>12.78288564558409</v>
       </c>
       <c r="C29">
         <v>6517</v>
@@ -5193,16 +5199,16 @@
         <v>36</v>
       </c>
       <c r="F29">
-        <v>0.1575741597748921</v>
+        <v>0.1564591951654445</v>
       </c>
       <c r="G29">
-        <v>0.01908296177812404</v>
+        <v>0.01894793439129586</v>
       </c>
       <c r="H29">
-        <v>0.5692120444388139</v>
+        <v>0.5651844089069015</v>
       </c>
       <c r="I29" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -5210,7 +5216,7 @@
         <v>410115</v>
       </c>
       <c r="B30">
-        <v>6.072693210742867</v>
+        <v>6.125098715851931</v>
       </c>
       <c r="C30">
         <v>3357</v>
@@ -5219,7 +5225,7 @@
         <v>0</v>
       </c>
       <c r="E30" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F30">
         <v>0</v>
@@ -5228,10 +5234,10 @@
         <v>0</v>
       </c>
       <c r="H30">
-        <v>0.607453616722831</v>
+        <v>0.6022563268355186</v>
       </c>
       <c r="I30" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -5239,7 +5245,7 @@
         <v>411160</v>
       </c>
       <c r="B31">
-        <v>4.879576017837054</v>
+        <v>4.909434013964724</v>
       </c>
       <c r="C31">
         <v>2685</v>
@@ -5248,19 +5254,19 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
+        <v>253</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0.7513858916569688</v>
+      </c>
+      <c r="I31" t="s">
         <v>251</v>
-      </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
-      <c r="G31">
-        <v>0</v>
-      </c>
-      <c r="H31">
-        <v>0.7559836019829214</v>
-      </c>
-      <c r="I31" t="s">
-        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -5275,7 +5281,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -5286,10 +5292,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B2">
-        <v>1477</v>
+        <v>1489</v>
       </c>
       <c r="C2">
         <v>97</v>
@@ -5297,7 +5303,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B3">
         <v>23</v>
@@ -5308,7 +5314,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B4">
         <v>8</v>
@@ -5319,13 +5325,13 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B5">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5354,10 +5360,10 @@
         <v>40</v>
       </c>
       <c r="B2">
-        <v>60.9</v>
+        <v>60.8</v>
       </c>
       <c r="C2">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5365,10 +5371,10 @@
         <v>41</v>
       </c>
       <c r="B3">
-        <v>61.3</v>
+        <v>61.2</v>
       </c>
       <c r="C3">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5379,7 +5385,7 @@
         <v>61.4</v>
       </c>
       <c r="C4">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5390,7 +5396,7 @@
         <v>61.4</v>
       </c>
       <c r="C5">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -5398,10 +5404,10 @@
         <v>44</v>
       </c>
       <c r="B6">
-        <v>90.5</v>
+        <v>91.5</v>
       </c>
       <c r="C6">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5409,10 +5415,10 @@
         <v>45</v>
       </c>
       <c r="B7">
-        <v>95.7</v>
+        <v>96</v>
       </c>
       <c r="C7">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5423,7 +5429,7 @@
         <v>98.7</v>
       </c>
       <c r="C8">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -5431,10 +5437,10 @@
         <v>47</v>
       </c>
       <c r="B9">
-        <v>98.90000000000001</v>
+        <v>98.8</v>
       </c>
       <c r="C9">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -5445,7 +5451,7 @@
         <v>99.09999999999999</v>
       </c>
       <c r="C10">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -5456,7 +5462,7 @@
         <v>99.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -5467,7 +5473,7 @@
         <v>100</v>
       </c>
       <c r="C12">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -5478,7 +5484,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -5489,7 +5495,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -5500,7 +5506,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1522</v>
+        <v>1535</v>
       </c>
     </row>
   </sheetData>
@@ -5515,10 +5521,10 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>55</v>
@@ -5532,10 +5538,10 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C2">
         <v>160</v>
@@ -5549,10 +5555,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C3">
         <v>230</v>
@@ -5566,7 +5572,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B4" t="s">
         <v>82</v>
@@ -5586,16 +5592,16 @@
         <v>92</v>
       </c>
       <c r="B5" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C5">
         <v>30</v>
       </c>
       <c r="D5">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E5">
-        <v>53.6</v>
+        <v>52.6</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -5603,16 +5609,16 @@
         <v>92</v>
       </c>
       <c r="B6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C6">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E6">
-        <v>46.4</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -5626,7 +5632,7 @@
         <v>0</v>
       </c>
       <c r="D7">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -5644,7 +5650,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>77</v>
@@ -5666,10 +5672,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B3">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="C3">
         <v>40.7</v>
@@ -5677,10 +5683,10 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B4">
-        <v>901</v>
+        <v>908</v>
       </c>
       <c r="C4">
         <v>59.2</v>
@@ -5712,10 +5718,10 @@
         <v>42</v>
       </c>
       <c r="B2">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="C2">
-        <v>30.3</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5723,7 +5729,7 @@
         <v>41</v>
       </c>
       <c r="B3">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C3">
         <v>15.2</v>
@@ -5734,10 +5740,10 @@
         <v>57</v>
       </c>
       <c r="B4">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C4">
-        <v>12.5</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5748,7 +5754,7 @@
         <v>181</v>
       </c>
       <c r="C5">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -5759,7 +5765,7 @@
         <v>167</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5767,10 +5773,10 @@
         <v>60</v>
       </c>
       <c r="B7">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C7">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5803,7 +5809,7 @@
         <v>16</v>
       </c>
       <c r="C10">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -5849,10 +5855,10 @@
         <v>65</v>
       </c>
       <c r="B2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -5866,10 +5872,10 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="C3">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -5954,7 +5960,7 @@
         <v>50</v>
       </c>
       <c r="C8">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -5971,13 +5977,13 @@
         <v>93</v>
       </c>
       <c r="C9">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -6005,7 +6011,7 @@
         <v>128</v>
       </c>
       <c r="C11">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -6019,16 +6025,16 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="C12">
-        <v>601</v>
+        <v>621</v>
       </c>
       <c r="D12">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E12">
-        <v>15.5</v>
+        <v>15.3</v>
       </c>
     </row>
   </sheetData>
@@ -6060,13 +6066,13 @@
         <v>65</v>
       </c>
       <c r="B2">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C2">
         <v>64</v>
       </c>
       <c r="D2">
-        <v>43.8</v>
+        <v>43.5</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -6074,13 +6080,13 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="C3">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D3">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -6200,13 +6206,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="C12">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D12">
-        <v>28.9</v>
+        <v>29.1</v>
       </c>
     </row>
   </sheetData>
@@ -6235,10 +6241,10 @@
         <v>78</v>
       </c>
       <c r="B2">
-        <v>871</v>
+        <v>878</v>
       </c>
       <c r="C2">
-        <v>98.90000000000001</v>
+        <v>98.8</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6246,10 +6252,10 @@
         <v>79</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6289,10 +6295,10 @@
         <v>82</v>
       </c>
       <c r="B2">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C2">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6300,10 +6306,10 @@
         <v>83</v>
       </c>
       <c r="B3">
-        <v>1130</v>
+        <v>1140</v>
       </c>
       <c r="C3">
-        <v>74.2</v>
+        <v>74.3</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6314,7 +6320,7 @@
         <v>376</v>
       </c>
       <c r="C4">
-        <v>24.7</v>
+        <v>24.5</v>
       </c>
     </row>
   </sheetData>
@@ -6412,22 +6418,22 @@
         <v>92</v>
       </c>
       <c r="B2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D2">
-        <v>73.2</v>
+        <v>73.7</v>
       </c>
       <c r="E2">
         <v>15</v>
       </c>
       <c r="F2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G2">
-        <v>51.2</v>
+        <v>52.4</v>
       </c>
       <c r="H2">
         <v>2</v>
@@ -6438,22 +6444,22 @@
         <v>93</v>
       </c>
       <c r="B3">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="C3">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D3">
         <v>68.2</v>
       </c>
       <c r="E3">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F3">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G3">
-        <v>52.4</v>
+        <v>51.8</v>
       </c>
       <c r="H3">
         <v>2</v>

</xml_diff>

<commit_message>
Atualização de dados — 07/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -105,12 +105,12 @@
     <t>Marialva</t>
   </si>
   <si>
+    <t>Sarandi</t>
+  </si>
+  <si>
     <t>Paranacity</t>
   </si>
   <si>
-    <t>Sarandi</t>
-  </si>
-  <si>
     <t>Munhoz De Melo</t>
   </si>
   <si>
@@ -513,19 +513,19 @@
     <t>100,0% (64)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 29,0% (972)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 77,0% (969)</t>
+    <t xml:space="preserve"> 29,0% (974)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 76,9% (971)</t>
   </si>
   <si>
     <t xml:space="preserve"> 98,0% (350)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 99,7% (971)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,8% (934)</t>
+    <t xml:space="preserve"> 99,7% (973)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,8% (938)</t>
   </si>
   <si>
     <t xml:space="preserve"> 25,0% (8)</t>
@@ -534,13 +534,13 @@
     <t xml:space="preserve"> 87,5% (8)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 26,3% (114)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,1% (114)</t>
-  </si>
-  <si>
-    <t>100,0% (112)</t>
+    <t xml:space="preserve"> 25,9% (116)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,2% (116)</t>
+  </si>
+  <si>
+    <t>100,0% (114)</t>
   </si>
   <si>
     <t>100,0% (106)</t>
@@ -594,13 +594,13 @@
     <t xml:space="preserve"> 83,3% (12)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 24,6% (130)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 68,5% (130)</t>
-  </si>
-  <si>
-    <t>100,0% (130)</t>
+    <t xml:space="preserve"> 24,4% (131)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 67,9% (131)</t>
+  </si>
+  <si>
+    <t>100,0% (131)</t>
   </si>
   <si>
     <t xml:space="preserve"> 93,8% (128)</t>
@@ -735,10 +735,10 @@
     <t>inconsistentes</t>
   </si>
   <si>
+    <t>Antiviral informado sem data de início</t>
+  </si>
+  <si>
     <t>Classificação final informada sem data de encerramento</t>
-  </si>
-  <si>
-    <t>Antiviral informado sem data de início</t>
   </si>
   <si>
     <t>Internação mais de 30 dias após o início dos sintomas</t>
@@ -1209,7 +1209,7 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C2">
         <v>106</v>
@@ -1221,7 +1221,7 @@
         <v>6</v>
       </c>
       <c r="F2">
-        <v>420</v>
+        <v>427.4</v>
       </c>
       <c r="G2">
         <v>40.5</v>
@@ -1230,7 +1230,7 @@
         <v>10.4</v>
       </c>
       <c r="I2">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1412,28 +1412,28 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>977</v>
+        <v>979</v>
       </c>
       <c r="C9">
-        <v>883</v>
+        <v>909</v>
       </c>
       <c r="D9">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E9">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="F9">
-        <v>227.4</v>
+        <v>227.9</v>
       </c>
       <c r="G9">
-        <v>19.1</v>
+        <v>19.6</v>
       </c>
       <c r="H9">
-        <v>9.300000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I9">
-        <v>29.6</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1615,28 +1615,28 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>10</v>
+        <v>135</v>
       </c>
       <c r="C16">
-        <v>10</v>
+        <v>130</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="F16">
-        <v>104.7</v>
+        <v>105.4</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="I16">
-        <v>20</v>
+        <v>39.3</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1644,28 +1644,28 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>134</v>
+        <v>10</v>
       </c>
       <c r="C17">
-        <v>130</v>
+        <v>10</v>
       </c>
       <c r="D17">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="F17">
-        <v>104.6</v>
+        <v>104.7</v>
       </c>
       <c r="G17">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>6.9</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>38.8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -2042,13 +2042,13 @@
         <v>96</v>
       </c>
       <c r="B2">
-        <v>1521</v>
+        <v>1526</v>
       </c>
       <c r="C2">
         <v>433</v>
       </c>
       <c r="D2">
-        <v>28.5</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2056,10 +2056,10 @@
         <v>97</v>
       </c>
       <c r="B3">
-        <v>1518</v>
+        <v>1523</v>
       </c>
       <c r="C3">
-        <v>1166</v>
+        <v>1169</v>
       </c>
       <c r="D3">
         <v>76.8</v>
@@ -2084,10 +2084,10 @@
         <v>99</v>
       </c>
       <c r="B5">
-        <v>1516</v>
+        <v>1521</v>
       </c>
       <c r="C5">
-        <v>1509</v>
+        <v>1514</v>
       </c>
       <c r="D5">
         <v>99.5</v>
@@ -2098,13 +2098,13 @@
         <v>100</v>
       </c>
       <c r="B6">
-        <v>1453</v>
+        <v>1457</v>
       </c>
       <c r="C6">
-        <v>1368</v>
+        <v>1371</v>
       </c>
       <c r="D6">
-        <v>94.2</v>
+        <v>94.09999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2174,7 +2174,7 @@
         <v>105</v>
       </c>
       <c r="B3">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -2186,7 +2186,7 @@
         <v>42663</v>
       </c>
       <c r="F3">
-        <v>625.8</v>
+        <v>628.2</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2200,25 +2200,25 @@
         <v>106</v>
       </c>
       <c r="B4">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4">
         <v>58201</v>
       </c>
       <c r="F4">
-        <v>159.8</v>
+        <v>161.5</v>
       </c>
       <c r="G4">
         <v>1.7</v>
       </c>
       <c r="H4">
-        <v>37.8</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2232,7 +2232,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E5">
         <v>57229</v>
@@ -2244,7 +2244,7 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>10.5</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2333,7 +2333,7 @@
         <v>50</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9">
         <v>18</v>
@@ -2345,7 +2345,7 @@
         <v>38.5</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="H9">
         <v>13.9</v>
@@ -2382,25 +2382,25 @@
         <v>113</v>
       </c>
       <c r="B11">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C11">
         <v>15</v>
       </c>
       <c r="D11">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E11">
         <v>91102</v>
       </c>
       <c r="F11">
-        <v>162.5</v>
+        <v>163.6</v>
       </c>
       <c r="G11">
         <v>16.5</v>
       </c>
       <c r="H11">
-        <v>67</v>
+        <v>69.2</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2408,25 +2408,25 @@
         <v>114</v>
       </c>
       <c r="B12">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C12">
         <v>27</v>
       </c>
       <c r="D12">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E12">
         <v>53206</v>
       </c>
       <c r="F12">
-        <v>381.5</v>
+        <v>383.4</v>
       </c>
       <c r="G12">
         <v>50.7</v>
       </c>
       <c r="H12">
-        <v>107.1</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2434,25 +2434,25 @@
         <v>115</v>
       </c>
       <c r="B13">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C13">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D13">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E13">
         <v>23417</v>
       </c>
       <c r="F13">
-        <v>1362.3</v>
+        <v>1366.5</v>
       </c>
       <c r="G13">
-        <v>226.3</v>
+        <v>230.6</v>
       </c>
       <c r="H13">
-        <v>328.8</v>
+        <v>341.6</v>
       </c>
     </row>
   </sheetData>
@@ -2887,7 +2887,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B22" t="s">
         <v>174</v>
@@ -3007,7 +3007,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B28" t="s">
         <v>186</v>
@@ -3086,7 +3086,7 @@
         <v>198</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2">
         <v>9</v>
@@ -3138,10 +3138,10 @@
         <v>200</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -3150,7 +3150,7 @@
         <v>5</v>
       </c>
       <c r="F4">
-        <v>38.5</v>
+        <v>38.4</v>
       </c>
       <c r="G4">
         <v>98.40000000000001</v>
@@ -3167,7 +3167,7 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -3176,10 +3176,10 @@
         <v>5</v>
       </c>
       <c r="F5">
-        <v>40.9</v>
+        <v>41</v>
       </c>
       <c r="G5">
-        <v>97.59999999999999</v>
+        <v>97.7</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -3375,7 +3375,7 @@
         <v>16</v>
       </c>
       <c r="C13">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -3384,7 +3384,7 @@
         <v>2</v>
       </c>
       <c r="F13">
-        <v>86.90000000000001</v>
+        <v>86.3</v>
       </c>
       <c r="G13">
         <v>99.3</v>
@@ -3774,16 +3774,16 @@
         <v>46266</v>
       </c>
       <c r="B10">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10">
         <v>4</v>
       </c>
       <c r="E10">
-        <v>73.90000000000001</v>
+        <v>65.5</v>
       </c>
       <c r="F10">
         <v>100</v>
@@ -3830,7 +3830,7 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>1528</v>
+        <v>1533</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -3847,10 +3847,10 @@
         <v>227</v>
       </c>
       <c r="B3">
-        <v>886</v>
+        <v>888</v>
       </c>
       <c r="C3">
-        <v>1535</v>
+        <v>1540</v>
       </c>
       <c r="D3">
         <v>57.7</v>
@@ -3891,10 +3891,10 @@
         <v>233</v>
       </c>
       <c r="B2">
-        <v>1504</v>
+        <v>387</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -3905,13 +3905,13 @@
         <v>234</v>
       </c>
       <c r="B3">
-        <v>387</v>
+        <v>1506</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -3919,7 +3919,7 @@
         <v>235</v>
       </c>
       <c r="B4">
-        <v>1545</v>
+        <v>1550</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -3933,7 +3933,7 @@
         <v>236</v>
       </c>
       <c r="B5">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -3947,7 +3947,7 @@
         <v>237</v>
       </c>
       <c r="B6">
-        <v>1428</v>
+        <v>1453</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -3961,7 +3961,7 @@
         <v>238</v>
       </c>
       <c r="B7">
-        <v>1417</v>
+        <v>1442</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -4017,7 +4017,7 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -4028,16 +4028,16 @@
         <v>16</v>
       </c>
       <c r="C3">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>5.3</v>
+        <v>6.5</v>
       </c>
       <c r="F3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -4057,7 +4057,7 @@
         <v>5</v>
       </c>
       <c r="F4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -4085,10 +4085,10 @@
         <v>200</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D6">
         <v>8</v>
@@ -4097,7 +4097,7 @@
         <v>2.4</v>
       </c>
       <c r="F6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -4137,7 +4137,7 @@
         <v>1.6</v>
       </c>
       <c r="F8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -4148,7 +4148,7 @@
         <v>9</v>
       </c>
       <c r="C9">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -4162,42 +4162,42 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C10">
-        <v>284</v>
+        <v>102</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C11">
-        <v>102</v>
+        <v>285</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="F11" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -4325,7 +4325,7 @@
         <v>198</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C18">
         <v>9</v>
@@ -4404,25 +4404,25 @@
         <v>411690</v>
       </c>
       <c r="B2">
-        <v>47.96421738600731</v>
+        <v>48.12545502286392</v>
       </c>
       <c r="C2">
         <v>27142</v>
       </c>
       <c r="D2">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>
       </c>
       <c r="F2">
-        <v>2.376771814758254</v>
+        <v>2.410366820321793</v>
       </c>
       <c r="G2">
-        <v>1.960543657059412</v>
+        <v>1.99173274218134</v>
       </c>
       <c r="H2">
-        <v>2.855228982136748</v>
+        <v>2.891005402695876</v>
       </c>
       <c r="I2" t="s">
         <v>249</v>
@@ -4433,7 +4433,7 @@
         <v>412360</v>
       </c>
       <c r="B3">
-        <v>3.144135478454948</v>
+        <v>3.155116935819763</v>
       </c>
       <c r="C3">
         <v>1745</v>
@@ -4445,13 +4445,13 @@
         <v>10</v>
       </c>
       <c r="F3">
-        <v>1.590262262635399</v>
+        <v>1.584727318102046</v>
       </c>
       <c r="G3">
-        <v>0.5163538280214993</v>
+        <v>0.5145566465975075</v>
       </c>
       <c r="H3">
-        <v>3.711141634728976</v>
+        <v>3.698224920557817</v>
       </c>
       <c r="I3" t="s">
         <v>250</v>
@@ -4462,7 +4462,7 @@
         <v>412830</v>
       </c>
       <c r="B4">
-        <v>3.846634840978511</v>
+        <v>3.859567657577198</v>
       </c>
       <c r="C4">
         <v>2106</v>
@@ -4474,13 +4474,13 @@
         <v>11</v>
       </c>
       <c r="F4">
-        <v>1.559804932893946</v>
+        <v>1.55457826687418</v>
       </c>
       <c r="G4">
-        <v>0.5724209197176435</v>
+        <v>0.5705028254053373</v>
       </c>
       <c r="H4">
-        <v>3.395038666887498</v>
+        <v>3.383662415369246</v>
       </c>
       <c r="I4" t="s">
         <v>250</v>
@@ -4491,7 +4491,7 @@
         <v>410220</v>
       </c>
       <c r="B5">
-        <v>7.229864258194739</v>
+        <v>7.255090852582689</v>
       </c>
       <c r="C5">
         <v>4046</v>
@@ -4503,13 +4503,13 @@
         <v>12</v>
       </c>
       <c r="F5">
-        <v>1.521467016138232</v>
+        <v>1.516176740375923</v>
       </c>
       <c r="G5">
-        <v>0.7595108526433044</v>
+        <v>0.7568699660435098</v>
       </c>
       <c r="H5">
-        <v>2.722324764395571</v>
+        <v>2.712858999731958</v>
       </c>
       <c r="I5" t="s">
         <v>250</v>
@@ -4520,7 +4520,7 @@
         <v>411090</v>
       </c>
       <c r="B6">
-        <v>7.99422861813144</v>
+        <v>8.021518270582693</v>
       </c>
       <c r="C6">
         <v>4530</v>
@@ -4532,13 +4532,13 @@
         <v>14</v>
       </c>
       <c r="F6">
-        <v>1.375992672395091</v>
+        <v>1.371311468595701</v>
       </c>
       <c r="G6">
-        <v>0.6868905843876572</v>
+        <v>0.6845537443172779</v>
       </c>
       <c r="H6">
-        <v>2.462030979281952</v>
+        <v>2.453655012603023</v>
       </c>
       <c r="I6" t="s">
         <v>250</v>
@@ -4549,25 +4549,25 @@
         <v>411520</v>
       </c>
       <c r="B7">
-        <v>714.2098872198766</v>
+        <v>716.5637350054662</v>
       </c>
       <c r="C7">
         <v>429660</v>
       </c>
       <c r="D7">
-        <v>977</v>
+        <v>979</v>
       </c>
       <c r="E7" t="s">
         <v>16</v>
       </c>
       <c r="F7">
-        <v>1.36794521818097</v>
+        <v>1.366242739025206</v>
       </c>
       <c r="G7">
-        <v>1.283502241155937</v>
+        <v>1.281989679080585</v>
       </c>
       <c r="H7">
-        <v>1.456484349211052</v>
+        <v>1.454578453179668</v>
       </c>
       <c r="I7" t="s">
         <v>249</v>
@@ -4578,7 +4578,7 @@
         <v>411740</v>
       </c>
       <c r="B8">
-        <v>5.9266473822138</v>
+        <v>5.947173844366641</v>
       </c>
       <c r="C8">
         <v>3193</v>
@@ -4590,13 +4590,13 @@
         <v>13</v>
       </c>
       <c r="F8">
-        <v>1.34983566324672</v>
+        <v>1.345176752749184</v>
       </c>
       <c r="G8">
-        <v>0.5827632308805218</v>
+        <v>0.5807518440073994</v>
       </c>
       <c r="H8">
-        <v>2.659714371990398</v>
+        <v>2.650534461023824</v>
       </c>
       <c r="I8" t="s">
         <v>250</v>
@@ -4607,7 +4607,7 @@
         <v>411640</v>
       </c>
       <c r="B9">
-        <v>6.106002803986375</v>
+        <v>6.127295797859569</v>
       </c>
       <c r="C9">
         <v>3669</v>
@@ -4619,13 +4619,13 @@
         <v>17</v>
       </c>
       <c r="F9">
-        <v>1.310186099943667</v>
+        <v>1.305633066187961</v>
       </c>
       <c r="G9">
-        <v>0.5656453636892579</v>
+        <v>0.5636796868783484</v>
       </c>
       <c r="H9">
-        <v>2.581588925884891</v>
+        <v>2.572617634307752</v>
       </c>
       <c r="I9" t="s">
         <v>250</v>
@@ -4636,7 +4636,7 @@
         <v>412530</v>
       </c>
       <c r="B10">
-        <v>9.943131633395389</v>
+        <v>9.977716427528796</v>
       </c>
       <c r="C10">
         <v>5170</v>
@@ -4648,13 +4648,13 @@
         <v>15</v>
       </c>
       <c r="F10">
-        <v>1.20686323408375</v>
+        <v>1.202680000695517</v>
       </c>
       <c r="G10">
-        <v>0.6236038440743078</v>
+        <v>0.6214423063392198</v>
       </c>
       <c r="H10">
-        <v>2.108147193563702</v>
+        <v>2.100839926693383</v>
       </c>
       <c r="I10" t="s">
         <v>250</v>
@@ -4665,7 +4665,7 @@
         <v>412450</v>
       </c>
       <c r="B11">
-        <v>11.71986363210249</v>
+        <v>11.75741838428178</v>
       </c>
       <c r="C11">
         <v>6463</v>
@@ -4677,13 +4677,13 @@
         <v>18</v>
       </c>
       <c r="F11">
-        <v>1.194553148353354</v>
+        <v>1.190737587319022</v>
       </c>
       <c r="G11">
-        <v>0.6530733220594237</v>
+        <v>0.650987319336442</v>
       </c>
       <c r="H11">
-        <v>2.00425720462258</v>
+        <v>1.997855341546602</v>
       </c>
       <c r="I11" t="s">
         <v>250</v>
@@ -4694,7 +4694,7 @@
         <v>410590</v>
       </c>
       <c r="B12">
-        <v>40.96748889977696</v>
+        <v>41.10532485985631</v>
       </c>
       <c r="C12">
         <v>23313</v>
@@ -4706,13 +4706,13 @@
         <v>19</v>
       </c>
       <c r="F12">
-        <v>1.049612782106206</v>
+        <v>1.04609318005887</v>
       </c>
       <c r="G12">
-        <v>0.7596099748290065</v>
+        <v>0.7570628213756917</v>
       </c>
       <c r="H12">
-        <v>1.413821529361517</v>
+        <v>1.409080648501317</v>
       </c>
       <c r="I12" t="s">
         <v>250</v>
@@ -4723,7 +4723,7 @@
         <v>411110</v>
       </c>
       <c r="B13">
-        <v>10.79983434460729</v>
+        <v>10.83622974078015</v>
       </c>
       <c r="C13">
         <v>6228</v>
@@ -4735,13 +4735,13 @@
         <v>20</v>
       </c>
       <c r="F13">
-        <v>0.9259401284236665</v>
+        <v>0.9228301945617525</v>
       </c>
       <c r="G13">
-        <v>0.4440242825138264</v>
+        <v>0.4425329483451123</v>
       </c>
       <c r="H13">
-        <v>1.702836863530289</v>
+        <v>1.697117584431517</v>
       </c>
       <c r="I13" t="s">
         <v>250</v>
@@ -4752,7 +4752,7 @@
         <v>411480</v>
       </c>
       <c r="B14">
-        <v>76.80636875810966</v>
+        <v>77.05655825943418</v>
       </c>
       <c r="C14">
         <v>44749</v>
@@ -4764,13 +4764,13 @@
         <v>22</v>
       </c>
       <c r="F14">
-        <v>0.8462839872655342</v>
+        <v>0.84353624750742</v>
       </c>
       <c r="G14">
-        <v>0.6531441147442282</v>
+        <v>0.651023467208807</v>
       </c>
       <c r="H14">
-        <v>1.078658412778094</v>
+        <v>1.075156192895864</v>
       </c>
       <c r="I14" t="s">
         <v>250</v>
@@ -4781,7 +4781,7 @@
         <v>410780</v>
       </c>
       <c r="B15">
-        <v>9.716834185999264</v>
+        <v>9.751270044256897</v>
       </c>
       <c r="C15">
         <v>4805</v>
@@ -4793,13 +4793,13 @@
         <v>21</v>
       </c>
       <c r="F15">
-        <v>0.7203992438284189</v>
+        <v>0.7178552094475854</v>
       </c>
       <c r="G15">
-        <v>0.2896378591676504</v>
+        <v>0.288615025401477</v>
       </c>
       <c r="H15">
-        <v>1.484297774936166</v>
+        <v>1.479056091795627</v>
       </c>
       <c r="I15" t="s">
         <v>250</v>
@@ -4810,25 +4810,25 @@
         <v>412625</v>
       </c>
       <c r="B16">
-        <v>205.1262256501793</v>
+        <v>205.7501103536692</v>
       </c>
       <c r="C16">
         <v>128106</v>
       </c>
       <c r="D16">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F16">
-        <v>0.6532563038941817</v>
+        <v>0.6561357355675045</v>
       </c>
       <c r="G16">
-        <v>0.5473373897687619</v>
+        <v>0.5501270519024235</v>
       </c>
       <c r="H16">
-        <v>0.7736923554173603</v>
+        <v>0.7766160524041902</v>
       </c>
       <c r="I16" t="s">
         <v>251</v>
@@ -4839,7 +4839,7 @@
         <v>411810</v>
       </c>
       <c r="B17">
-        <v>16.11760058906637</v>
+        <v>16.17068824093462</v>
       </c>
       <c r="C17">
         <v>9549</v>
@@ -4848,16 +4848,16 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F17">
-        <v>0.6204397450315068</v>
+        <v>0.6184028688825943</v>
       </c>
       <c r="G17">
-        <v>0.2975249739955377</v>
+        <v>0.296548212709546</v>
       </c>
       <c r="H17">
-        <v>1.141010781374814</v>
+        <v>1.137264893615615</v>
       </c>
       <c r="I17" t="s">
         <v>250</v>
@@ -4868,7 +4868,7 @@
         <v>410210</v>
       </c>
       <c r="B18">
-        <v>48.22934288769908</v>
+        <v>48.39199414901175</v>
       </c>
       <c r="C18">
         <v>26203</v>
@@ -4880,13 +4880,13 @@
         <v>26</v>
       </c>
       <c r="F18">
-        <v>0.3939510443723247</v>
+        <v>0.3926269279479158</v>
       </c>
       <c r="G18">
-        <v>0.2371842633436401</v>
+        <v>0.2363870587589816</v>
       </c>
       <c r="H18">
-        <v>0.6152033553654982</v>
+        <v>0.6131355835475842</v>
       </c>
       <c r="I18" t="s">
         <v>251</v>
@@ -4897,7 +4897,7 @@
         <v>411360</v>
       </c>
       <c r="B19">
-        <v>7.730903745984839</v>
+        <v>7.757545209160687</v>
       </c>
       <c r="C19">
         <v>4707</v>
@@ -4909,13 +4909,13 @@
         <v>27</v>
       </c>
       <c r="F19">
-        <v>0.3880529493797016</v>
+        <v>0.3867202728586585</v>
       </c>
       <c r="G19">
-        <v>0.08002584732954644</v>
+        <v>0.07975101739207749</v>
       </c>
       <c r="H19">
-        <v>1.134055390910246</v>
+        <v>1.130160744585706</v>
       </c>
       <c r="I19" t="s">
         <v>250</v>
@@ -4926,7 +4926,7 @@
         <v>411630</v>
       </c>
       <c r="B20">
-        <v>7.99254170451731</v>
+        <v>8.01975541942967</v>
       </c>
       <c r="C20">
         <v>4057</v>
@@ -4938,13 +4938,13 @@
         <v>25</v>
       </c>
       <c r="F20">
-        <v>0.3753499338394979</v>
+        <v>0.3740762458580498</v>
       </c>
       <c r="G20">
-        <v>0.07740618013240189</v>
+        <v>0.07714351504993885</v>
       </c>
       <c r="H20">
-        <v>1.096931788893531</v>
+        <v>1.093209532113863</v>
       </c>
       <c r="I20" t="s">
         <v>250</v>
@@ -4955,7 +4955,7 @@
         <v>410790</v>
       </c>
       <c r="B21">
-        <v>20.09957764655562</v>
+        <v>20.16185207845889</v>
       </c>
       <c r="C21">
         <v>11522</v>
@@ -4967,13 +4967,13 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>0.3482660244455216</v>
+        <v>0.3471903262041519</v>
       </c>
       <c r="G21">
-        <v>0.140021004471313</v>
+        <v>0.1395885179877278</v>
       </c>
       <c r="H21">
-        <v>0.7175611157269233</v>
+        <v>0.7153447662237189</v>
       </c>
       <c r="I21" t="s">
         <v>251</v>
@@ -4984,7 +4984,7 @@
         <v>411750</v>
       </c>
       <c r="B22">
-        <v>80.00855318129641</v>
+        <v>80.26117696248403</v>
       </c>
       <c r="C22">
         <v>48695</v>
@@ -4996,13 +4996,13 @@
         <v>29</v>
       </c>
       <c r="F22">
-        <v>0.299967928999002</v>
+        <v>0.29902377348912</v>
       </c>
       <c r="G22">
-        <v>0.1921951121880954</v>
+        <v>0.1915901739376953</v>
       </c>
       <c r="H22">
-        <v>0.4463285008145998</v>
+        <v>0.4449236722562011</v>
       </c>
       <c r="I22" t="s">
         <v>251</v>
@@ -5013,7 +5013,7 @@
         <v>411410</v>
       </c>
       <c r="B23">
-        <v>59.38056063714926</v>
+        <v>59.56060795845098</v>
       </c>
       <c r="C23">
         <v>34521</v>
@@ -5025,13 +5025,13 @@
         <v>30</v>
       </c>
       <c r="F23">
-        <v>0.2862889776989505</v>
+        <v>0.285423547252222</v>
       </c>
       <c r="G23">
-        <v>0.1667738795886639</v>
+        <v>0.1662697344613345</v>
       </c>
       <c r="H23">
-        <v>0.4583763865455704</v>
+        <v>0.4569907485647919</v>
       </c>
       <c r="I23" t="s">
         <v>251</v>
@@ -5042,7 +5042,7 @@
         <v>412040</v>
       </c>
       <c r="B24">
-        <v>7.100523496262464</v>
+        <v>7.123815275624222</v>
       </c>
       <c r="C24">
         <v>4304</v>
@@ -5054,13 +5054,13 @@
         <v>31</v>
       </c>
       <c r="F24">
-        <v>0.2816693728360662</v>
+        <v>0.2807484364233112</v>
       </c>
       <c r="G24">
-        <v>0.03411146779127732</v>
+        <v>0.0339999381192182</v>
       </c>
       <c r="H24">
-        <v>1.017486622152134</v>
+        <v>1.01415988318014</v>
       </c>
       <c r="I24" t="s">
         <v>250</v>
@@ -5071,7 +5071,7 @@
         <v>412340</v>
       </c>
       <c r="B25">
-        <v>20.73664061668979</v>
+        <v>20.80731228216598</v>
       </c>
       <c r="C25">
         <v>11730</v>
@@ -5083,13 +5083,13 @@
         <v>32</v>
       </c>
       <c r="F25">
-        <v>0.2411190940916328</v>
+        <v>0.240300137384179</v>
       </c>
       <c r="G25">
-        <v>0.07829071353108977</v>
+        <v>0.07802480051736026</v>
       </c>
       <c r="H25">
-        <v>0.562691532105324</v>
+        <v>0.5607803603410919</v>
       </c>
       <c r="I25" t="s">
         <v>251</v>
@@ -5100,7 +5100,7 @@
         <v>411420</v>
       </c>
       <c r="B26">
-        <v>67.84653078949061</v>
+        <v>68.07110150340571</v>
       </c>
       <c r="C26">
         <v>38313</v>
@@ -5112,13 +5112,13 @@
         <v>33</v>
       </c>
       <c r="F26">
-        <v>0.2210872070458685</v>
+        <v>0.2203578268709156</v>
       </c>
       <c r="G26">
-        <v>0.1237408314779118</v>
+        <v>0.1233326029308234</v>
       </c>
       <c r="H26">
-        <v>0.3646497261333528</v>
+        <v>0.3634467244554291</v>
       </c>
       <c r="I26" t="s">
         <v>251</v>
@@ -5129,7 +5129,7 @@
         <v>411000</v>
       </c>
       <c r="B27">
-        <v>9.470975222399511</v>
+        <v>9.501847971583485</v>
       </c>
       <c r="C27">
         <v>5693</v>
@@ -5141,13 +5141,13 @@
         <v>35</v>
       </c>
       <c r="F27">
-        <v>0.2111714953355449</v>
+        <v>0.2104853714752394</v>
       </c>
       <c r="G27">
-        <v>0.02557384776713629</v>
+        <v>0.02549075498453809</v>
       </c>
       <c r="H27">
-        <v>0.7628240490627693</v>
+        <v>0.7603455337667292</v>
       </c>
       <c r="I27" t="s">
         <v>251</v>
@@ -5158,7 +5158,7 @@
         <v>410810</v>
       </c>
       <c r="B28">
-        <v>4.967466015473944</v>
+        <v>4.983881987554243</v>
       </c>
       <c r="C28">
         <v>2711</v>
@@ -5170,13 +5170,13 @@
         <v>34</v>
       </c>
       <c r="F28">
-        <v>0.2013098825205733</v>
+        <v>0.2006468055417848</v>
       </c>
       <c r="G28">
-        <v>0.005096724950995828</v>
+        <v>0.005079937295368057</v>
       </c>
       <c r="H28">
-        <v>1.121626876476438</v>
+        <v>1.117932448009888</v>
       </c>
       <c r="I28" t="s">
         <v>250</v>
@@ -5187,7 +5187,7 @@
         <v>410730</v>
       </c>
       <c r="B29">
-        <v>12.78288564558409</v>
+        <v>12.82663853797248</v>
       </c>
       <c r="C29">
         <v>6517</v>
@@ -5199,13 +5199,13 @@
         <v>36</v>
       </c>
       <c r="F29">
-        <v>0.1564591951654445</v>
+        <v>0.1559254978675139</v>
       </c>
       <c r="G29">
-        <v>0.01894793439129586</v>
+        <v>0.01888330117254954</v>
       </c>
       <c r="H29">
-        <v>0.5651844089069015</v>
+        <v>0.5632565107635732</v>
       </c>
       <c r="I29" t="s">
         <v>251</v>
@@ -5216,7 +5216,7 @@
         <v>410115</v>
       </c>
       <c r="B30">
-        <v>6.125098715851931</v>
+        <v>6.145522885780435</v>
       </c>
       <c r="C30">
         <v>3357</v>
@@ -5234,7 +5234,7 @@
         <v>0</v>
       </c>
       <c r="H30">
-        <v>0.6022563268355186</v>
+        <v>0.6002547745203743</v>
       </c>
       <c r="I30" t="s">
         <v>251</v>
@@ -5245,7 +5245,7 @@
         <v>411160</v>
       </c>
       <c r="B31">
-        <v>4.909434013964724</v>
+        <v>4.926678081056779</v>
       </c>
       <c r="C31">
         <v>2685</v>
@@ -5263,7 +5263,7 @@
         <v>0</v>
       </c>
       <c r="H31">
-        <v>0.7513858916569688</v>
+        <v>0.7487559352208915</v>
       </c>
       <c r="I31" t="s">
         <v>251</v>
@@ -5295,7 +5295,7 @@
         <v>254</v>
       </c>
       <c r="B2">
-        <v>1489</v>
+        <v>1494</v>
       </c>
       <c r="C2">
         <v>97</v>
@@ -5360,10 +5360,10 @@
         <v>40</v>
       </c>
       <c r="B2">
-        <v>60.8</v>
+        <v>60.9</v>
       </c>
       <c r="C2">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5371,10 +5371,10 @@
         <v>41</v>
       </c>
       <c r="B3">
-        <v>61.2</v>
+        <v>61.3</v>
       </c>
       <c r="C3">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5385,7 +5385,7 @@
         <v>61.4</v>
       </c>
       <c r="C4">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5396,7 +5396,7 @@
         <v>61.4</v>
       </c>
       <c r="C5">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -5404,10 +5404,10 @@
         <v>44</v>
       </c>
       <c r="B6">
-        <v>91.5</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="C6">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5415,10 +5415,10 @@
         <v>45</v>
       </c>
       <c r="B7">
-        <v>96</v>
+        <v>95.8</v>
       </c>
       <c r="C7">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5429,7 +5429,7 @@
         <v>98.7</v>
       </c>
       <c r="C8">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -5440,7 +5440,7 @@
         <v>98.8</v>
       </c>
       <c r="C9">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -5451,7 +5451,7 @@
         <v>99.09999999999999</v>
       </c>
       <c r="C10">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -5462,7 +5462,7 @@
         <v>99.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -5473,7 +5473,7 @@
         <v>100</v>
       </c>
       <c r="C12">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -5484,7 +5484,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -5495,7 +5495,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -5506,7 +5506,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1535</v>
+        <v>1540</v>
       </c>
     </row>
   </sheetData>
@@ -5595,13 +5595,13 @@
         <v>261</v>
       </c>
       <c r="C5">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D5">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E5">
-        <v>52.6</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -5612,13 +5612,13 @@
         <v>262</v>
       </c>
       <c r="C6">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E6">
-        <v>47.4</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -5632,7 +5632,7 @@
         <v>0</v>
       </c>
       <c r="D7">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -5675,7 +5675,7 @@
         <v>262</v>
       </c>
       <c r="B3">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C3">
         <v>40.7</v>
@@ -5686,7 +5686,7 @@
         <v>261</v>
       </c>
       <c r="B4">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="C4">
         <v>59.2</v>
@@ -5718,10 +5718,10 @@
         <v>42</v>
       </c>
       <c r="B2">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="C2">
-        <v>30.2</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5729,10 +5729,10 @@
         <v>41</v>
       </c>
       <c r="B3">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C3">
-        <v>15.2</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5740,10 +5740,10 @@
         <v>57</v>
       </c>
       <c r="B4">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C4">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5751,7 +5751,7 @@
         <v>58</v>
       </c>
       <c r="B5">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C5">
         <v>11.8</v>
@@ -5762,10 +5762,10 @@
         <v>59</v>
       </c>
       <c r="B6">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C6">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5773,10 +5773,10 @@
         <v>60</v>
       </c>
       <c r="B7">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C7">
-        <v>3.8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5795,7 +5795,7 @@
         <v>43</v>
       </c>
       <c r="B9">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -5820,7 +5820,7 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -5858,13 +5858,13 @@
         <v>147</v>
       </c>
       <c r="C2">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D2">
         <v>4</v>
       </c>
       <c r="E2">
-        <v>3.1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -5872,10 +5872,10 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C3">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -5892,7 +5892,7 @@
         <v>33</v>
       </c>
       <c r="C4">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -5926,7 +5926,7 @@
         <v>21</v>
       </c>
       <c r="C6">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -5960,13 +5960,13 @@
         <v>50</v>
       </c>
       <c r="C8">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -5974,10 +5974,10 @@
         <v>72</v>
       </c>
       <c r="B9">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C9">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -6025,16 +6025,16 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="C12">
-        <v>621</v>
+        <v>638</v>
       </c>
       <c r="D12">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E12">
-        <v>15.3</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -6080,13 +6080,13 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C3">
         <v>59</v>
       </c>
       <c r="D3">
-        <v>22.1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -6097,10 +6097,10 @@
         <v>33</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D4">
-        <v>18.2</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -6164,13 +6164,13 @@
         <v>72</v>
       </c>
       <c r="B9">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C9">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D9">
-        <v>23.7</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -6206,13 +6206,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="C12">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="D12">
-        <v>29.1</v>
+        <v>29.9</v>
       </c>
     </row>
   </sheetData>
@@ -6241,7 +6241,7 @@
         <v>78</v>
       </c>
       <c r="B2">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="C2">
         <v>98.8</v>
@@ -6306,10 +6306,10 @@
         <v>83</v>
       </c>
       <c r="B3">
-        <v>1140</v>
+        <v>1145</v>
       </c>
       <c r="C3">
-        <v>74.3</v>
+        <v>74.40000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6320,7 +6320,7 @@
         <v>376</v>
       </c>
       <c r="C4">
-        <v>24.5</v>
+        <v>24.4</v>
       </c>
     </row>
   </sheetData>
@@ -6418,22 +6418,22 @@
         <v>92</v>
       </c>
       <c r="B2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C2">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D2">
-        <v>73.7</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="E2">
         <v>15</v>
       </c>
       <c r="F2">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G2">
-        <v>52.4</v>
+        <v>52.3</v>
       </c>
       <c r="H2">
         <v>2</v>
@@ -6444,22 +6444,22 @@
         <v>93</v>
       </c>
       <c r="B3">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="C3">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="D3">
-        <v>68.2</v>
+        <v>69.8</v>
       </c>
       <c r="E3">
         <v>91</v>
       </c>
       <c r="F3">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="G3">
-        <v>51.8</v>
+        <v>50.7</v>
       </c>
       <c r="H3">
         <v>2</v>

</xml_diff>

<commit_message>
Atualização de layout/texto — 08/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -19,22 +19,23 @@
     <sheet name="oportunidade" sheetId="10" r:id="rId10"/>
     <sheet name="taxas_faixa_etaria" sheetId="11" r:id="rId11"/>
     <sheet name="oportunidade_mun" sheetId="12" r:id="rId12"/>
-    <sheet name="digitacao_unidade" sheetId="13" r:id="rId13"/>
-    <sheet name="digitacao_mes" sheetId="14" r:id="rId14"/>
-    <sheet name="qualidade" sheetId="15" r:id="rId15"/>
-    <sheet name="consistencia_regras" sheetId="16" r:id="rId16"/>
-    <sheet name="consistencia_unidade" sheetId="17" r:id="rId17"/>
-    <sheet name="representatividade_rip" sheetId="18" r:id="rId18"/>
-    <sheet name="internacao_fora" sheetId="19" r:id="rId19"/>
-    <sheet name="vacina_influenza" sheetId="20" r:id="rId20"/>
-    <sheet name="vacinal" sheetId="21" r:id="rId21"/>
+    <sheet name="metas_opas" sheetId="13" r:id="rId13"/>
+    <sheet name="digitacao_unidade" sheetId="14" r:id="rId14"/>
+    <sheet name="digitacao_mes" sheetId="15" r:id="rId15"/>
+    <sheet name="qualidade" sheetId="16" r:id="rId16"/>
+    <sheet name="consistencia_regras" sheetId="17" r:id="rId17"/>
+    <sheet name="consistencia_unidade" sheetId="18" r:id="rId18"/>
+    <sheet name="representatividade_rip" sheetId="19" r:id="rId19"/>
+    <sheet name="internacao_fora" sheetId="20" r:id="rId20"/>
+    <sheet name="vacina_influenza" sheetId="21" r:id="rId21"/>
+    <sheet name="vacinal" sheetId="22" r:id="rId22"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="277">
   <si>
     <t>municipio</t>
   </si>
@@ -615,6 +616,48 @@
     <t>unidade</t>
   </si>
   <si>
+    <t>meta</t>
+  </si>
+  <si>
+    <t>valor</t>
+  </si>
+  <si>
+    <t>atinge</t>
+  </si>
+  <si>
+    <t>situacao</t>
+  </si>
+  <si>
+    <t>Oportunidade da notificação (internação → notificação, mediana)</t>
+  </si>
+  <si>
+    <t>dias</t>
+  </si>
+  <si>
+    <t>Atinge a meta</t>
+  </si>
+  <si>
+    <t>Cobertura de investigação (casos com desfecho já encerrados)</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Cobertura de amostragem (SRAG com amostra coletada até 10 dias dos sintomas)</t>
+  </si>
+  <si>
+    <t>Oportunidade da coleta (internação → coleta, mediana)</t>
+  </si>
+  <si>
+    <t>Cobertura de amostragem em UTI</t>
+  </si>
+  <si>
+    <t>Abaixo da meta</t>
+  </si>
+  <si>
+    <t>Cobertura de amostragem nos óbitos</t>
+  </si>
+  <si>
     <t>mediana</t>
   </si>
   <si>
@@ -717,7 +760,7 @@
     <t>Aceitável</t>
   </si>
   <si>
-    <t>Valor preditivo positivo (vírus respiratório confirmado)</t>
+    <t>Proporção com vírus respiratório confirmado ("VPP" de Ribeiro &amp; Sanchez, 2020)</t>
   </si>
   <si>
     <t>&gt; 20%</t>
@@ -778,9 +821,6 @@
   </si>
   <si>
     <t>ls</t>
-  </si>
-  <si>
-    <t>situacao</t>
   </si>
   <si>
     <t>acima</t>
@@ -3052,6 +3092,177 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>1550</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C3">
+        <v>90</v>
+      </c>
+      <c r="D3">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="E3">
+        <v>1361</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C4">
+        <v>90</v>
+      </c>
+      <c r="D4">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="E4">
+        <v>1564</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>203</v>
+      </c>
+      <c r="B5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>1557</v>
+      </c>
+      <c r="F5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>204</v>
+      </c>
+      <c r="B6" t="s">
+        <v>201</v>
+      </c>
+      <c r="C6">
+        <v>100</v>
+      </c>
+      <c r="D6">
+        <v>99.8</v>
+      </c>
+      <c r="E6">
+        <v>485</v>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B7" t="s">
+        <v>201</v>
+      </c>
+      <c r="C7">
+        <v>100</v>
+      </c>
+      <c r="D7">
+        <v>100</v>
+      </c>
+      <c r="E7">
+        <v>116</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>199</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -3066,24 +3277,24 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>198</v>
+        <v>212</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
@@ -3109,7 +3320,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>199</v>
+        <v>213</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
@@ -3135,7 +3346,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>200</v>
+        <v>214</v>
       </c>
       <c r="B4" t="s">
         <v>23</v>
@@ -3161,7 +3372,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>201</v>
+        <v>215</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
@@ -3187,7 +3398,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>202</v>
+        <v>216</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
@@ -3213,7 +3424,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
@@ -3239,7 +3450,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>204</v>
+        <v>218</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -3265,7 +3476,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>205</v>
+        <v>219</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
@@ -3291,7 +3502,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="B10" t="s">
         <v>16</v>
@@ -3317,7 +3528,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
@@ -3343,7 +3554,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>208</v>
+        <v>222</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
@@ -3369,7 +3580,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
@@ -3395,7 +3606,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
@@ -3421,7 +3632,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -3447,7 +3658,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
@@ -3473,7 +3684,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -3499,7 +3710,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
@@ -3525,10 +3736,10 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>215</v>
+        <v>229</v>
       </c>
       <c r="B19" t="s">
-        <v>216</v>
+        <v>230</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -3554,7 +3765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3564,25 +3775,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>217</v>
+        <v>231</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>196</v>
+        <v>210</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>197</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3790,76 +4001,6 @@
       </c>
       <c r="G10">
         <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>224</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>1533</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2" t="s">
-        <v>225</v>
-      </c>
-      <c r="F2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>227</v>
-      </c>
-      <c r="B3">
-        <v>888</v>
-      </c>
-      <c r="C3">
-        <v>1540</v>
-      </c>
-      <c r="D3">
-        <v>57.7</v>
-      </c>
-      <c r="E3" t="s">
-        <v>228</v>
-      </c>
-      <c r="F3" t="s">
-        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3869,105 +4010,67 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+        <v>235</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="B2">
-        <v>387</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>1533</v>
       </c>
       <c r="D2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>239</v>
+      </c>
+      <c r="F2" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="B3">
-        <v>1506</v>
+        <v>888</v>
       </c>
       <c r="C3">
-        <v>14</v>
+        <v>1540</v>
       </c>
       <c r="D3">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>235</v>
-      </c>
-      <c r="B4">
-        <v>1550</v>
-      </c>
-      <c r="C4">
-        <v>7</v>
-      </c>
-      <c r="D4">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
-        <v>236</v>
-      </c>
-      <c r="B5">
-        <v>485</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>237</v>
-      </c>
-      <c r="B6">
-        <v>1453</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>238</v>
-      </c>
-      <c r="B7">
-        <v>1442</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-      <c r="D7">
-        <v>0.1</v>
+        <v>57.7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>242</v>
+      </c>
+      <c r="F3" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -3977,387 +4080,105 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
+    <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>244</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>245</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>203</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
+        <v>247</v>
+      </c>
+      <c r="B2">
+        <v>387</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B3">
+        <v>1506</v>
+      </c>
+      <c r="C3">
+        <v>14</v>
+      </c>
+      <c r="D3">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B4">
+        <v>1550</v>
+      </c>
+      <c r="C4">
+        <v>7</v>
+      </c>
+      <c r="D4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>250</v>
+      </c>
+      <c r="B5">
+        <v>485</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>251</v>
+      </c>
+      <c r="B6">
+        <v>1453</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>252</v>
+      </c>
+      <c r="B7">
+        <v>1442</v>
+      </c>
+      <c r="C7">
         <v>2</v>
       </c>
-      <c r="E2">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3">
-        <v>77</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="E3">
-        <v>6.5</v>
-      </c>
-      <c r="F3" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>208</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4">
-        <v>100</v>
-      </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
-      <c r="E4">
-        <v>5</v>
-      </c>
-      <c r="F4" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5">
-        <v>78</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5">
-        <v>2.6</v>
-      </c>
-      <c r="F5" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>200</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6">
-        <v>332</v>
-      </c>
-      <c r="D6">
-        <v>8</v>
-      </c>
-      <c r="E6">
-        <v>2.4</v>
-      </c>
-      <c r="F6" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>212</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7">
-        <v>43</v>
-      </c>
       <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>2.3</v>
-      </c>
-      <c r="F7" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>211</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8">
-        <v>63</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>1.6</v>
-      </c>
-      <c r="F8" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>204</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9">
-        <v>133</v>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9">
-        <v>1.5</v>
-      </c>
-      <c r="F9" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>207</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10">
-        <v>102</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>201</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11">
-        <v>285</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11">
-        <v>0.4</v>
-      </c>
-      <c r="F11" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>209</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12">
-        <v>155</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>199</v>
-      </c>
-      <c r="B13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13">
-        <v>101</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
-        <v>206</v>
-      </c>
-      <c r="B14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14">
-        <v>18</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
-        <v>202</v>
-      </c>
-      <c r="B15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15">
-        <v>15</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
-        <v>213</v>
-      </c>
-      <c r="B16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16">
-        <v>14</v>
-      </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
-        <v>214</v>
-      </c>
-      <c r="B17" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17">
-        <v>13</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
-        <v>198</v>
-      </c>
-      <c r="B18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C18">
-        <v>9</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-      <c r="F18" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" t="s">
-        <v>215</v>
-      </c>
-      <c r="B19" t="s">
-        <v>216</v>
-      </c>
-      <c r="C19">
-        <v>6</v>
-      </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
-      <c r="E19">
-        <v>16.7</v>
-      </c>
-      <c r="F19" t="s">
-        <v>235</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -4367,906 +4188,387 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1">
+    <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>242</v>
+        <v>192</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>243</v>
+        <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>102</v>
+        <v>253</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="I1" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2">
-        <v>411690</v>
-      </c>
-      <c r="B2">
-        <v>48.12545502286392</v>
-      </c>
-      <c r="C2">
-        <v>27142</v>
-      </c>
-      <c r="D2">
-        <v>116</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2">
-        <v>2.410366820321793</v>
-      </c>
-      <c r="G2">
-        <v>1.99173274218134</v>
-      </c>
-      <c r="H2">
-        <v>2.891005402695876</v>
-      </c>
-      <c r="I2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3">
-        <v>412360</v>
-      </c>
-      <c r="B3">
-        <v>3.155116935819763</v>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
       </c>
       <c r="C3">
-        <v>1745</v>
+        <v>77</v>
       </c>
       <c r="D3">
         <v>5</v>
       </c>
-      <c r="E3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3">
-        <v>1.584727318102046</v>
-      </c>
-      <c r="G3">
-        <v>0.5145566465975075</v>
-      </c>
-      <c r="H3">
-        <v>3.698224920557817</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="E3">
+        <v>6.5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>222</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>100</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>78</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>2.6</v>
+      </c>
+      <c r="F5" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>214</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>332</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>2.4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>226</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7">
+        <v>43</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>2.3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>225</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8">
+        <v>63</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1.6</v>
+      </c>
+      <c r="F8" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>218</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>133</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>1.5</v>
+      </c>
+      <c r="F9" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
-      <c r="A4">
-        <v>412830</v>
-      </c>
-      <c r="B4">
-        <v>3.859567657577198</v>
-      </c>
-      <c r="C4">
-        <v>2106</v>
-      </c>
-      <c r="D4">
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10">
+        <v>102</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>215</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11">
+        <v>285</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>0.4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12">
+        <v>155</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>213</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13">
+        <v>101</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>220</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14">
+        <v>18</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>216</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15">
+        <v>15</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>227</v>
+      </c>
+      <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16">
+        <v>14</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>228</v>
+      </c>
+      <c r="B17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17">
+        <v>13</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>212</v>
+      </c>
+      <c r="B18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18">
+        <v>9</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>229</v>
+      </c>
+      <c r="B19" t="s">
+        <v>230</v>
+      </c>
+      <c r="C19">
         <v>6</v>
       </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4">
-        <v>1.55457826687418</v>
-      </c>
-      <c r="G4">
-        <v>0.5705028254053373</v>
-      </c>
-      <c r="H4">
-        <v>3.383662415369246</v>
-      </c>
-      <c r="I4" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5">
-        <v>410220</v>
-      </c>
-      <c r="B5">
-        <v>7.255090852582689</v>
-      </c>
-      <c r="C5">
-        <v>4046</v>
-      </c>
-      <c r="D5">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5">
-        <v>1.516176740375923</v>
-      </c>
-      <c r="G5">
-        <v>0.7568699660435098</v>
-      </c>
-      <c r="H5">
-        <v>2.712858999731958</v>
-      </c>
-      <c r="I5" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6">
-        <v>411090</v>
-      </c>
-      <c r="B6">
-        <v>8.021518270582693</v>
-      </c>
-      <c r="C6">
-        <v>4530</v>
-      </c>
-      <c r="D6">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6">
-        <v>1.371311468595701</v>
-      </c>
-      <c r="G6">
-        <v>0.6845537443172779</v>
-      </c>
-      <c r="H6">
-        <v>2.453655012603023</v>
-      </c>
-      <c r="I6" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7">
-        <v>411520</v>
-      </c>
-      <c r="B7">
-        <v>716.5637350054662</v>
-      </c>
-      <c r="C7">
-        <v>429660</v>
-      </c>
-      <c r="D7">
-        <v>979</v>
-      </c>
-      <c r="E7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7">
-        <v>1.366242739025206</v>
-      </c>
-      <c r="G7">
-        <v>1.281989679080585</v>
-      </c>
-      <c r="H7">
-        <v>1.454578453179668</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>16.7</v>
+      </c>
+      <c r="F19" t="s">
         <v>249</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8">
-        <v>411740</v>
-      </c>
-      <c r="B8">
-        <v>5.947173844366641</v>
-      </c>
-      <c r="C8">
-        <v>3193</v>
-      </c>
-      <c r="D8">
-        <v>8</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8">
-        <v>1.345176752749184</v>
-      </c>
-      <c r="G8">
-        <v>0.5807518440073994</v>
-      </c>
-      <c r="H8">
-        <v>2.650534461023824</v>
-      </c>
-      <c r="I8" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9">
-        <v>411640</v>
-      </c>
-      <c r="B9">
-        <v>6.127295797859569</v>
-      </c>
-      <c r="C9">
-        <v>3669</v>
-      </c>
-      <c r="D9">
-        <v>8</v>
-      </c>
-      <c r="E9" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9">
-        <v>1.305633066187961</v>
-      </c>
-      <c r="G9">
-        <v>0.5636796868783484</v>
-      </c>
-      <c r="H9">
-        <v>2.572617634307752</v>
-      </c>
-      <c r="I9" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10">
-        <v>412530</v>
-      </c>
-      <c r="B10">
-        <v>9.977716427528796</v>
-      </c>
-      <c r="C10">
-        <v>5170</v>
-      </c>
-      <c r="D10">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
-      <c r="F10">
-        <v>1.202680000695517</v>
-      </c>
-      <c r="G10">
-        <v>0.6214423063392198</v>
-      </c>
-      <c r="H10">
-        <v>2.100839926693383</v>
-      </c>
-      <c r="I10" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11">
-        <v>412450</v>
-      </c>
-      <c r="B11">
-        <v>11.75741838428178</v>
-      </c>
-      <c r="C11">
-        <v>6463</v>
-      </c>
-      <c r="D11">
-        <v>14</v>
-      </c>
-      <c r="E11" t="s">
-        <v>18</v>
-      </c>
-      <c r="F11">
-        <v>1.190737587319022</v>
-      </c>
-      <c r="G11">
-        <v>0.650987319336442</v>
-      </c>
-      <c r="H11">
-        <v>1.997855341546602</v>
-      </c>
-      <c r="I11" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12">
-        <v>410590</v>
-      </c>
-      <c r="B12">
-        <v>41.10532485985631</v>
-      </c>
-      <c r="C12">
-        <v>23313</v>
-      </c>
-      <c r="D12">
-        <v>43</v>
-      </c>
-      <c r="E12" t="s">
-        <v>19</v>
-      </c>
-      <c r="F12">
-        <v>1.04609318005887</v>
-      </c>
-      <c r="G12">
-        <v>0.7570628213756917</v>
-      </c>
-      <c r="H12">
-        <v>1.409080648501317</v>
-      </c>
-      <c r="I12" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13">
-        <v>411110</v>
-      </c>
-      <c r="B13">
-        <v>10.83622974078015</v>
-      </c>
-      <c r="C13">
-        <v>6228</v>
-      </c>
-      <c r="D13">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13">
-        <v>0.9228301945617525</v>
-      </c>
-      <c r="G13">
-        <v>0.4425329483451123</v>
-      </c>
-      <c r="H13">
-        <v>1.697117584431517</v>
-      </c>
-      <c r="I13" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14">
-        <v>411480</v>
-      </c>
-      <c r="B14">
-        <v>77.05655825943418</v>
-      </c>
-      <c r="C14">
-        <v>44749</v>
-      </c>
-      <c r="D14">
-        <v>65</v>
-      </c>
-      <c r="E14" t="s">
-        <v>22</v>
-      </c>
-      <c r="F14">
-        <v>0.84353624750742</v>
-      </c>
-      <c r="G14">
-        <v>0.651023467208807</v>
-      </c>
-      <c r="H14">
-        <v>1.075156192895864</v>
-      </c>
-      <c r="I14" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15">
-        <v>410780</v>
-      </c>
-      <c r="B15">
-        <v>9.751270044256897</v>
-      </c>
-      <c r="C15">
-        <v>4805</v>
-      </c>
-      <c r="D15">
-        <v>7</v>
-      </c>
-      <c r="E15" t="s">
-        <v>21</v>
-      </c>
-      <c r="F15">
-        <v>0.7178552094475854</v>
-      </c>
-      <c r="G15">
-        <v>0.288615025401477</v>
-      </c>
-      <c r="H15">
-        <v>1.479056091795627</v>
-      </c>
-      <c r="I15" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16">
-        <v>412625</v>
-      </c>
-      <c r="B16">
-        <v>205.7501103536692</v>
-      </c>
-      <c r="C16">
-        <v>128106</v>
-      </c>
-      <c r="D16">
-        <v>135</v>
-      </c>
-      <c r="E16" t="s">
-        <v>23</v>
-      </c>
-      <c r="F16">
-        <v>0.6561357355675045</v>
-      </c>
-      <c r="G16">
-        <v>0.5501270519024235</v>
-      </c>
-      <c r="H16">
-        <v>0.7766160524041902</v>
-      </c>
-      <c r="I16" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17">
-        <v>411810</v>
-      </c>
-      <c r="B17">
-        <v>16.17068824093462</v>
-      </c>
-      <c r="C17">
-        <v>9549</v>
-      </c>
-      <c r="D17">
-        <v>10</v>
-      </c>
-      <c r="E17" t="s">
-        <v>24</v>
-      </c>
-      <c r="F17">
-        <v>0.6184028688825943</v>
-      </c>
-      <c r="G17">
-        <v>0.296548212709546</v>
-      </c>
-      <c r="H17">
-        <v>1.137264893615615</v>
-      </c>
-      <c r="I17" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18">
-        <v>410210</v>
-      </c>
-      <c r="B18">
-        <v>48.39199414901175</v>
-      </c>
-      <c r="C18">
-        <v>26203</v>
-      </c>
-      <c r="D18">
-        <v>19</v>
-      </c>
-      <c r="E18" t="s">
-        <v>26</v>
-      </c>
-      <c r="F18">
-        <v>0.3926269279479158</v>
-      </c>
-      <c r="G18">
-        <v>0.2363870587589816</v>
-      </c>
-      <c r="H18">
-        <v>0.6131355835475842</v>
-      </c>
-      <c r="I18" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19">
-        <v>411360</v>
-      </c>
-      <c r="B19">
-        <v>7.757545209160687</v>
-      </c>
-      <c r="C19">
-        <v>4707</v>
-      </c>
-      <c r="D19">
-        <v>3</v>
-      </c>
-      <c r="E19" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19">
-        <v>0.3867202728586585</v>
-      </c>
-      <c r="G19">
-        <v>0.07975101739207749</v>
-      </c>
-      <c r="H19">
-        <v>1.130160744585706</v>
-      </c>
-      <c r="I19" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20">
-        <v>411630</v>
-      </c>
-      <c r="B20">
-        <v>8.01975541942967</v>
-      </c>
-      <c r="C20">
-        <v>4057</v>
-      </c>
-      <c r="D20">
-        <v>3</v>
-      </c>
-      <c r="E20" t="s">
-        <v>25</v>
-      </c>
-      <c r="F20">
-        <v>0.3740762458580498</v>
-      </c>
-      <c r="G20">
-        <v>0.07714351504993885</v>
-      </c>
-      <c r="H20">
-        <v>1.093209532113863</v>
-      </c>
-      <c r="I20" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21">
-        <v>410790</v>
-      </c>
-      <c r="B21">
-        <v>20.16185207845889</v>
-      </c>
-      <c r="C21">
-        <v>11522</v>
-      </c>
-      <c r="D21">
-        <v>7</v>
-      </c>
-      <c r="E21" t="s">
-        <v>28</v>
-      </c>
-      <c r="F21">
-        <v>0.3471903262041519</v>
-      </c>
-      <c r="G21">
-        <v>0.1395885179877278</v>
-      </c>
-      <c r="H21">
-        <v>0.7153447662237189</v>
-      </c>
-      <c r="I21" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22">
-        <v>411750</v>
-      </c>
-      <c r="B22">
-        <v>80.26117696248403</v>
-      </c>
-      <c r="C22">
-        <v>48695</v>
-      </c>
-      <c r="D22">
-        <v>24</v>
-      </c>
-      <c r="E22" t="s">
-        <v>29</v>
-      </c>
-      <c r="F22">
-        <v>0.29902377348912</v>
-      </c>
-      <c r="G22">
-        <v>0.1915901739376953</v>
-      </c>
-      <c r="H22">
-        <v>0.4449236722562011</v>
-      </c>
-      <c r="I22" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23">
-        <v>411410</v>
-      </c>
-      <c r="B23">
-        <v>59.56060795845098</v>
-      </c>
-      <c r="C23">
-        <v>34521</v>
-      </c>
-      <c r="D23">
-        <v>17</v>
-      </c>
-      <c r="E23" t="s">
-        <v>30</v>
-      </c>
-      <c r="F23">
-        <v>0.285423547252222</v>
-      </c>
-      <c r="G23">
-        <v>0.1662697344613345</v>
-      </c>
-      <c r="H23">
-        <v>0.4569907485647919</v>
-      </c>
-      <c r="I23" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24">
-        <v>412040</v>
-      </c>
-      <c r="B24">
-        <v>7.123815275624222</v>
-      </c>
-      <c r="C24">
-        <v>4304</v>
-      </c>
-      <c r="D24">
-        <v>2</v>
-      </c>
-      <c r="E24" t="s">
-        <v>31</v>
-      </c>
-      <c r="F24">
-        <v>0.2807484364233112</v>
-      </c>
-      <c r="G24">
-        <v>0.0339999381192182</v>
-      </c>
-      <c r="H24">
-        <v>1.01415988318014</v>
-      </c>
-      <c r="I24" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25">
-        <v>412340</v>
-      </c>
-      <c r="B25">
-        <v>20.80731228216598</v>
-      </c>
-      <c r="C25">
-        <v>11730</v>
-      </c>
-      <c r="D25">
-        <v>5</v>
-      </c>
-      <c r="E25" t="s">
-        <v>32</v>
-      </c>
-      <c r="F25">
-        <v>0.240300137384179</v>
-      </c>
-      <c r="G25">
-        <v>0.07802480051736026</v>
-      </c>
-      <c r="H25">
-        <v>0.5607803603410919</v>
-      </c>
-      <c r="I25" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26">
-        <v>411420</v>
-      </c>
-      <c r="B26">
-        <v>68.07110150340571</v>
-      </c>
-      <c r="C26">
-        <v>38313</v>
-      </c>
-      <c r="D26">
-        <v>15</v>
-      </c>
-      <c r="E26" t="s">
-        <v>33</v>
-      </c>
-      <c r="F26">
-        <v>0.2203578268709156</v>
-      </c>
-      <c r="G26">
-        <v>0.1233326029308234</v>
-      </c>
-      <c r="H26">
-        <v>0.3634467244554291</v>
-      </c>
-      <c r="I26" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="A27">
-        <v>411000</v>
-      </c>
-      <c r="B27">
-        <v>9.501847971583485</v>
-      </c>
-      <c r="C27">
-        <v>5693</v>
-      </c>
-      <c r="D27">
-        <v>2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>35</v>
-      </c>
-      <c r="F27">
-        <v>0.2104853714752394</v>
-      </c>
-      <c r="G27">
-        <v>0.02549075498453809</v>
-      </c>
-      <c r="H27">
-        <v>0.7603455337667292</v>
-      </c>
-      <c r="I27" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="A28">
-        <v>410810</v>
-      </c>
-      <c r="B28">
-        <v>4.983881987554243</v>
-      </c>
-      <c r="C28">
-        <v>2711</v>
-      </c>
-      <c r="D28">
-        <v>1</v>
-      </c>
-      <c r="E28" t="s">
-        <v>34</v>
-      </c>
-      <c r="F28">
-        <v>0.2006468055417848</v>
-      </c>
-      <c r="G28">
-        <v>0.005079937295368057</v>
-      </c>
-      <c r="H28">
-        <v>1.117932448009888</v>
-      </c>
-      <c r="I28" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="A29">
-        <v>410730</v>
-      </c>
-      <c r="B29">
-        <v>12.82663853797248</v>
-      </c>
-      <c r="C29">
-        <v>6517</v>
-      </c>
-      <c r="D29">
-        <v>2</v>
-      </c>
-      <c r="E29" t="s">
-        <v>36</v>
-      </c>
-      <c r="F29">
-        <v>0.1559254978675139</v>
-      </c>
-      <c r="G29">
-        <v>0.01888330117254954</v>
-      </c>
-      <c r="H29">
-        <v>0.5632565107635732</v>
-      </c>
-      <c r="I29" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9">
-      <c r="A30">
-        <v>410115</v>
-      </c>
-      <c r="B30">
-        <v>6.145522885780435</v>
-      </c>
-      <c r="C30">
-        <v>3357</v>
-      </c>
-      <c r="D30">
-        <v>0</v>
-      </c>
-      <c r="E30" t="s">
-        <v>252</v>
-      </c>
-      <c r="F30">
-        <v>0</v>
-      </c>
-      <c r="G30">
-        <v>0</v>
-      </c>
-      <c r="H30">
-        <v>0.6002547745203743</v>
-      </c>
-      <c r="I30" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9">
-      <c r="A31">
-        <v>411160</v>
-      </c>
-      <c r="B31">
-        <v>4.926678081056779</v>
-      </c>
-      <c r="C31">
-        <v>2685</v>
-      </c>
-      <c r="D31">
-        <v>0</v>
-      </c>
-      <c r="E31" t="s">
-        <v>253</v>
-      </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
-      <c r="G31">
-        <v>0</v>
-      </c>
-      <c r="H31">
-        <v>0.7487559352208915</v>
-      </c>
-      <c r="I31" t="s">
-        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -5276,62 +4578,906 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1">
+    <row r="1" spans="1:9" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2">
+        <v>411690</v>
+      </c>
+      <c r="B2">
+        <v>48.12545502286392</v>
+      </c>
+      <c r="C2">
+        <v>27142</v>
+      </c>
+      <c r="D2">
+        <v>116</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2">
+        <v>2.410366820321793</v>
+      </c>
+      <c r="G2">
+        <v>1.99173274218134</v>
+      </c>
+      <c r="H2">
+        <v>2.891005402695876</v>
+      </c>
+      <c r="I2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3">
+        <v>412360</v>
+      </c>
+      <c r="B3">
+        <v>3.155116935819763</v>
+      </c>
+      <c r="C3">
+        <v>1745</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>1.584727318102046</v>
+      </c>
+      <c r="G3">
+        <v>0.5145566465975075</v>
+      </c>
+      <c r="H3">
+        <v>3.698224920557817</v>
+      </c>
+      <c r="I3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4">
+        <v>412830</v>
+      </c>
+      <c r="B4">
+        <v>3.859567657577198</v>
+      </c>
+      <c r="C4">
+        <v>2106</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4">
+        <v>1.55457826687418</v>
+      </c>
+      <c r="G4">
+        <v>0.5705028254053373</v>
+      </c>
+      <c r="H4">
+        <v>3.383662415369246</v>
+      </c>
+      <c r="I4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>410220</v>
+      </c>
+      <c r="B5">
+        <v>7.255090852582689</v>
+      </c>
+      <c r="C5">
+        <v>4046</v>
+      </c>
+      <c r="D5">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5">
+        <v>1.516176740375923</v>
+      </c>
+      <c r="G5">
+        <v>0.7568699660435098</v>
+      </c>
+      <c r="H5">
+        <v>2.712858999731958</v>
+      </c>
+      <c r="I5" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6">
+        <v>411090</v>
+      </c>
+      <c r="B6">
+        <v>8.021518270582693</v>
+      </c>
+      <c r="C6">
+        <v>4530</v>
+      </c>
+      <c r="D6">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>1.371311468595701</v>
+      </c>
+      <c r="G6">
+        <v>0.6845537443172779</v>
+      </c>
+      <c r="H6">
+        <v>2.453655012603023</v>
+      </c>
+      <c r="I6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7">
+        <v>411520</v>
+      </c>
+      <c r="B7">
+        <v>716.5637350054662</v>
+      </c>
+      <c r="C7">
+        <v>429660</v>
+      </c>
+      <c r="D7">
+        <v>979</v>
+      </c>
+      <c r="E7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7">
+        <v>1.366242739025206</v>
+      </c>
+      <c r="G7">
+        <v>1.281989679080585</v>
+      </c>
+      <c r="H7">
+        <v>1.454578453179668</v>
+      </c>
+      <c r="I7" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8">
+        <v>411740</v>
+      </c>
+      <c r="B8">
+        <v>5.947173844366641</v>
+      </c>
+      <c r="C8">
+        <v>3193</v>
+      </c>
+      <c r="D8">
+        <v>8</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8">
+        <v>1.345176752749184</v>
+      </c>
+      <c r="G8">
+        <v>0.5807518440073994</v>
+      </c>
+      <c r="H8">
+        <v>2.650534461023824</v>
+      </c>
+      <c r="I8" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9">
+        <v>411640</v>
+      </c>
+      <c r="B9">
+        <v>6.127295797859569</v>
+      </c>
+      <c r="C9">
+        <v>3669</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9">
+        <v>1.305633066187961</v>
+      </c>
+      <c r="G9">
+        <v>0.5636796868783484</v>
+      </c>
+      <c r="H9">
+        <v>2.572617634307752</v>
+      </c>
+      <c r="I9" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10">
+        <v>412530</v>
+      </c>
+      <c r="B10">
+        <v>9.977716427528796</v>
+      </c>
+      <c r="C10">
+        <v>5170</v>
+      </c>
+      <c r="D10">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10">
+        <v>1.202680000695517</v>
+      </c>
+      <c r="G10">
+        <v>0.6214423063392198</v>
+      </c>
+      <c r="H10">
+        <v>2.100839926693383</v>
+      </c>
+      <c r="I10" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11">
+        <v>412450</v>
+      </c>
+      <c r="B11">
+        <v>11.75741838428178</v>
+      </c>
+      <c r="C11">
+        <v>6463</v>
+      </c>
+      <c r="D11">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11">
+        <v>1.190737587319022</v>
+      </c>
+      <c r="G11">
+        <v>0.650987319336442</v>
+      </c>
+      <c r="H11">
+        <v>1.997855341546602</v>
+      </c>
+      <c r="I11" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12">
+        <v>410590</v>
+      </c>
+      <c r="B12">
+        <v>41.10532485985631</v>
+      </c>
+      <c r="C12">
+        <v>23313</v>
+      </c>
+      <c r="D12">
+        <v>43</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12">
+        <v>1.04609318005887</v>
+      </c>
+      <c r="G12">
+        <v>0.7570628213756917</v>
+      </c>
+      <c r="H12">
+        <v>1.409080648501317</v>
+      </c>
+      <c r="I12" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13">
+        <v>411110</v>
+      </c>
+      <c r="B13">
+        <v>10.83622974078015</v>
+      </c>
+      <c r="C13">
+        <v>6228</v>
+      </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13">
+        <v>0.9228301945617525</v>
+      </c>
+      <c r="G13">
+        <v>0.4425329483451123</v>
+      </c>
+      <c r="H13">
+        <v>1.697117584431517</v>
+      </c>
+      <c r="I13" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14">
+        <v>411480</v>
+      </c>
+      <c r="B14">
+        <v>77.05655825943418</v>
+      </c>
+      <c r="C14">
+        <v>44749</v>
+      </c>
+      <c r="D14">
+        <v>65</v>
+      </c>
+      <c r="E14" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14">
+        <v>0.84353624750742</v>
+      </c>
+      <c r="G14">
+        <v>0.651023467208807</v>
+      </c>
+      <c r="H14">
+        <v>1.075156192895864</v>
+      </c>
+      <c r="I14" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15">
+        <v>410780</v>
+      </c>
+      <c r="B15">
+        <v>9.751270044256897</v>
+      </c>
+      <c r="C15">
+        <v>4805</v>
+      </c>
+      <c r="D15">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15">
+        <v>0.7178552094475854</v>
+      </c>
+      <c r="G15">
+        <v>0.288615025401477</v>
+      </c>
+      <c r="H15">
+        <v>1.479056091795627</v>
+      </c>
+      <c r="I15" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16">
+        <v>412625</v>
+      </c>
+      <c r="B16">
+        <v>205.7501103536692</v>
+      </c>
+      <c r="C16">
+        <v>128106</v>
+      </c>
+      <c r="D16">
+        <v>135</v>
+      </c>
+      <c r="E16" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16">
+        <v>0.6561357355675045</v>
+      </c>
+      <c r="G16">
+        <v>0.5501270519024235</v>
+      </c>
+      <c r="H16">
+        <v>0.7766160524041902</v>
+      </c>
+      <c r="I16" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17">
+        <v>411810</v>
+      </c>
+      <c r="B17">
+        <v>16.17068824093462</v>
+      </c>
+      <c r="C17">
+        <v>9549</v>
+      </c>
+      <c r="D17">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17">
+        <v>0.6184028688825943</v>
+      </c>
+      <c r="G17">
+        <v>0.296548212709546</v>
+      </c>
+      <c r="H17">
+        <v>1.137264893615615</v>
+      </c>
+      <c r="I17" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18">
+        <v>410210</v>
+      </c>
+      <c r="B18">
+        <v>48.39199414901175</v>
+      </c>
+      <c r="C18">
+        <v>26203</v>
+      </c>
+      <c r="D18">
+        <v>19</v>
+      </c>
+      <c r="E18" t="s">
+        <v>26</v>
+      </c>
+      <c r="F18">
+        <v>0.3926269279479158</v>
+      </c>
+      <c r="G18">
+        <v>0.2363870587589816</v>
+      </c>
+      <c r="H18">
+        <v>0.6131355835475842</v>
+      </c>
+      <c r="I18" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19">
+        <v>411360</v>
+      </c>
+      <c r="B19">
+        <v>7.757545209160687</v>
+      </c>
+      <c r="C19">
+        <v>4707</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>27</v>
+      </c>
+      <c r="F19">
+        <v>0.3867202728586585</v>
+      </c>
+      <c r="G19">
+        <v>0.07975101739207749</v>
+      </c>
+      <c r="H19">
+        <v>1.130160744585706</v>
+      </c>
+      <c r="I19" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20">
+        <v>411630</v>
+      </c>
+      <c r="B20">
+        <v>8.01975541942967</v>
+      </c>
+      <c r="C20">
+        <v>4057</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20">
+        <v>0.3740762458580498</v>
+      </c>
+      <c r="G20">
+        <v>0.07714351504993885</v>
+      </c>
+      <c r="H20">
+        <v>1.093209532113863</v>
+      </c>
+      <c r="I20" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21">
+        <v>410790</v>
+      </c>
+      <c r="B21">
+        <v>20.16185207845889</v>
+      </c>
+      <c r="C21">
+        <v>11522</v>
+      </c>
+      <c r="D21">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21">
+        <v>0.3471903262041519</v>
+      </c>
+      <c r="G21">
+        <v>0.1395885179877278</v>
+      </c>
+      <c r="H21">
+        <v>0.7153447662237189</v>
+      </c>
+      <c r="I21" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22">
+        <v>411750</v>
+      </c>
+      <c r="B22">
+        <v>80.26117696248403</v>
+      </c>
+      <c r="C22">
+        <v>48695</v>
+      </c>
+      <c r="D22">
+        <v>24</v>
+      </c>
+      <c r="E22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22">
+        <v>0.29902377348912</v>
+      </c>
+      <c r="G22">
+        <v>0.1915901739376953</v>
+      </c>
+      <c r="H22">
+        <v>0.4449236722562011</v>
+      </c>
+      <c r="I22" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23">
+        <v>411410</v>
+      </c>
+      <c r="B23">
+        <v>59.56060795845098</v>
+      </c>
+      <c r="C23">
+        <v>34521</v>
+      </c>
+      <c r="D23">
+        <v>17</v>
+      </c>
+      <c r="E23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23">
+        <v>0.285423547252222</v>
+      </c>
+      <c r="G23">
+        <v>0.1662697344613345</v>
+      </c>
+      <c r="H23">
+        <v>0.4569907485647919</v>
+      </c>
+      <c r="I23" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24">
+        <v>412040</v>
+      </c>
+      <c r="B24">
+        <v>7.123815275624222</v>
+      </c>
+      <c r="C24">
+        <v>4304</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24">
+        <v>0.2807484364233112</v>
+      </c>
+      <c r="G24">
+        <v>0.0339999381192182</v>
+      </c>
+      <c r="H24">
+        <v>1.01415988318014</v>
+      </c>
+      <c r="I24" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25">
+        <v>412340</v>
+      </c>
+      <c r="B25">
+        <v>20.80731228216598</v>
+      </c>
+      <c r="C25">
+        <v>11730</v>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+      <c r="E25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25">
+        <v>0.240300137384179</v>
+      </c>
+      <c r="G25">
+        <v>0.07802480051736026</v>
+      </c>
+      <c r="H25">
+        <v>0.5607803603410919</v>
+      </c>
+      <c r="I25" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26">
+        <v>411420</v>
+      </c>
+      <c r="B26">
+        <v>68.07110150340571</v>
+      </c>
+      <c r="C26">
+        <v>38313</v>
+      </c>
+      <c r="D26">
+        <v>15</v>
+      </c>
+      <c r="E26" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26">
+        <v>0.2203578268709156</v>
+      </c>
+      <c r="G26">
+        <v>0.1233326029308234</v>
+      </c>
+      <c r="H26">
+        <v>0.3634467244554291</v>
+      </c>
+      <c r="I26" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27">
+        <v>411000</v>
+      </c>
+      <c r="B27">
+        <v>9.501847971583485</v>
+      </c>
+      <c r="C27">
+        <v>5693</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27" t="s">
+        <v>35</v>
+      </c>
+      <c r="F27">
+        <v>0.2104853714752394</v>
+      </c>
+      <c r="G27">
+        <v>0.02549075498453809</v>
+      </c>
+      <c r="H27">
+        <v>0.7603455337667292</v>
+      </c>
+      <c r="I27" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28">
+        <v>410810</v>
+      </c>
+      <c r="B28">
+        <v>4.983881987554243</v>
+      </c>
+      <c r="C28">
+        <v>2711</v>
+      </c>
+      <c r="D28">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>254</v>
-      </c>
-      <c r="B2">
-        <v>1494</v>
-      </c>
-      <c r="C2">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>255</v>
-      </c>
-      <c r="B3">
-        <v>23</v>
-      </c>
-      <c r="C3">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>256</v>
-      </c>
-      <c r="B4">
-        <v>8</v>
-      </c>
-      <c r="C4">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>257</v>
-      </c>
-      <c r="B5">
-        <v>15</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
+      <c r="E28" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28">
+        <v>0.2006468055417848</v>
+      </c>
+      <c r="G28">
+        <v>0.005079937295368057</v>
+      </c>
+      <c r="H28">
+        <v>1.117932448009888</v>
+      </c>
+      <c r="I28" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29">
+        <v>410730</v>
+      </c>
+      <c r="B29">
+        <v>12.82663853797248</v>
+      </c>
+      <c r="C29">
+        <v>6517</v>
+      </c>
+      <c r="D29">
+        <v>2</v>
+      </c>
+      <c r="E29" t="s">
+        <v>36</v>
+      </c>
+      <c r="F29">
+        <v>0.1559254978675139</v>
+      </c>
+      <c r="G29">
+        <v>0.01888330117254954</v>
+      </c>
+      <c r="H29">
+        <v>0.5632565107635732</v>
+      </c>
+      <c r="I29" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30">
+        <v>410115</v>
+      </c>
+      <c r="B30">
+        <v>6.145522885780435</v>
+      </c>
+      <c r="C30">
+        <v>3357</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>265</v>
+      </c>
+      <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="H30">
+        <v>0.6002547745203743</v>
+      </c>
+      <c r="I30" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31">
+        <v>411160</v>
+      </c>
+      <c r="B31">
+        <v>4.926678081056779</v>
+      </c>
+      <c r="C31">
+        <v>2685</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>266</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0.7487559352208915</v>
+      </c>
+      <c r="I31" t="s">
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -5516,126 +5662,62 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>258</v>
+        <v>196</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>259</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>260</v>
-      </c>
-      <c r="B2" t="s">
-        <v>261</v>
+        <v>267</v>
+      </c>
+      <c r="B2">
+        <v>1494</v>
       </c>
       <c r="C2">
-        <v>160</v>
-      </c>
-      <c r="D2">
-        <v>392</v>
-      </c>
-      <c r="E2">
-        <v>40.8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>260</v>
-      </c>
-      <c r="B3" t="s">
-        <v>262</v>
+        <v>268</v>
+      </c>
+      <c r="B3">
+        <v>23</v>
       </c>
       <c r="C3">
-        <v>230</v>
-      </c>
-      <c r="D3">
-        <v>392</v>
-      </c>
-      <c r="E3">
-        <v>58.7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>260</v>
-      </c>
-      <c r="B4" t="s">
-        <v>82</v>
+        <v>269</v>
+      </c>
+      <c r="B4">
+        <v>8</v>
       </c>
       <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4">
-        <v>392</v>
-      </c>
-      <c r="E4">
         <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" t="s">
-        <v>261</v>
+        <v>270</v>
+      </c>
+      <c r="B5">
+        <v>15</v>
       </c>
       <c r="C5">
-        <v>31</v>
-      </c>
-      <c r="D5">
-        <v>59</v>
-      </c>
-      <c r="E5">
-        <v>52.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B6" t="s">
-        <v>262</v>
-      </c>
-      <c r="C6">
-        <v>28</v>
-      </c>
-      <c r="D6">
-        <v>59</v>
-      </c>
-      <c r="E6">
-        <v>47.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>59</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5645,12 +5727,141 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>273</v>
+      </c>
+      <c r="B2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C2">
+        <v>160</v>
+      </c>
+      <c r="D2">
+        <v>392</v>
+      </c>
+      <c r="E2">
+        <v>40.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C3">
+        <v>230</v>
+      </c>
+      <c r="D3">
+        <v>392</v>
+      </c>
+      <c r="E3">
+        <v>58.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>392</v>
+      </c>
+      <c r="E4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C5">
+        <v>31</v>
+      </c>
+      <c r="D5">
+        <v>59</v>
+      </c>
+      <c r="E5">
+        <v>52.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" t="s">
+        <v>275</v>
+      </c>
+      <c r="C6">
+        <v>28</v>
+      </c>
+      <c r="D6">
+        <v>59</v>
+      </c>
+      <c r="E6">
+        <v>47.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>59</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>77</v>
@@ -5672,7 +5883,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="B3">
         <v>627</v>
@@ -5683,7 +5894,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="B4">
         <v>911</v>

</xml_diff>

<commit_message>
Atualização de dados — 09/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -67,15 +67,15 @@
     <t>Nova Esperanca</t>
   </si>
   <si>
+    <t>Atalaia</t>
+  </si>
+  <si>
     <t>Santa Ines</t>
   </si>
   <si>
     <t>Uniflor</t>
   </si>
   <si>
-    <t>Atalaia</t>
-  </si>
-  <si>
     <t>Ourizona</t>
   </si>
   <si>
@@ -124,12 +124,12 @@
     <t>Floresta</t>
   </si>
   <si>
+    <t>Mandaguacu</t>
+  </si>
+  <si>
     <t>Paicandu</t>
   </si>
   <si>
-    <t>Mandaguacu</t>
-  </si>
-  <si>
     <t>Presidente Castelo Branco</t>
   </si>
   <si>
@@ -163,12 +163,12 @@
     <t>Diabetes</t>
   </si>
   <si>
+    <t>Imunodepressão</t>
+  </si>
+  <si>
     <t>Cardiopatia</t>
   </si>
   <si>
-    <t>Imunodepressão</t>
-  </si>
-  <si>
     <t>Evolução (Desfecho)</t>
   </si>
   <si>
@@ -400,25 +400,25 @@
     <t>100,0% (17)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 27,3% (11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 72,7% (11)</t>
-  </si>
-  <si>
-    <t>100,0% (11)</t>
+    <t xml:space="preserve"> 25,0% (12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 75,0% (12)</t>
+  </si>
+  <si>
+    <t>100,0% (12)</t>
   </si>
   <si>
     <t>100,0% (9)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 28,6% (42)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 95,2% (42)</t>
-  </si>
-  <si>
-    <t>100,0% (41)</t>
+    <t xml:space="preserve"> 27,9% (43)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 95,3% (43)</t>
+  </si>
+  <si>
+    <t>100,0% (42)</t>
   </si>
   <si>
     <t>100,0% (40)</t>
@@ -478,13 +478,16 @@
     <t>100,0% (3)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 29,4% (17)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 64,7% (17)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 81,2% (16)</t>
+    <t xml:space="preserve"> 27,8% (18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 66,7% (18)</t>
+  </si>
+  <si>
+    <t>100,0% (18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 83,3% (18)</t>
   </si>
   <si>
     <t xml:space="preserve"> 40,0% (15)</t>
@@ -514,19 +517,19 @@
     <t>100,0% (64)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 29,0% (974)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 76,9% (971)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 98,0% (350)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 99,7% (973)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,8% (938)</t>
+    <t xml:space="preserve"> 30,1% (941)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 76,8% (938)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 98,0% (347)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 99,7% (940)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,6% (902)</t>
   </si>
   <si>
     <t xml:space="preserve"> 25,0% (8)</t>
@@ -544,7 +547,7 @@
     <t>100,0% (114)</t>
   </si>
   <si>
-    <t>100,0% (106)</t>
+    <t>100,0% (108)</t>
   </si>
   <si>
     <t xml:space="preserve"> 37,5% (24)</t>
@@ -586,22 +589,19 @@
     <t>100,0% (14)</t>
   </si>
   <si>
-    <t>100,0% (12)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 16,7% (12)</t>
   </si>
   <si>
     <t xml:space="preserve"> 83,3% (12)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 24,4% (131)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 67,9% (131)</t>
-  </si>
-  <si>
-    <t>100,0% (131)</t>
+    <t xml:space="preserve"> 24,4% (135)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 68,1% (135)</t>
+  </si>
+  <si>
+    <t>100,0% (135)</t>
   </si>
   <si>
     <t xml:space="preserve"> 93,8% (128)</t>
@@ -676,12 +676,12 @@
     <t>UPA 24 HS GUSTAVO FARIAS</t>
   </si>
   <si>
+    <t>METROPOLITANA DE SARANDI</t>
+  </si>
+  <si>
     <t>UNIDADE DE PRONTO ATENDIMENTO UPA ZONA NORTE</t>
   </si>
   <si>
-    <t>METROPOLITANA DE SARANDI</t>
-  </si>
-  <si>
     <t>PRONTO ATENDIMENTO DA CRIANCA PAC</t>
   </si>
   <si>
@@ -778,22 +778,22 @@
     <t>inconsistentes</t>
   </si>
   <si>
+    <t>Classificação final informada sem data de encerramento</t>
+  </si>
+  <si>
     <t>Antiviral informado sem data de início</t>
   </si>
   <si>
-    <t>Classificação final informada sem data de encerramento</t>
-  </si>
-  <si>
     <t>Internação mais de 30 dias após o início dos sintomas</t>
   </si>
   <si>
     <t>Internação em UTI informada sem data de entrada</t>
   </si>
   <si>
+    <t>Evolução mais de 120 dias após a internação</t>
+  </si>
+  <si>
     <t>Evolução (cura ou óbito) informada sem classificação final</t>
-  </si>
-  <si>
-    <t>Evolução mais de 120 dias após a internação</t>
   </si>
   <si>
     <t>registros</t>
@@ -1252,10 +1252,10 @@
         <v>116</v>
       </c>
       <c r="C2">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2">
         <v>6</v>
@@ -1264,10 +1264,10 @@
         <v>427.4</v>
       </c>
       <c r="G2">
-        <v>40.5</v>
+        <v>44.2</v>
       </c>
       <c r="H2">
-        <v>10.4</v>
+        <v>11.1</v>
       </c>
       <c r="I2">
         <v>5.2</v>
@@ -1278,19 +1278,19 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>286.5</v>
+        <v>296.6</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1307,25 +1307,25 @@
         <v>11</v>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4">
-        <v>284.9</v>
+        <v>286.5</v>
       </c>
       <c r="G4">
-        <v>47.5</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -1336,28 +1336,28 @@
         <v>12</v>
       </c>
       <c r="B5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C5">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>271.9</v>
+        <v>284.9</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>47.5</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>16.7</v>
       </c>
       <c r="I5">
-        <v>9.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1452,28 +1452,28 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>979</v>
+        <v>945</v>
       </c>
       <c r="C9">
-        <v>909</v>
+        <v>867</v>
       </c>
       <c r="D9">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E9">
-        <v>296</v>
+        <v>281</v>
       </c>
       <c r="F9">
-        <v>227.9</v>
+        <v>219.9</v>
       </c>
       <c r="G9">
-        <v>19.6</v>
+        <v>18.2</v>
       </c>
       <c r="H9">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="I9">
-        <v>30.2</v>
+        <v>29.7</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1539,7 +1539,7 @@
         <v>19</v>
       </c>
       <c r="B12">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12">
         <v>40</v>
@@ -1551,7 +1551,7 @@
         <v>2</v>
       </c>
       <c r="F12">
-        <v>184.4</v>
+        <v>188.7</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1560,7 +1560,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>4.7</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1655,25 +1655,25 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="C16">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E16">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F16">
-        <v>105.4</v>
+        <v>109.3</v>
       </c>
       <c r="G16">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="H16">
-        <v>6.9</v>
+        <v>7.6</v>
       </c>
       <c r="I16">
         <v>39.3</v>
@@ -1748,7 +1748,7 @@
         <v>17</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19">
         <v>5</v>
@@ -1757,10 +1757,10 @@
         <v>72.5</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>5.9</v>
       </c>
       <c r="I19">
         <v>26.3</v>
@@ -1829,28 +1829,28 @@
         <v>29</v>
       </c>
       <c r="B22">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C22">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D22">
         <v>1</v>
       </c>
       <c r="E22">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F22">
-        <v>49.3</v>
+        <v>52.1</v>
       </c>
       <c r="G22">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="H22">
-        <v>4.2</v>
+        <v>5.9</v>
       </c>
       <c r="I22">
-        <v>62.5</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1858,28 +1858,28 @@
         <v>30</v>
       </c>
       <c r="B23">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C23">
+        <v>24</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
         <v>15</v>
       </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23">
-        <v>7</v>
-      </c>
       <c r="F23">
-        <v>49.2</v>
+        <v>49.3</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="I23">
-        <v>41.2</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -2082,13 +2082,13 @@
         <v>96</v>
       </c>
       <c r="B2">
-        <v>1526</v>
+        <v>1500</v>
       </c>
       <c r="C2">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D2">
-        <v>28.4</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2096,13 +2096,13 @@
         <v>97</v>
       </c>
       <c r="B3">
-        <v>1523</v>
+        <v>1497</v>
       </c>
       <c r="C3">
-        <v>1169</v>
+        <v>1148</v>
       </c>
       <c r="D3">
-        <v>76.8</v>
+        <v>76.7</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2110,10 +2110,10 @@
         <v>98</v>
       </c>
       <c r="B4">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C4">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D4">
         <v>97.8</v>
@@ -2124,10 +2124,10 @@
         <v>99</v>
       </c>
       <c r="B5">
-        <v>1521</v>
+        <v>1495</v>
       </c>
       <c r="C5">
-        <v>1514</v>
+        <v>1488</v>
       </c>
       <c r="D5">
         <v>99.5</v>
@@ -2138,13 +2138,13 @@
         <v>100</v>
       </c>
       <c r="B6">
-        <v>1457</v>
+        <v>1425</v>
       </c>
       <c r="C6">
-        <v>1371</v>
+        <v>1340</v>
       </c>
       <c r="D6">
-        <v>94.09999999999999</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2188,25 +2188,25 @@
         <v>104</v>
       </c>
       <c r="B2">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E2">
         <v>10254</v>
       </c>
       <c r="F2">
-        <v>2681.9</v>
+        <v>2720.9</v>
       </c>
       <c r="G2">
         <v>39</v>
       </c>
       <c r="H2">
-        <v>946</v>
+        <v>955.7</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2214,25 +2214,25 @@
         <v>105</v>
       </c>
       <c r="B3">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E3">
         <v>42663</v>
       </c>
       <c r="F3">
-        <v>628.2</v>
+        <v>630.5</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>138.3</v>
+        <v>135.9</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2240,7 +2240,7 @@
         <v>106</v>
       </c>
       <c r="B4">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -2252,7 +2252,7 @@
         <v>58201</v>
       </c>
       <c r="F4">
-        <v>161.5</v>
+        <v>163.2</v>
       </c>
       <c r="G4">
         <v>1.7</v>
@@ -2266,7 +2266,7 @@
         <v>107</v>
       </c>
       <c r="B5">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -2278,7 +2278,7 @@
         <v>57229</v>
       </c>
       <c r="F5">
-        <v>57.7</v>
+        <v>59.4</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -2344,7 +2344,7 @@
         <v>110</v>
       </c>
       <c r="B8">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -2356,7 +2356,7 @@
         <v>139537</v>
       </c>
       <c r="F8">
-        <v>23.6</v>
+        <v>22.9</v>
       </c>
       <c r="G8">
         <v>0.7</v>
@@ -2370,25 +2370,25 @@
         <v>111</v>
       </c>
       <c r="B9">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E9">
         <v>129814</v>
       </c>
       <c r="F9">
-        <v>38.5</v>
+        <v>37.7</v>
       </c>
       <c r="G9">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="H9">
-        <v>13.9</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2399,10 +2399,10 @@
         <v>84</v>
       </c>
       <c r="C10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D10">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E10">
         <v>114639</v>
@@ -2411,10 +2411,10 @@
         <v>73.3</v>
       </c>
       <c r="G10">
-        <v>4.4</v>
+        <v>5.2</v>
       </c>
       <c r="H10">
-        <v>25.3</v>
+        <v>24.4</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2422,25 +2422,25 @@
         <v>113</v>
       </c>
       <c r="B11">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="C11">
         <v>15</v>
       </c>
       <c r="D11">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E11">
         <v>91102</v>
       </c>
       <c r="F11">
-        <v>163.6</v>
+        <v>158.1</v>
       </c>
       <c r="G11">
         <v>16.5</v>
       </c>
       <c r="H11">
-        <v>69.2</v>
+        <v>63.7</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2448,25 +2448,25 @@
         <v>114</v>
       </c>
       <c r="B12">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="C12">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D12">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E12">
         <v>53206</v>
       </c>
       <c r="F12">
-        <v>383.4</v>
+        <v>364.6</v>
       </c>
       <c r="G12">
-        <v>50.7</v>
+        <v>48.9</v>
       </c>
       <c r="H12">
-        <v>109</v>
+        <v>105.3</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2474,25 +2474,25 @@
         <v>115</v>
       </c>
       <c r="B13">
-        <v>320</v>
+        <v>304</v>
       </c>
       <c r="C13">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D13">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E13">
         <v>23417</v>
       </c>
       <c r="F13">
-        <v>1366.5</v>
+        <v>1298.2</v>
       </c>
       <c r="G13">
-        <v>230.6</v>
+        <v>217.8</v>
       </c>
       <c r="H13">
-        <v>341.6</v>
+        <v>320.3</v>
       </c>
     </row>
   </sheetData>
@@ -2547,7 +2547,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
         <v>121</v>
@@ -2747,7 +2747,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
         <v>147</v>
@@ -2756,13 +2756,13 @@
         <v>148</v>
       </c>
       <c r="D13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E13" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="F13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2770,19 +2770,19 @@
         <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D14" t="s">
         <v>131</v>
       </c>
       <c r="E14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2790,19 +2790,19 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2810,19 +2810,19 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C16" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D16" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2850,10 +2850,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C18" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D18" t="s">
         <v>118</v>
@@ -2870,19 +2870,19 @@
         <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C19" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D19" t="s">
         <v>131</v>
       </c>
       <c r="E19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2890,10 +2890,10 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D20" t="s">
         <v>118</v>
@@ -2902,27 +2902,27 @@
         <v>145</v>
       </c>
       <c r="F20" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D21" t="s">
         <v>131</v>
       </c>
       <c r="E21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2930,7 +2930,7 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C22" t="s">
         <v>141</v>
@@ -2970,39 +2970,39 @@
         <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C24" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D24" t="s">
         <v>131</v>
       </c>
       <c r="E24" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F24" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B25" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C25" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D25" t="s">
         <v>118</v>
       </c>
       <c r="E25" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F25" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -3010,19 +3010,19 @@
         <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D26" t="s">
         <v>118</v>
       </c>
       <c r="E26" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F26" t="s">
-        <v>183</v>
+        <v>123</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -3039,10 +3039,10 @@
         <v>118</v>
       </c>
       <c r="E27" t="s">
-        <v>183</v>
+        <v>123</v>
       </c>
       <c r="F27" t="s">
-        <v>183</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -3056,7 +3056,7 @@
         <v>187</v>
       </c>
       <c r="D28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E28" t="s">
         <v>188</v>
@@ -3067,7 +3067,7 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B29" t="s">
         <v>190</v>
@@ -3132,7 +3132,7 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1550</v>
+        <v>1522</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -3152,10 +3152,10 @@
         <v>90</v>
       </c>
       <c r="D3">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="E3">
-        <v>1361</v>
+        <v>1327</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -3178,7 +3178,7 @@
         <v>92.90000000000001</v>
       </c>
       <c r="E4">
-        <v>1564</v>
+        <v>1537</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -3201,7 +3201,7 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1557</v>
+        <v>1531</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -3224,7 +3224,7 @@
         <v>99.8</v>
       </c>
       <c r="E6">
-        <v>485</v>
+        <v>473</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
@@ -3247,7 +3247,7 @@
         <v>100</v>
       </c>
       <c r="E7">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -3323,10 +3323,10 @@
         <v>213</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C3">
-        <v>101</v>
+        <v>277</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -3335,10 +3335,10 @@
         <v>5</v>
       </c>
       <c r="F3">
-        <v>37.6</v>
+        <v>36.5</v>
       </c>
       <c r="G3">
-        <v>97</v>
+        <v>98.2</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -3349,10 +3349,10 @@
         <v>214</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C4">
-        <v>315</v>
+        <v>101</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -3361,10 +3361,10 @@
         <v>5</v>
       </c>
       <c r="F4">
-        <v>38.4</v>
+        <v>37.6</v>
       </c>
       <c r="G4">
-        <v>98.40000000000001</v>
+        <v>97</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -3378,7 +3378,7 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -3387,7 +3387,7 @@
         <v>5</v>
       </c>
       <c r="F5">
-        <v>41</v>
+        <v>41.5</v>
       </c>
       <c r="G5">
         <v>97.7</v>
@@ -3436,7 +3436,7 @@
         <v>1</v>
       </c>
       <c r="E7">
-        <v>86</v>
+        <v>138</v>
       </c>
       <c r="F7">
         <v>55.6</v>
@@ -3445,7 +3445,7 @@
         <v>66.7</v>
       </c>
       <c r="H7">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -3482,7 +3482,7 @@
         <v>16</v>
       </c>
       <c r="C9">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -3491,10 +3491,10 @@
         <v>5</v>
       </c>
       <c r="F9">
-        <v>67.2</v>
+        <v>69</v>
       </c>
       <c r="G9">
-        <v>97</v>
+        <v>97.2</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -3560,7 +3560,7 @@
         <v>16</v>
       </c>
       <c r="C12">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -3569,10 +3569,10 @@
         <v>4</v>
       </c>
       <c r="F12">
-        <v>80.2</v>
+        <v>80.7</v>
       </c>
       <c r="G12">
-        <v>98.8</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -3586,7 +3586,7 @@
         <v>16</v>
       </c>
       <c r="C13">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -3595,7 +3595,7 @@
         <v>2</v>
       </c>
       <c r="F13">
-        <v>86.3</v>
+        <v>86.7</v>
       </c>
       <c r="G13">
         <v>99.3</v>
@@ -3612,7 +3612,7 @@
         <v>16</v>
       </c>
       <c r="C14">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -3621,10 +3621,10 @@
         <v>4</v>
       </c>
       <c r="F14">
-        <v>88.5</v>
+        <v>88</v>
       </c>
       <c r="G14">
-        <v>90.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="H14">
         <v>4</v>
@@ -3801,7 +3801,7 @@
         <v>46023</v>
       </c>
       <c r="B2">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -3810,7 +3810,7 @@
         <v>3</v>
       </c>
       <c r="E2">
-        <v>64.90000000000001</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="F2">
         <v>100</v>
@@ -3824,7 +3824,7 @@
         <v>46054</v>
       </c>
       <c r="B3">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -3833,10 +3833,10 @@
         <v>5</v>
       </c>
       <c r="E3">
-        <v>57.7</v>
+        <v>58.5</v>
       </c>
       <c r="F3">
-        <v>95.90000000000001</v>
+        <v>95.7</v>
       </c>
       <c r="G3">
         <v>4</v>
@@ -3847,7 +3847,7 @@
         <v>46082</v>
       </c>
       <c r="B4">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -3856,13 +3856,13 @@
         <v>4</v>
       </c>
       <c r="E4">
-        <v>67.2</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="F4">
-        <v>98.3</v>
+        <v>97.5</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -3870,16 +3870,16 @@
         <v>46113</v>
       </c>
       <c r="B5">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D5">
         <v>5</v>
       </c>
       <c r="E5">
-        <v>48.8</v>
+        <v>50</v>
       </c>
       <c r="F5">
         <v>99.40000000000001</v>
@@ -3893,7 +3893,7 @@
         <v>46143</v>
       </c>
       <c r="B6">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -3902,7 +3902,7 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>51.2</v>
+        <v>50.8</v>
       </c>
       <c r="F6">
         <v>97.5</v>
@@ -3916,7 +3916,7 @@
         <v>46174</v>
       </c>
       <c r="B7">
-        <v>286</v>
+        <v>268</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -3925,10 +3925,10 @@
         <v>5</v>
       </c>
       <c r="E7">
-        <v>59.8</v>
+        <v>59.3</v>
       </c>
       <c r="F7">
-        <v>97.2</v>
+        <v>97</v>
       </c>
       <c r="G7">
         <v>2</v>
@@ -3939,7 +3939,7 @@
         <v>46204</v>
       </c>
       <c r="B8">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -3948,10 +3948,10 @@
         <v>4</v>
       </c>
       <c r="E8">
-        <v>65</v>
+        <v>65.2</v>
       </c>
       <c r="F8">
-        <v>95</v>
+        <v>95.3</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -3962,7 +3962,7 @@
         <v>46235</v>
       </c>
       <c r="B9">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -3971,7 +3971,7 @@
         <v>3</v>
       </c>
       <c r="E9">
-        <v>62.8</v>
+        <v>62.7</v>
       </c>
       <c r="F9">
         <v>99.40000000000001</v>
@@ -3985,16 +3985,16 @@
         <v>46266</v>
       </c>
       <c r="B10">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>65.5</v>
+        <v>76.2</v>
       </c>
       <c r="F10">
         <v>100</v>
@@ -4041,7 +4041,7 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>1533</v>
+        <v>1508</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -4058,13 +4058,13 @@
         <v>241</v>
       </c>
       <c r="B3">
-        <v>888</v>
+        <v>867</v>
       </c>
       <c r="C3">
-        <v>1540</v>
+        <v>1514</v>
       </c>
       <c r="D3">
-        <v>57.7</v>
+        <v>57.3</v>
       </c>
       <c r="E3" t="s">
         <v>242</v>
@@ -4102,13 +4102,13 @@
         <v>247</v>
       </c>
       <c r="B2">
-        <v>387</v>
+        <v>1477</v>
       </c>
       <c r="C2">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -4116,13 +4116,13 @@
         <v>248</v>
       </c>
       <c r="B3">
-        <v>1506</v>
+        <v>385</v>
       </c>
       <c r="C3">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D3">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -4130,7 +4130,7 @@
         <v>249</v>
       </c>
       <c r="B4">
-        <v>1550</v>
+        <v>1522</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -4144,7 +4144,7 @@
         <v>250</v>
       </c>
       <c r="B5">
-        <v>485</v>
+        <v>473</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -4158,10 +4158,10 @@
         <v>251</v>
       </c>
       <c r="B6">
-        <v>1453</v>
+        <v>1405</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6">
         <v>0.1</v>
@@ -4172,13 +4172,13 @@
         <v>252</v>
       </c>
       <c r="B7">
-        <v>1442</v>
+        <v>1415</v>
       </c>
       <c r="C7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -4228,87 +4228,87 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="D3">
         <v>5</v>
       </c>
       <c r="E3">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="F3" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E4">
         <v>5</v>
       </c>
       <c r="F4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C5">
-        <v>78</v>
+        <v>294</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="F5" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C6">
-        <v>332</v>
+        <v>79</v>
       </c>
       <c r="D6">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="F6" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -4328,7 +4328,7 @@
         <v>2.3</v>
       </c>
       <c r="F7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -4339,7 +4339,7 @@
         <v>16</v>
       </c>
       <c r="C8">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -4348,7 +4348,7 @@
         <v>1.6</v>
       </c>
       <c r="F8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -4359,7 +4359,7 @@
         <v>9</v>
       </c>
       <c r="C9">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -4379,7 +4379,7 @@
         <v>19</v>
       </c>
       <c r="C10">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -4388,7 +4388,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -4399,16 +4399,16 @@
         <v>16</v>
       </c>
       <c r="C11">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D11">
         <v>1</v>
       </c>
       <c r="E11">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="F11" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -4433,13 +4433,13 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
       </c>
       <c r="C13">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -4615,7 +4615,7 @@
         <v>411690</v>
       </c>
       <c r="B2">
-        <v>48.12545502286392</v>
+        <v>47.17340460873341</v>
       </c>
       <c r="C2">
         <v>27142</v>
@@ -4627,13 +4627,13 @@
         <v>9</v>
       </c>
       <c r="F2">
-        <v>2.410366820321793</v>
+        <v>2.459012678057255</v>
       </c>
       <c r="G2">
-        <v>1.99173274218134</v>
+        <v>2.031929755684155</v>
       </c>
       <c r="H2">
-        <v>2.891005402695876</v>
+        <v>2.94935147531283</v>
       </c>
       <c r="I2" t="s">
         <v>262</v>
@@ -4641,28 +4641,28 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3">
-        <v>412360</v>
+        <v>410220</v>
       </c>
       <c r="B3">
-        <v>3.155116935819763</v>
+        <v>7.075974315720881</v>
       </c>
       <c r="C3">
-        <v>1745</v>
+        <v>4046</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
       </c>
       <c r="F3">
-        <v>1.584727318102046</v>
+        <v>1.695879530447034</v>
       </c>
       <c r="G3">
-        <v>0.5145566465975075</v>
+        <v>0.8762857003234499</v>
       </c>
       <c r="H3">
-        <v>3.698224920557817</v>
+        <v>2.962360250743992</v>
       </c>
       <c r="I3" t="s">
         <v>263</v>
@@ -4670,28 +4670,28 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4">
-        <v>412830</v>
+        <v>412360</v>
       </c>
       <c r="B4">
-        <v>3.859567657577198</v>
+        <v>3.088664657852097</v>
       </c>
       <c r="C4">
-        <v>2106</v>
+        <v>1745</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E4" t="s">
         <v>11</v>
       </c>
       <c r="F4">
-        <v>1.55457826687418</v>
+        <v>1.618822550803257</v>
       </c>
       <c r="G4">
-        <v>0.5705028254053373</v>
+        <v>0.5256272758491746</v>
       </c>
       <c r="H4">
-        <v>3.383662415369246</v>
+        <v>3.777791820053717</v>
       </c>
       <c r="I4" t="s">
         <v>263</v>
@@ -4699,28 +4699,28 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5">
-        <v>410220</v>
+        <v>412830</v>
       </c>
       <c r="B5">
-        <v>7.255090852582689</v>
+        <v>3.77163137528971</v>
       </c>
       <c r="C5">
-        <v>4046</v>
+        <v>2106</v>
       </c>
       <c r="D5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
       </c>
       <c r="F5">
-        <v>1.516176740375923</v>
+        <v>1.590823546359729</v>
       </c>
       <c r="G5">
-        <v>0.7568699660435098</v>
+        <v>0.5838042041745707</v>
       </c>
       <c r="H5">
-        <v>2.712858999731958</v>
+        <v>3.462553129682656</v>
       </c>
       <c r="I5" t="s">
         <v>263</v>
@@ -4731,7 +4731,7 @@
         <v>411090</v>
       </c>
       <c r="B6">
-        <v>8.021518270582693</v>
+        <v>7.882157468873373</v>
       </c>
       <c r="C6">
         <v>4530</v>
@@ -4743,13 +4743,13 @@
         <v>14</v>
       </c>
       <c r="F6">
-        <v>1.371311468595701</v>
+        <v>1.395556996093897</v>
       </c>
       <c r="G6">
-        <v>0.6845537443172779</v>
+        <v>0.6966570242882638</v>
       </c>
       <c r="H6">
-        <v>2.453655012603023</v>
+        <v>2.497036958602552</v>
       </c>
       <c r="I6" t="s">
         <v>263</v>
@@ -4757,60 +4757,60 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7">
-        <v>411520</v>
+        <v>411740</v>
       </c>
       <c r="B7">
-        <v>716.5637350054662</v>
+        <v>5.801644657208181</v>
       </c>
       <c r="C7">
-        <v>429660</v>
+        <v>3193</v>
       </c>
       <c r="D7">
-        <v>979</v>
+        <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F7">
-        <v>1.366242739025206</v>
+        <v>1.378919336271397</v>
       </c>
       <c r="G7">
-        <v>1.281989679080585</v>
+        <v>0.5953194965943547</v>
       </c>
       <c r="H7">
-        <v>1.454578453179668</v>
+        <v>2.717020802128675</v>
       </c>
       <c r="I7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8">
-        <v>411740</v>
+        <v>411520</v>
       </c>
       <c r="B8">
-        <v>5.947173844366641</v>
+        <v>702.8120800949052</v>
       </c>
       <c r="C8">
-        <v>3193</v>
+        <v>429660</v>
       </c>
       <c r="D8">
-        <v>8</v>
+        <v>945</v>
       </c>
       <c r="E8" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F8">
-        <v>1.345176752749184</v>
+        <v>1.34459840228186</v>
       </c>
       <c r="G8">
-        <v>0.5807518440073994</v>
+        <v>1.260225507373135</v>
       </c>
       <c r="H8">
-        <v>2.650534461023824</v>
+        <v>1.433134622212923</v>
       </c>
       <c r="I8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -4818,7 +4818,7 @@
         <v>411640</v>
       </c>
       <c r="B9">
-        <v>6.127295797859569</v>
+        <v>6.014727501602308</v>
       </c>
       <c r="C9">
         <v>3669</v>
@@ -4830,13 +4830,13 @@
         <v>17</v>
       </c>
       <c r="F9">
-        <v>1.305633066187961</v>
+        <v>1.330068568836879</v>
       </c>
       <c r="G9">
-        <v>0.5636796868783484</v>
+        <v>0.5742292025413304</v>
       </c>
       <c r="H9">
-        <v>2.572617634307752</v>
+        <v>2.620765315800931</v>
       </c>
       <c r="I9" t="s">
         <v>263</v>
@@ -4847,7 +4847,7 @@
         <v>412530</v>
       </c>
       <c r="B10">
-        <v>9.977716427528796</v>
+        <v>9.719069353135639</v>
       </c>
       <c r="C10">
         <v>5170</v>
@@ -4859,13 +4859,13 @@
         <v>15</v>
       </c>
       <c r="F10">
-        <v>1.202680000695517</v>
+        <v>1.234686116950948</v>
       </c>
       <c r="G10">
-        <v>0.6214423063392198</v>
+        <v>0.6379803336542443</v>
       </c>
       <c r="H10">
-        <v>2.100839926693383</v>
+        <v>2.15674817068922</v>
       </c>
       <c r="I10" t="s">
         <v>263</v>
@@ -4876,7 +4876,7 @@
         <v>412450</v>
       </c>
       <c r="B11">
-        <v>11.75741838428178</v>
+        <v>11.59266493344602</v>
       </c>
       <c r="C11">
         <v>6463</v>
@@ -4888,13 +4888,13 @@
         <v>18</v>
       </c>
       <c r="F11">
-        <v>1.190737587319022</v>
+        <v>1.207660195509367</v>
       </c>
       <c r="G11">
-        <v>0.650987319336442</v>
+        <v>0.6602390667065885</v>
       </c>
       <c r="H11">
-        <v>1.997855341546602</v>
+        <v>2.026248602602636</v>
       </c>
       <c r="I11" t="s">
         <v>263</v>
@@ -4905,25 +4905,25 @@
         <v>410590</v>
       </c>
       <c r="B12">
-        <v>41.10532485985631</v>
+        <v>40.27819798679241</v>
       </c>
       <c r="C12">
         <v>23313</v>
       </c>
       <c r="D12">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E12" t="s">
         <v>19</v>
       </c>
       <c r="F12">
-        <v>1.04609318005887</v>
+        <v>1.092402396314453</v>
       </c>
       <c r="G12">
-        <v>0.7570628213756917</v>
+        <v>0.7937412534847694</v>
       </c>
       <c r="H12">
-        <v>1.409080648501317</v>
+        <v>1.466499228681399</v>
       </c>
       <c r="I12" t="s">
         <v>263</v>
@@ -4934,7 +4934,7 @@
         <v>411110</v>
       </c>
       <c r="B13">
-        <v>10.83622974078015</v>
+        <v>10.61352899729195</v>
       </c>
       <c r="C13">
         <v>6228</v>
@@ -4946,13 +4946,13 @@
         <v>20</v>
       </c>
       <c r="F13">
-        <v>0.9228301945617525</v>
+        <v>0.9421936853002909</v>
       </c>
       <c r="G13">
-        <v>0.4425329483451123</v>
+        <v>0.4518184948056375</v>
       </c>
       <c r="H13">
-        <v>1.697117584431517</v>
+        <v>1.73272773332132</v>
       </c>
       <c r="I13" t="s">
         <v>263</v>
@@ -4963,7 +4963,7 @@
         <v>411480</v>
       </c>
       <c r="B14">
-        <v>77.05655825943418</v>
+        <v>75.81634682008129</v>
       </c>
       <c r="C14">
         <v>44749</v>
@@ -4975,13 +4975,13 @@
         <v>22</v>
       </c>
       <c r="F14">
-        <v>0.84353624750742</v>
+        <v>0.8573348984256731</v>
       </c>
       <c r="G14">
-        <v>0.651023467208807</v>
+        <v>0.6616729746723569</v>
       </c>
       <c r="H14">
-        <v>1.075156192895864</v>
+        <v>1.092743706215186</v>
       </c>
       <c r="I14" t="s">
         <v>263</v>
@@ -4992,7 +4992,7 @@
         <v>410780</v>
       </c>
       <c r="B15">
-        <v>9.751270044256897</v>
+        <v>9.495864216988322</v>
       </c>
       <c r="C15">
         <v>4805</v>
@@ -5004,13 +5004,13 @@
         <v>21</v>
       </c>
       <c r="F15">
-        <v>0.7178552094475854</v>
+        <v>0.7371630259283655</v>
       </c>
       <c r="G15">
-        <v>0.288615025401477</v>
+        <v>0.2963777690170533</v>
       </c>
       <c r="H15">
-        <v>1.479056091795627</v>
+        <v>1.518837573087858</v>
       </c>
       <c r="I15" t="s">
         <v>263</v>
@@ -5021,25 +5021,25 @@
         <v>412625</v>
       </c>
       <c r="B16">
-        <v>205.7501103536692</v>
+        <v>203.9851658248778</v>
       </c>
       <c r="C16">
         <v>128106</v>
       </c>
       <c r="D16">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="E16" t="s">
         <v>23</v>
       </c>
       <c r="F16">
-        <v>0.6561357355675045</v>
+        <v>0.6863244169440763</v>
       </c>
       <c r="G16">
-        <v>0.5501270519024235</v>
+        <v>0.5773487045345095</v>
       </c>
       <c r="H16">
-        <v>0.7766160524041902</v>
+        <v>0.8098897276804955</v>
       </c>
       <c r="I16" t="s">
         <v>264</v>
@@ -5050,7 +5050,7 @@
         <v>411810</v>
       </c>
       <c r="B17">
-        <v>16.17068824093462</v>
+        <v>15.88641562521915</v>
       </c>
       <c r="C17">
         <v>9549</v>
@@ -5062,13 +5062,13 @@
         <v>24</v>
       </c>
       <c r="F17">
-        <v>0.6184028688825943</v>
+        <v>0.629468612424148</v>
       </c>
       <c r="G17">
-        <v>0.296548212709546</v>
+        <v>0.3018546668588927</v>
       </c>
       <c r="H17">
-        <v>1.137264893615615</v>
+        <v>1.157615189975498</v>
       </c>
       <c r="I17" t="s">
         <v>263</v>
@@ -5079,7 +5079,7 @@
         <v>410210</v>
       </c>
       <c r="B18">
-        <v>48.39199414901175</v>
+        <v>47.42039187706349</v>
       </c>
       <c r="C18">
         <v>26203</v>
@@ -5091,13 +5091,13 @@
         <v>26</v>
       </c>
       <c r="F18">
-        <v>0.3926269279479158</v>
+        <v>0.4006715096167311</v>
       </c>
       <c r="G18">
-        <v>0.2363870587589816</v>
+        <v>0.2412304224314038</v>
       </c>
       <c r="H18">
-        <v>0.6131355835475842</v>
+        <v>0.6256981943233779</v>
       </c>
       <c r="I18" t="s">
         <v>264</v>
@@ -5108,7 +5108,7 @@
         <v>411360</v>
       </c>
       <c r="B19">
-        <v>7.757545209160687</v>
+        <v>7.600136934499216</v>
       </c>
       <c r="C19">
         <v>4707</v>
@@ -5120,13 +5120,13 @@
         <v>27</v>
       </c>
       <c r="F19">
-        <v>0.3867202728586585</v>
+        <v>0.3947297299844867</v>
       </c>
       <c r="G19">
-        <v>0.07975101739207749</v>
+        <v>0.0814027600065033</v>
       </c>
       <c r="H19">
-        <v>1.130160744585706</v>
+        <v>1.153567777173216</v>
       </c>
       <c r="I19" t="s">
         <v>263</v>
@@ -5137,7 +5137,7 @@
         <v>411630</v>
       </c>
       <c r="B20">
-        <v>8.01975541942967</v>
+        <v>7.846553373876229</v>
       </c>
       <c r="C20">
         <v>4057</v>
@@ -5149,13 +5149,13 @@
         <v>25</v>
       </c>
       <c r="F20">
-        <v>0.3740762458580498</v>
+        <v>0.3823334726796089</v>
       </c>
       <c r="G20">
-        <v>0.07714351504993885</v>
+        <v>0.07884635373224701</v>
       </c>
       <c r="H20">
-        <v>1.093209532113863</v>
+        <v>1.117340652894999</v>
       </c>
       <c r="I20" t="s">
         <v>263</v>
@@ -5166,7 +5166,7 @@
         <v>410790</v>
       </c>
       <c r="B21">
-        <v>20.16185207845889</v>
+        <v>19.93317023758988</v>
       </c>
       <c r="C21">
         <v>11522</v>
@@ -5178,13 +5178,13 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>0.3471903262041519</v>
+        <v>0.3511734418842935</v>
       </c>
       <c r="G21">
-        <v>0.1395885179877278</v>
+        <v>0.1411899370734592</v>
       </c>
       <c r="H21">
-        <v>0.7153447662237189</v>
+        <v>0.7235515068498317</v>
       </c>
       <c r="I21" t="s">
         <v>264</v>
@@ -5192,28 +5192,28 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22">
-        <v>411750</v>
+        <v>411410</v>
       </c>
       <c r="B22">
-        <v>80.26117696248403</v>
+        <v>58.9758919548884</v>
       </c>
       <c r="C22">
-        <v>48695</v>
+        <v>34521</v>
       </c>
       <c r="D22">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
       </c>
       <c r="F22">
-        <v>0.29902377348912</v>
+        <v>0.3052094576843108</v>
       </c>
       <c r="G22">
-        <v>0.1915901739376953</v>
+        <v>0.1808864677885602</v>
       </c>
       <c r="H22">
-        <v>0.4449236722562011</v>
+        <v>0.4823625268658613</v>
       </c>
       <c r="I22" t="s">
         <v>264</v>
@@ -5221,28 +5221,28 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23">
-        <v>411410</v>
+        <v>411750</v>
       </c>
       <c r="B23">
-        <v>59.56060795845098</v>
+        <v>79.35135855529957</v>
       </c>
       <c r="C23">
-        <v>34521</v>
+        <v>48695</v>
       </c>
       <c r="D23">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="E23" t="s">
         <v>30</v>
       </c>
       <c r="F23">
-        <v>0.285423547252222</v>
+        <v>0.3024522886180269</v>
       </c>
       <c r="G23">
-        <v>0.1662697344613345</v>
+        <v>0.1937868882732503</v>
       </c>
       <c r="H23">
-        <v>0.4569907485647919</v>
+        <v>0.4500250310001563</v>
       </c>
       <c r="I23" t="s">
         <v>264</v>
@@ -5253,7 +5253,7 @@
         <v>412040</v>
       </c>
       <c r="B24">
-        <v>7.123815275624222</v>
+        <v>7.013238548555828</v>
       </c>
       <c r="C24">
         <v>4304</v>
@@ -5265,13 +5265,13 @@
         <v>31</v>
       </c>
       <c r="F24">
-        <v>0.2807484364233112</v>
+        <v>0.2851749567839585</v>
       </c>
       <c r="G24">
-        <v>0.0339999381192182</v>
+        <v>0.03453601027072448</v>
       </c>
       <c r="H24">
-        <v>1.01415988318014</v>
+        <v>1.030149996710389</v>
       </c>
       <c r="I24" t="s">
         <v>263</v>
@@ -5282,7 +5282,7 @@
         <v>412340</v>
       </c>
       <c r="B25">
-        <v>20.80731228216598</v>
+        <v>20.37211620262686</v>
       </c>
       <c r="C25">
         <v>11730</v>
@@ -5294,13 +5294,13 @@
         <v>32</v>
       </c>
       <c r="F25">
-        <v>0.240300137384179</v>
+        <v>0.245433510700046</v>
       </c>
       <c r="G25">
-        <v>0.07802480051736026</v>
+        <v>0.07969159286010168</v>
       </c>
       <c r="H25">
-        <v>0.5607803603410919</v>
+        <v>0.5727599412484259</v>
       </c>
       <c r="I25" t="s">
         <v>264</v>
@@ -5311,7 +5311,7 @@
         <v>411420</v>
       </c>
       <c r="B26">
-        <v>68.07110150340571</v>
+        <v>66.84912943328723</v>
       </c>
       <c r="C26">
         <v>38313</v>
@@ -5323,13 +5323,13 @@
         <v>33</v>
       </c>
       <c r="F26">
-        <v>0.2203578268709156</v>
+        <v>0.2243858690032666</v>
       </c>
       <c r="G26">
-        <v>0.1233326029308234</v>
+        <v>0.1255870675348371</v>
       </c>
       <c r="H26">
-        <v>0.3634467244554291</v>
+        <v>0.370090367387291</v>
       </c>
       <c r="I26" t="s">
         <v>264</v>
@@ -5340,7 +5340,7 @@
         <v>411000</v>
       </c>
       <c r="B27">
-        <v>9.501847971583485</v>
+        <v>9.364617544753736</v>
       </c>
       <c r="C27">
         <v>5693</v>
@@ -5352,13 +5352,13 @@
         <v>35</v>
       </c>
       <c r="F27">
-        <v>0.2104853714752394</v>
+        <v>0.2135698538079052</v>
       </c>
       <c r="G27">
-        <v>0.02549075498453809</v>
+        <v>0.02586430010477639</v>
       </c>
       <c r="H27">
-        <v>0.7603455337667292</v>
+        <v>0.7714877445017908</v>
       </c>
       <c r="I27" t="s">
         <v>264</v>
@@ -5369,7 +5369,7 @@
         <v>410810</v>
       </c>
       <c r="B28">
-        <v>4.983881987554243</v>
+        <v>4.896886753566739</v>
       </c>
       <c r="C28">
         <v>2711</v>
@@ -5381,13 +5381,13 @@
         <v>34</v>
       </c>
       <c r="F28">
-        <v>0.2006468055417848</v>
+        <v>0.2042113796631362</v>
       </c>
       <c r="G28">
-        <v>0.005079937295368057</v>
+        <v>0.005170184498518202</v>
       </c>
       <c r="H28">
-        <v>1.117932448009888</v>
+        <v>1.137792983854627</v>
       </c>
       <c r="I28" t="s">
         <v>263</v>
@@ -5398,7 +5398,7 @@
         <v>410730</v>
       </c>
       <c r="B29">
-        <v>12.82663853797248</v>
+        <v>12.53112036852488</v>
       </c>
       <c r="C29">
         <v>6517</v>
@@ -5410,13 +5410,13 @@
         <v>36</v>
       </c>
       <c r="F29">
-        <v>0.1559254978675139</v>
+        <v>0.1596026485407891</v>
       </c>
       <c r="G29">
-        <v>0.01888330117254954</v>
+        <v>0.01932862117838526</v>
       </c>
       <c r="H29">
-        <v>0.5632565107635732</v>
+        <v>0.57653964332436</v>
       </c>
       <c r="I29" t="s">
         <v>264</v>
@@ -5427,7 +5427,7 @@
         <v>410115</v>
       </c>
       <c r="B30">
-        <v>6.145522885780435</v>
+        <v>6.039275026784384</v>
       </c>
       <c r="C30">
         <v>3357</v>
@@ -5445,7 +5445,7 @@
         <v>0</v>
       </c>
       <c r="H30">
-        <v>0.6002547745203743</v>
+        <v>0.6108149467864328</v>
       </c>
       <c r="I30" t="s">
         <v>264</v>
@@ -5456,7 +5456,7 @@
         <v>411160</v>
       </c>
       <c r="B31">
-        <v>4.926678081056779</v>
+        <v>4.798574750665755</v>
       </c>
       <c r="C31">
         <v>2685</v>
@@ -5474,7 +5474,7 @@
         <v>0</v>
       </c>
       <c r="H31">
-        <v>0.7487559352208915</v>
+        <v>0.7687448139892246</v>
       </c>
       <c r="I31" t="s">
         <v>264</v>
@@ -5506,10 +5506,10 @@
         <v>40</v>
       </c>
       <c r="B2">
-        <v>60.9</v>
+        <v>59.9</v>
       </c>
       <c r="C2">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5517,10 +5517,10 @@
         <v>41</v>
       </c>
       <c r="B3">
-        <v>61.3</v>
+        <v>60.4</v>
       </c>
       <c r="C3">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5528,10 +5528,10 @@
         <v>42</v>
       </c>
       <c r="B4">
-        <v>61.4</v>
+        <v>60.4</v>
       </c>
       <c r="C4">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5539,10 +5539,10 @@
         <v>43</v>
       </c>
       <c r="B5">
-        <v>61.4</v>
+        <v>60.5</v>
       </c>
       <c r="C5">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -5550,10 +5550,10 @@
         <v>44</v>
       </c>
       <c r="B6">
-        <v>92.90000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="C6">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5561,10 +5561,10 @@
         <v>45</v>
       </c>
       <c r="B7">
-        <v>95.8</v>
+        <v>95.5</v>
       </c>
       <c r="C7">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5575,7 +5575,7 @@
         <v>98.7</v>
       </c>
       <c r="C8">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -5583,10 +5583,10 @@
         <v>47</v>
       </c>
       <c r="B9">
-        <v>98.8</v>
+        <v>98.7</v>
       </c>
       <c r="C9">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -5597,7 +5597,7 @@
         <v>99.09999999999999</v>
       </c>
       <c r="C10">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -5608,7 +5608,7 @@
         <v>99.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -5619,7 +5619,7 @@
         <v>100</v>
       </c>
       <c r="C12">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -5630,7 +5630,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -5641,7 +5641,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -5652,7 +5652,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1540</v>
+        <v>1514</v>
       </c>
     </row>
   </sheetData>
@@ -5681,10 +5681,10 @@
         <v>267</v>
       </c>
       <c r="B2">
-        <v>1494</v>
+        <v>1467</v>
       </c>
       <c r="C2">
-        <v>97</v>
+        <v>96.90000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5703,10 +5703,10 @@
         <v>269</v>
       </c>
       <c r="B4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C4">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5755,13 +5755,13 @@
         <v>274</v>
       </c>
       <c r="C2">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="D2">
-        <v>392</v>
+        <v>373</v>
       </c>
       <c r="E2">
-        <v>40.8</v>
+        <v>40.2</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -5772,13 +5772,13 @@
         <v>275</v>
       </c>
       <c r="C3">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="D3">
-        <v>392</v>
+        <v>373</v>
       </c>
       <c r="E3">
-        <v>58.7</v>
+        <v>59.2</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -5792,7 +5792,7 @@
         <v>2</v>
       </c>
       <c r="D4">
-        <v>392</v>
+        <v>373</v>
       </c>
       <c r="E4">
         <v>0.5</v>
@@ -5806,13 +5806,13 @@
         <v>274</v>
       </c>
       <c r="C5">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E5">
-        <v>52.5</v>
+        <v>52.6</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -5823,13 +5823,13 @@
         <v>275</v>
       </c>
       <c r="C6">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E6">
-        <v>47.5</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -5843,7 +5843,7 @@
         <v>0</v>
       </c>
       <c r="D7">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -5886,10 +5886,10 @@
         <v>275</v>
       </c>
       <c r="B3">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="C3">
-        <v>40.7</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5897,10 +5897,10 @@
         <v>274</v>
       </c>
       <c r="B4">
-        <v>911</v>
+        <v>879</v>
       </c>
       <c r="C4">
-        <v>59.2</v>
+        <v>58.1</v>
       </c>
     </row>
   </sheetData>
@@ -5926,13 +5926,13 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B2">
-        <v>466</v>
+        <v>455</v>
       </c>
       <c r="C2">
-        <v>30.3</v>
+        <v>30.1</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5940,10 +5940,10 @@
         <v>41</v>
       </c>
       <c r="B3">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C3">
-        <v>15.3</v>
+        <v>15.1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5951,10 +5951,10 @@
         <v>57</v>
       </c>
       <c r="B4">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="C4">
-        <v>12.8</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5962,7 +5962,7 @@
         <v>58</v>
       </c>
       <c r="B5">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C5">
         <v>11.8</v>
@@ -5973,10 +5973,10 @@
         <v>59</v>
       </c>
       <c r="B6">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="C6">
-        <v>11.1</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5984,10 +5984,10 @@
         <v>60</v>
       </c>
       <c r="B7">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C7">
-        <v>4</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -6003,13 +6003,13 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C9">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -6020,7 +6020,7 @@
         <v>16</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -6031,7 +6031,7 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>
@@ -6066,7 +6066,7 @@
         <v>65</v>
       </c>
       <c r="B2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C2">
         <v>132</v>
@@ -6083,10 +6083,10 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C3">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -6100,10 +6100,10 @@
         <v>67</v>
       </c>
       <c r="B4">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C4">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -6137,7 +6137,7 @@
         <v>21</v>
       </c>
       <c r="C6">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -6151,16 +6151,16 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -6168,16 +6168,16 @@
         <v>71</v>
       </c>
       <c r="B8">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C8">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
-        <v>2.1</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -6185,10 +6185,10 @@
         <v>72</v>
       </c>
       <c r="B9">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C9">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -6208,10 +6208,10 @@
         <v>79</v>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E10">
-        <v>6.3</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -6219,7 +6219,7 @@
         <v>74</v>
       </c>
       <c r="B11">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C11">
         <v>119</v>
@@ -6236,16 +6236,16 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>673</v>
+        <v>642</v>
       </c>
       <c r="C12">
-        <v>638</v>
+        <v>606</v>
       </c>
       <c r="D12">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E12">
-        <v>15</v>
+        <v>15.2</v>
       </c>
     </row>
   </sheetData>
@@ -6277,13 +6277,13 @@
         <v>65</v>
       </c>
       <c r="B2">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C2">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D2">
-        <v>43.5</v>
+        <v>43.9</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -6291,13 +6291,13 @@
         <v>66</v>
       </c>
       <c r="B3">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C3">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3">
-        <v>22</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -6305,13 +6305,13 @@
         <v>67</v>
       </c>
       <c r="B4">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C4">
         <v>7</v>
       </c>
       <c r="D4">
-        <v>21.2</v>
+        <v>20.6</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -6347,13 +6347,13 @@
         <v>70</v>
       </c>
       <c r="B7">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7">
         <v>13</v>
       </c>
       <c r="D7">
-        <v>39.4</v>
+        <v>40.6</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -6361,13 +6361,13 @@
         <v>71</v>
       </c>
       <c r="B8">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C8">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D8">
-        <v>36</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -6375,13 +6375,13 @@
         <v>72</v>
       </c>
       <c r="B9">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C9">
         <v>23</v>
       </c>
       <c r="D9">
-        <v>24.5</v>
+        <v>24.2</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -6392,10 +6392,10 @@
         <v>84</v>
       </c>
       <c r="C10">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10">
-        <v>34.5</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -6403,13 +6403,13 @@
         <v>74</v>
       </c>
       <c r="B11">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C11">
         <v>33</v>
       </c>
       <c r="D11">
-        <v>25.8</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -6417,13 +6417,13 @@
         <v>75</v>
       </c>
       <c r="B12">
-        <v>673</v>
+        <v>642</v>
       </c>
       <c r="C12">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="D12">
-        <v>29.9</v>
+        <v>29.4</v>
       </c>
     </row>
   </sheetData>
@@ -6452,10 +6452,10 @@
         <v>78</v>
       </c>
       <c r="B2">
-        <v>880</v>
+        <v>858</v>
       </c>
       <c r="C2">
-        <v>98.8</v>
+        <v>98.59999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6474,10 +6474,10 @@
         <v>80</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>
@@ -6506,10 +6506,10 @@
         <v>82</v>
       </c>
       <c r="B2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6517,10 +6517,10 @@
         <v>83</v>
       </c>
       <c r="B3">
-        <v>1145</v>
+        <v>1120</v>
       </c>
       <c r="C3">
-        <v>74.40000000000001</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6528,10 +6528,10 @@
         <v>84</v>
       </c>
       <c r="B4">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C4">
-        <v>24.4</v>
+        <v>24.7</v>
       </c>
     </row>
   </sheetData>
@@ -6571,10 +6571,10 @@
         <v>83</v>
       </c>
       <c r="B3">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="C3">
-        <v>28.6</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6582,10 +6582,10 @@
         <v>84</v>
       </c>
       <c r="B4">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C4">
-        <v>70.90000000000001</v>
+        <v>74.3</v>
       </c>
     </row>
   </sheetData>
@@ -6629,16 +6629,16 @@
         <v>92</v>
       </c>
       <c r="B2">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C2">
         <v>44</v>
       </c>
       <c r="D2">
-        <v>74.59999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="E2">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F2">
         <v>23</v>
@@ -6655,22 +6655,22 @@
         <v>93</v>
       </c>
       <c r="B3">
-        <v>308</v>
+        <v>291</v>
       </c>
       <c r="C3">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D3">
-        <v>69.8</v>
+        <v>73.5</v>
       </c>
       <c r="E3">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="F3">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3">
-        <v>50.7</v>
+        <v>50.5</v>
       </c>
       <c r="H3">
         <v>2</v>

</xml_diff>

<commit_message>
Atualização de layout/texto — 10/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -643,7 +643,7 @@
     <t>%</t>
   </si>
   <si>
-    <t>Cobertura de amostragem (SRAG com amostra coletada até 10 dias dos sintomas)</t>
+    <t>Cobertura de amostragem (internados até 10 dias dos sintomas com amostra coletada até o 10º dia)</t>
   </si>
   <si>
     <t>Oportunidade da coleta (internação → coleta, mediana)</t>
@@ -3175,10 +3175,10 @@
         <v>90</v>
       </c>
       <c r="D4">
-        <v>92.90000000000001</v>
+        <v>98.5</v>
       </c>
       <c r="E4">
-        <v>1537</v>
+        <v>1431</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização de dados — 15/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="277">
   <si>
     <t>municipio</t>
   </si>
@@ -148,6 +148,9 @@
     <t>Doutor Camargo</t>
   </si>
   <si>
+    <t>Angulo</t>
+  </si>
+  <si>
     <t>variavel</t>
   </si>
   <si>
@@ -175,12 +178,12 @@
     <t>Critério Confirmação</t>
   </si>
   <si>
+    <t>Antiviral</t>
+  </si>
+  <si>
     <t>Raça/Cor</t>
   </si>
   <si>
-    <t>Antiviral</t>
-  </si>
-  <si>
     <t>Data Internação</t>
   </si>
   <si>
@@ -385,226 +388,226 @@
     <t>80 e mais</t>
   </si>
   <si>
+    <t>100,0% (1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  0,0% (1)</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 47,4% (19)</t>
   </si>
   <si>
     <t xml:space="preserve"> 78,9% (19)</t>
   </si>
   <si>
-    <t>—</t>
-  </si>
-  <si>
     <t>100,0% (19)</t>
   </si>
   <si>
-    <t>100,0% (17)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 25,0% (12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 75,0% (12)</t>
+    <t>100,0% (18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 23,1% (13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 76,9% (13)</t>
+  </si>
+  <si>
+    <t>100,0% (13)</t>
+  </si>
+  <si>
+    <t>100,0% (11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 27,9% (43)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 95,3% (43)</t>
+  </si>
+  <si>
+    <t>100,0% (42)</t>
+  </si>
+  <si>
+    <t>100,0% (41)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 50,0% (2)</t>
+  </si>
+  <si>
+    <t>100,0% (2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 28,6% (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 85,7% (7)</t>
+  </si>
+  <si>
+    <t>100,0% (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 57,1% (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 66,7% (3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 71,4% (7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  0,0% (2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 10,0% (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 90,0% (10)</t>
+  </si>
+  <si>
+    <t>100,0% (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 40,0% (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 70,0% (10)</t>
+  </si>
+  <si>
+    <t>100,0% (8)</t>
+  </si>
+  <si>
+    <t>100,0% (3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 27,8% (18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 66,7% (18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 83,3% (18)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 40,0% (15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 46,7% (15)</t>
+  </si>
+  <si>
+    <t>100,0% (15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,9% (14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 26,2% (65)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 56,9% (65)</t>
+  </si>
+  <si>
+    <t>100,0% (4)</t>
+  </si>
+  <si>
+    <t>100,0% (65)</t>
+  </si>
+  <si>
+    <t>100,0% (64)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 30,2% (945)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 76,5% (942)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 98,0% (347)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 99,7% (944)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,6% (910)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 25,0% (8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 87,5% (8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 25,9% (116)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,2% (116)</t>
+  </si>
+  <si>
+    <t>100,0% (114)</t>
+  </si>
+  <si>
+    <t>100,0% (109)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 37,5% (24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 75,0% (24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 95,8% (24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 82,6% (23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 50,0% (10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 20,0% (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 60,0% (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 80,0% (5)</t>
+  </si>
+  <si>
+    <t>100,0% (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 25,0% (4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 14,3% (14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 85,7% (14)</t>
+  </si>
+  <si>
+    <t>100,0% (14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 16,7% (12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 83,3% (12)</t>
   </si>
   <si>
     <t>100,0% (12)</t>
   </si>
   <si>
-    <t>100,0% (9)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 27,9% (43)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 95,3% (43)</t>
-  </si>
-  <si>
-    <t>100,0% (42)</t>
-  </si>
-  <si>
-    <t>100,0% (40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 50,0% (2)</t>
-  </si>
-  <si>
-    <t>100,0% (2)</t>
-  </si>
-  <si>
-    <t>100,0% (1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 28,6% (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 85,7% (7)</t>
-  </si>
-  <si>
-    <t>100,0% (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 57,1% (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 66,7% (3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 71,4% (7)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  0,0% (1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  0,0% (2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 10,0% (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 90,0% (10)</t>
-  </si>
-  <si>
-    <t>100,0% (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 40,0% (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 70,0% (10)</t>
-  </si>
-  <si>
-    <t>100,0% (8)</t>
-  </si>
-  <si>
-    <t>100,0% (3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 27,8% (18)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 66,7% (18)</t>
-  </si>
-  <si>
-    <t>100,0% (18)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 83,3% (18)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 40,0% (15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 46,7% (15)</t>
-  </si>
-  <si>
-    <t>100,0% (15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,9% (14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 27,7% (65)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 55,4% (65)</t>
-  </si>
-  <si>
-    <t>100,0% (4)</t>
-  </si>
-  <si>
-    <t>100,0% (65)</t>
-  </si>
-  <si>
-    <t>100,0% (64)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 30,1% (941)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 76,8% (938)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 98,0% (347)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 99,7% (940)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,6% (902)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 25,0% (8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 87,5% (8)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 25,9% (116)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,2% (116)</t>
-  </si>
-  <si>
-    <t>100,0% (114)</t>
-  </si>
-  <si>
-    <t>100,0% (108)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 37,5% (24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 75,0% (24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 95,8% (24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 82,6% (23)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 50,0% (10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 20,0% (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 60,0% (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 80,0% (5)</t>
-  </si>
-  <si>
-    <t>100,0% (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 25,0% (4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 14,3% (14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 85,7% (14)</t>
-  </si>
-  <si>
-    <t>100,0% (14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 16,7% (12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 83,3% (12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 24,4% (135)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 68,1% (135)</t>
-  </si>
-  <si>
-    <t>100,0% (135)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 93,8% (128)</t>
+    <t xml:space="preserve"> 25,0% (136)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 67,6% (136)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 99,3% (136)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 93,8% (130)</t>
   </si>
   <si>
     <t xml:space="preserve">  0,0% (6)</t>
@@ -694,12 +697,12 @@
     <t>HOSP MUN E REG SAGRADO CORACAO DE JESUS NOVA ESPERANCA</t>
   </si>
   <si>
+    <t>HOSPITAL E MATERNIDADE SAO MARCOS</t>
+  </si>
+  <si>
     <t>HOSPITAL MUNICIPAL DE MARINGA THELMA VILLANOVA KASPROWICZ</t>
   </si>
   <si>
-    <t>HOSPITAL E MATERNIDADE SAO MARCOS</t>
-  </si>
-  <si>
     <t>HOSPITAL E MATERNIDADE SANTA CLARA</t>
   </si>
   <si>
@@ -830,9 +833,6 @@
   </si>
   <si>
     <t>abaixo</t>
-  </si>
-  <si>
-    <t>Angulo</t>
   </si>
   <si>
     <t>Ivatuba</t>
@@ -1212,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1">
@@ -1252,7 +1252,7 @@
         <v>116</v>
       </c>
       <c r="C2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -1267,7 +1267,7 @@
         <v>44.2</v>
       </c>
       <c r="H2">
-        <v>11.1</v>
+        <v>11</v>
       </c>
       <c r="I2">
         <v>5.2</v>
@@ -1278,10 +1278,10 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -1290,7 +1290,7 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>296.6</v>
+        <v>321.3</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1299,7 +1299,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1310,10 +1310,10 @@
         <v>5</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -1322,10 +1322,10 @@
         <v>286.5</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>57.3</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -1397,7 +1397,7 @@
         <v>11</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1412,7 +1412,7 @@
         <v>22.1</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>9.1</v>
       </c>
       <c r="I7">
         <v>9.1</v>
@@ -1452,28 +1452,28 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>945</v>
+        <v>949</v>
       </c>
       <c r="C9">
-        <v>867</v>
+        <v>874</v>
       </c>
       <c r="D9">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E9">
         <v>281</v>
       </c>
       <c r="F9">
-        <v>219.9</v>
+        <v>220.9</v>
       </c>
       <c r="G9">
-        <v>18.2</v>
+        <v>18.6</v>
       </c>
       <c r="H9">
-        <v>9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I9">
-        <v>29.7</v>
+        <v>29.6</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1513,7 +1513,7 @@
         <v>14</v>
       </c>
       <c r="C11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -1542,7 +1542,7 @@
         <v>44</v>
       </c>
       <c r="C12">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -1635,7 +1635,7 @@
         <v>2</v>
       </c>
       <c r="E15">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F15">
         <v>145.3</v>
@@ -1647,7 +1647,7 @@
         <v>3.1</v>
       </c>
       <c r="I15">
-        <v>47.7</v>
+        <v>46.2</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1655,28 +1655,28 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C16">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D16">
         <v>10</v>
       </c>
       <c r="E16">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F16">
-        <v>109.3</v>
+        <v>110.1</v>
       </c>
       <c r="G16">
         <v>7.8</v>
       </c>
       <c r="H16">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="I16">
-        <v>39.3</v>
+        <v>39.7</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1745,7 +1745,7 @@
         <v>19</v>
       </c>
       <c r="C19">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1760,7 +1760,7 @@
         <v>3.8</v>
       </c>
       <c r="H19">
-        <v>5.9</v>
+        <v>5.6</v>
       </c>
       <c r="I19">
         <v>26.3</v>
@@ -2051,6 +2051,32 @@
       </c>
       <c r="I29">
         <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
+        <v>29.8</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2065,49 +2091,49 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B2">
-        <v>1500</v>
+        <v>1507</v>
       </c>
       <c r="C2">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="D2">
-        <v>29</v>
+        <v>29.1</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B3">
-        <v>1497</v>
+        <v>1504</v>
       </c>
       <c r="C3">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="D3">
-        <v>76.7</v>
+        <v>76.5</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B4">
         <v>370</v>
@@ -2121,13 +2147,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B5">
-        <v>1495</v>
+        <v>1502</v>
       </c>
       <c r="C5">
-        <v>1488</v>
+        <v>1494</v>
       </c>
       <c r="D5">
         <v>99.5</v>
@@ -2135,16 +2161,16 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B6">
-        <v>1425</v>
+        <v>1444</v>
       </c>
       <c r="C6">
-        <v>1340</v>
+        <v>1359</v>
       </c>
       <c r="D6">
-        <v>94</v>
+        <v>94.09999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2159,19 +2185,19 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
@@ -2180,41 +2206,41 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B2">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E2">
         <v>10254</v>
       </c>
       <c r="F2">
-        <v>2720.9</v>
+        <v>2750.1</v>
       </c>
       <c r="G2">
         <v>39</v>
       </c>
       <c r="H2">
-        <v>955.7</v>
+        <v>946</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B3">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -2226,7 +2252,7 @@
         <v>42663</v>
       </c>
       <c r="F3">
-        <v>630.5</v>
+        <v>628.2</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2237,33 +2263,33 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B4">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E4">
         <v>58201</v>
       </c>
       <c r="F4">
-        <v>163.2</v>
+        <v>168.4</v>
       </c>
       <c r="G4">
         <v>1.7</v>
       </c>
       <c r="H4">
-        <v>39.5</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B5">
         <v>34</v>
@@ -2289,7 +2315,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B6">
         <v>9</v>
@@ -2315,7 +2341,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B7">
         <v>21</v>
@@ -2341,7 +2367,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B8">
         <v>32</v>
@@ -2367,7 +2393,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B9">
         <v>49</v>
@@ -2393,7 +2419,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B10">
         <v>84</v>
@@ -2419,13 +2445,13 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B11">
         <v>144</v>
       </c>
       <c r="C11">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D11">
         <v>58</v>
@@ -2437,7 +2463,7 @@
         <v>158.1</v>
       </c>
       <c r="G11">
-        <v>16.5</v>
+        <v>17.6</v>
       </c>
       <c r="H11">
         <v>63.7</v>
@@ -2445,7 +2471,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B12">
         <v>194</v>
@@ -2471,13 +2497,13 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B13">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C13">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D13">
         <v>75</v>
@@ -2486,10 +2512,10 @@
         <v>23417</v>
       </c>
       <c r="F13">
-        <v>1298.2</v>
+        <v>1306.7</v>
       </c>
       <c r="G13">
-        <v>217.8</v>
+        <v>226.3</v>
       </c>
       <c r="H13">
         <v>320.3</v>
@@ -2502,7 +2528,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
@@ -2510,93 +2536,93 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E2" t="s">
         <v>117</v>
       </c>
-      <c r="D2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>119</v>
-      </c>
-      <c r="F2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" t="s">
         <v>121</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E3" t="s">
         <v>122</v>
       </c>
-      <c r="D3" t="s">
-        <v>118</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>123</v>
-      </c>
-      <c r="F3" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" t="s">
         <v>125</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E4" t="s">
         <v>126</v>
       </c>
-      <c r="D4" t="s">
-        <v>118</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>127</v>
-      </c>
-      <c r="F4" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C5" t="s">
         <v>129</v>
       </c>
       <c r="D5" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="E5" t="s">
         <v>130</v>
@@ -2607,139 +2633,139 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
         <v>132</v>
       </c>
       <c r="C6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D6" t="s">
         <v>133</v>
       </c>
-      <c r="D6" t="s">
-        <v>118</v>
-      </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F6" t="s">
-        <v>134</v>
+        <v>117</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C7" t="s">
         <v>135</v>
       </c>
       <c r="D7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" t="s">
         <v>136</v>
       </c>
-      <c r="E7" t="s">
-        <v>137</v>
-      </c>
       <c r="F7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D8" t="s">
         <v>138</v>
       </c>
-      <c r="C8" t="s">
-        <v>138</v>
-      </c>
-      <c r="D8" t="s">
-        <v>131</v>
-      </c>
       <c r="E8" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="F8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>139</v>
+        <v>118</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="D9" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="E9" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="F9" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
         <v>140</v>
       </c>
       <c r="C10" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="F10" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
+        <v>141</v>
+      </c>
+      <c r="C11" t="s">
+        <v>142</v>
+      </c>
+      <c r="D11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E11" t="s">
         <v>143</v>
       </c>
-      <c r="C11" t="s">
-        <v>144</v>
-      </c>
-      <c r="D11" t="s">
-        <v>131</v>
-      </c>
-      <c r="E11" t="s">
-        <v>142</v>
-      </c>
       <c r="F11" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="C12" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="D12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="F12" t="s">
         <v>146</v>
@@ -2747,342 +2773,362 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
+        <v>132</v>
+      </c>
+      <c r="C13" t="s">
+        <v>132</v>
+      </c>
+      <c r="D13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" t="s">
+        <v>133</v>
+      </c>
+      <c r="F13" t="s">
         <v>147</v>
-      </c>
-      <c r="C13" t="s">
-        <v>148</v>
-      </c>
-      <c r="D13" t="s">
-        <v>130</v>
-      </c>
-      <c r="E13" t="s">
-        <v>149</v>
-      </c>
-      <c r="F13" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C14" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E14" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
       <c r="F14" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C15" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D15" t="s">
-        <v>157</v>
+        <v>117</v>
       </c>
       <c r="E15" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F15" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C16" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D16" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E16" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="F16" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>129</v>
+        <v>160</v>
       </c>
       <c r="C17" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="D17" t="s">
-        <v>118</v>
+        <v>162</v>
       </c>
       <c r="E17" t="s">
-        <v>130</v>
+        <v>163</v>
       </c>
       <c r="F17" t="s">
-        <v>136</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>165</v>
+        <v>132</v>
       </c>
       <c r="C18" t="s">
-        <v>166</v>
+        <v>132</v>
       </c>
       <c r="D18" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E18" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="F18" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C19" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D19" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E19" t="s">
-        <v>169</v>
+        <v>146</v>
       </c>
       <c r="F19" t="s">
-        <v>170</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B20" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C20" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E20" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="F20" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C21" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D21" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E21" t="s">
-        <v>173</v>
+        <v>146</v>
       </c>
       <c r="F21" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B22" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C22" t="s">
-        <v>141</v>
+        <v>172</v>
       </c>
       <c r="D22" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="E22" t="s">
-        <v>142</v>
+        <v>173</v>
       </c>
       <c r="F22" t="s">
-        <v>142</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
       <c r="C23" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="D23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E23" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="F23" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>176</v>
+        <v>140</v>
       </c>
       <c r="C24" t="s">
-        <v>177</v>
+        <v>133</v>
       </c>
       <c r="D24" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>178</v>
+        <v>133</v>
       </c>
       <c r="F24" t="s">
-        <v>179</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C25" t="s">
-        <v>157</v>
+        <v>177</v>
       </c>
       <c r="D25" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E25" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="F25" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B26" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C26" t="s">
-        <v>182</v>
+        <v>157</v>
       </c>
       <c r="D26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E26" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="F26" t="s">
-        <v>123</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C27" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D27" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E27" t="s">
-        <v>123</v>
+        <v>183</v>
       </c>
       <c r="F27" t="s">
-        <v>123</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B28" t="s">
+        <v>184</v>
+      </c>
+      <c r="C28" t="s">
+        <v>185</v>
+      </c>
+      <c r="D28" t="s">
+        <v>119</v>
+      </c>
+      <c r="E28" t="s">
         <v>186</v>
       </c>
-      <c r="C28" t="s">
-        <v>187</v>
-      </c>
-      <c r="D28" t="s">
-        <v>157</v>
-      </c>
-      <c r="E28" t="s">
-        <v>188</v>
-      </c>
       <c r="F28" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" t="s">
+        <v>187</v>
+      </c>
+      <c r="C29" t="s">
+        <v>188</v>
+      </c>
+      <c r="D29" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" t="s">
+        <v>189</v>
+      </c>
+      <c r="F29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
         <v>12</v>
       </c>
-      <c r="B29" t="s">
-        <v>190</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="B30" t="s">
         <v>191</v>
       </c>
-      <c r="D29" t="s">
-        <v>118</v>
-      </c>
-      <c r="E29" t="s">
-        <v>191</v>
-      </c>
-      <c r="F29" t="s">
-        <v>191</v>
+      <c r="C30" t="s">
+        <v>192</v>
+      </c>
+      <c r="D30" t="s">
+        <v>119</v>
+      </c>
+      <c r="E30" t="s">
+        <v>192</v>
+      </c>
+      <c r="F30" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -3097,33 +3143,33 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -3132,21 +3178,21 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1522</v>
+        <v>1528</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C3">
         <v>90</v>
@@ -3155,21 +3201,21 @@
         <v>100</v>
       </c>
       <c r="E3">
-        <v>1327</v>
+        <v>1345</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" t="s">
         <v>202</v>
-      </c>
-      <c r="B4" t="s">
-        <v>201</v>
       </c>
       <c r="C4">
         <v>90</v>
@@ -3178,21 +3224,21 @@
         <v>98.5</v>
       </c>
       <c r="E4">
-        <v>1431</v>
+        <v>1437</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -3201,21 +3247,21 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1531</v>
+        <v>1537</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -3224,21 +3270,21 @@
         <v>99.8</v>
       </c>
       <c r="E6">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -3247,13 +3293,13 @@
         <v>100</v>
       </c>
       <c r="E7">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -3268,7 +3314,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3277,24 +3323,24 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
@@ -3320,13 +3366,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B3" t="s">
         <v>23</v>
       </c>
       <c r="C3">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -3335,7 +3381,7 @@
         <v>5</v>
       </c>
       <c r="F3">
-        <v>36.5</v>
+        <v>36.3</v>
       </c>
       <c r="G3">
         <v>98.2</v>
@@ -3346,7 +3392,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
@@ -3372,13 +3418,13 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
       </c>
       <c r="C5">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -3387,7 +3433,7 @@
         <v>5</v>
       </c>
       <c r="F5">
-        <v>41.5</v>
+        <v>41.6</v>
       </c>
       <c r="G5">
         <v>97.7</v>
@@ -3398,7 +3444,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
@@ -3424,7 +3470,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
@@ -3450,7 +3496,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -3476,65 +3522,65 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
       </c>
       <c r="C9">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E9">
         <v>5</v>
       </c>
       <c r="F9">
-        <v>69</v>
+        <v>66.7</v>
       </c>
       <c r="G9">
-        <v>97.2</v>
+        <v>100</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B10" t="s">
         <v>16</v>
       </c>
       <c r="C10">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10">
         <v>5</v>
       </c>
       <c r="F10">
-        <v>70.59999999999999</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="G10">
-        <v>100</v>
+        <v>97.2</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
       </c>
       <c r="C11">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -3543,7 +3589,7 @@
         <v>2</v>
       </c>
       <c r="F11">
-        <v>72.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G11">
         <v>99</v>
@@ -3554,7 +3600,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
@@ -3580,13 +3626,13 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
       </c>
       <c r="C13">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -3595,7 +3641,7 @@
         <v>2</v>
       </c>
       <c r="F13">
-        <v>86.7</v>
+        <v>86.8</v>
       </c>
       <c r="G13">
         <v>99.3</v>
@@ -3606,7 +3652,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
@@ -3632,7 +3678,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
@@ -3658,7 +3704,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
@@ -3684,7 +3730,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -3710,7 +3756,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
@@ -3736,10 +3782,10 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B19" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -3775,25 +3821,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -3985,16 +4031,16 @@
         <v>46266</v>
       </c>
       <c r="B10">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10">
-        <v>76.2</v>
+        <v>68.5</v>
       </c>
       <c r="F10">
         <v>100</v>
@@ -4015,62 +4061,62 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
       <c r="C2">
-        <v>1508</v>
+        <v>1515</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B3">
-        <v>867</v>
+        <v>880</v>
       </c>
       <c r="C3">
-        <v>1514</v>
+        <v>1521</v>
       </c>
       <c r="D3">
-        <v>57.3</v>
+        <v>57.9</v>
       </c>
       <c r="E3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -4085,24 +4131,24 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B2">
-        <v>1477</v>
+        <v>1495</v>
       </c>
       <c r="C2">
         <v>16</v>
@@ -4113,7 +4159,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B3">
         <v>385</v>
@@ -4127,10 +4173,10 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B4">
-        <v>1522</v>
+        <v>1528</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -4141,24 +4187,24 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B5">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B6">
-        <v>1405</v>
+        <v>1421</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -4169,10 +4215,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B7">
-        <v>1415</v>
+        <v>1432</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -4193,27 +4239,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -4228,64 +4274,64 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3">
-        <v>100</v>
+        <v>44</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>6.8</v>
       </c>
       <c r="F3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="D4">
         <v>4</v>
       </c>
       <c r="E4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C5">
-        <v>294</v>
+        <v>78</v>
       </c>
       <c r="D5">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="F5" t="s">
         <v>248</v>
@@ -4293,47 +4339,47 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C6">
-        <v>79</v>
+        <v>295</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E6">
-        <v>2.5</v>
+        <v>3.4</v>
       </c>
       <c r="F6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="C7">
-        <v>43</v>
+        <v>79</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="F7" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
@@ -4348,18 +4394,18 @@
         <v>1.6</v>
       </c>
       <c r="F8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
       <c r="C9">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -4368,12 +4414,12 @@
         <v>1.5</v>
       </c>
       <c r="F9" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B10" t="s">
         <v>19</v>
@@ -4388,32 +4434,32 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
       </c>
       <c r="C11">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="F11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
@@ -4428,12 +4474,12 @@
         <v>0</v>
       </c>
       <c r="F12" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
@@ -4448,7 +4494,7 @@
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -4468,12 +4514,12 @@
         <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
@@ -4488,12 +4534,12 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
@@ -4508,12 +4554,12 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -4528,12 +4574,12 @@
         <v>0</v>
       </c>
       <c r="F17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B18" t="s">
         <v>23</v>
@@ -4548,15 +4594,15 @@
         <v>0</v>
       </c>
       <c r="F18" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B19" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -4568,7 +4614,7 @@
         <v>16.7</v>
       </c>
       <c r="F19" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -4583,31 +4629,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -4615,7 +4661,7 @@
         <v>411690</v>
       </c>
       <c r="B2">
-        <v>47.17340460873341</v>
+        <v>47.38508409765746</v>
       </c>
       <c r="C2">
         <v>27142</v>
@@ -4627,16 +4673,16 @@
         <v>9</v>
       </c>
       <c r="F2">
-        <v>2.459012678057255</v>
+        <v>2.448027732966176</v>
       </c>
       <c r="G2">
-        <v>2.031929755684155</v>
+        <v>2.022852683006045</v>
       </c>
       <c r="H2">
-        <v>2.94935147531283</v>
+        <v>2.936176080041506</v>
       </c>
       <c r="I2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -4644,28 +4690,28 @@
         <v>410220</v>
       </c>
       <c r="B3">
-        <v>7.075974315720881</v>
+        <v>7.10530453020303</v>
       </c>
       <c r="C3">
         <v>4046</v>
       </c>
       <c r="D3">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
       </c>
       <c r="F3">
-        <v>1.695879530447034</v>
+        <v>1.829618976180396</v>
       </c>
       <c r="G3">
-        <v>0.8762857003234499</v>
+        <v>0.9741950484430553</v>
       </c>
       <c r="H3">
-        <v>2.962360250743992</v>
+        <v>3.128704170758977</v>
       </c>
       <c r="I3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -4673,7 +4719,7 @@
         <v>412360</v>
       </c>
       <c r="B4">
-        <v>3.088664657852097</v>
+        <v>3.10181828849193</v>
       </c>
       <c r="C4">
         <v>1745</v>
@@ -4685,16 +4731,16 @@
         <v>11</v>
       </c>
       <c r="F4">
-        <v>1.618822550803257</v>
+        <v>1.611957740577687</v>
       </c>
       <c r="G4">
-        <v>0.5256272758491746</v>
+        <v>0.5233982906547829</v>
       </c>
       <c r="H4">
-        <v>3.777791820053717</v>
+        <v>3.761771642979022</v>
       </c>
       <c r="I4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -4702,7 +4748,7 @@
         <v>412830</v>
       </c>
       <c r="B5">
-        <v>3.77163137528971</v>
+        <v>3.788441971696381</v>
       </c>
       <c r="C5">
         <v>2106</v>
@@ -4714,16 +4760,16 @@
         <v>12</v>
       </c>
       <c r="F5">
-        <v>1.590823546359729</v>
+        <v>1.583764525054433</v>
       </c>
       <c r="G5">
-        <v>0.5838042041745707</v>
+        <v>0.5812136677666706</v>
       </c>
       <c r="H5">
-        <v>3.462553129682656</v>
+        <v>3.447188612122503</v>
       </c>
       <c r="I5" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -4731,7 +4777,7 @@
         <v>411090</v>
       </c>
       <c r="B6">
-        <v>7.882157468873373</v>
+        <v>7.918213436783874</v>
       </c>
       <c r="C6">
         <v>4530</v>
@@ -4743,16 +4789,16 @@
         <v>14</v>
       </c>
       <c r="F6">
-        <v>1.395556996093897</v>
+        <v>1.389202259805193</v>
       </c>
       <c r="G6">
-        <v>0.6966570242882638</v>
+        <v>0.6934847628289208</v>
       </c>
       <c r="H6">
-        <v>2.497036958602552</v>
+        <v>2.485666580022901</v>
       </c>
       <c r="I6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -4760,7 +4806,7 @@
         <v>411740</v>
       </c>
       <c r="B7">
-        <v>5.801644657208181</v>
+        <v>5.827231889666747</v>
       </c>
       <c r="C7">
         <v>3193</v>
@@ -4772,16 +4818,16 @@
         <v>13</v>
       </c>
       <c r="F7">
-        <v>1.378919336271397</v>
+        <v>1.372864535249774</v>
       </c>
       <c r="G7">
-        <v>0.5953194965943547</v>
+        <v>0.5927054632703183</v>
       </c>
       <c r="H7">
-        <v>2.717020802128675</v>
+        <v>2.705090430354367</v>
       </c>
       <c r="I7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -4789,28 +4835,28 @@
         <v>411520</v>
       </c>
       <c r="B8">
-        <v>702.8120800949052</v>
+        <v>705.9502798612566</v>
       </c>
       <c r="C8">
         <v>429660</v>
       </c>
       <c r="D8">
-        <v>945</v>
+        <v>949</v>
       </c>
       <c r="E8" t="s">
         <v>16</v>
       </c>
       <c r="F8">
-        <v>1.34459840228186</v>
+        <v>1.344287306163418</v>
       </c>
       <c r="G8">
-        <v>1.260225507373135</v>
+        <v>1.260109023961197</v>
       </c>
       <c r="H8">
-        <v>1.433134622212923</v>
+        <v>1.432610311569867</v>
       </c>
       <c r="I8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -4818,7 +4864,7 @@
         <v>411640</v>
       </c>
       <c r="B9">
-        <v>6.014727501602308</v>
+        <v>6.040577057625908</v>
       </c>
       <c r="C9">
         <v>3669</v>
@@ -4830,16 +4876,16 @@
         <v>17</v>
       </c>
       <c r="F9">
-        <v>1.330068568836879</v>
+        <v>1.324376781171995</v>
       </c>
       <c r="G9">
-        <v>0.5742292025413304</v>
+        <v>0.5717718926188056</v>
       </c>
       <c r="H9">
-        <v>2.620765315800931</v>
+        <v>2.609550225055589</v>
       </c>
       <c r="I9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -4847,7 +4893,7 @@
         <v>412530</v>
       </c>
       <c r="B10">
-        <v>9.719069353135639</v>
+        <v>9.760875835952792</v>
       </c>
       <c r="C10">
         <v>5170</v>
@@ -4859,16 +4905,16 @@
         <v>15</v>
       </c>
       <c r="F10">
-        <v>1.234686116950948</v>
+        <v>1.229397873887476</v>
       </c>
       <c r="G10">
-        <v>0.6379803336542443</v>
+        <v>0.6352478212952247</v>
       </c>
       <c r="H10">
-        <v>2.15674817068922</v>
+        <v>2.147510674295021</v>
       </c>
       <c r="I10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -4876,7 +4922,7 @@
         <v>412450</v>
       </c>
       <c r="B11">
-        <v>11.59266493344602</v>
+        <v>11.64930804914038</v>
       </c>
       <c r="C11">
         <v>6463</v>
@@ -4888,16 +4934,16 @@
         <v>18</v>
       </c>
       <c r="F11">
-        <v>1.207660195509367</v>
+        <v>1.201788118310863</v>
       </c>
       <c r="G11">
-        <v>0.6602390667065885</v>
+        <v>0.6570287474598454</v>
       </c>
       <c r="H11">
-        <v>2.026248602602636</v>
+        <v>2.016396254846134</v>
       </c>
       <c r="I11" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -4905,7 +4951,7 @@
         <v>410590</v>
       </c>
       <c r="B12">
-        <v>40.27819798679241</v>
+        <v>40.455990582026</v>
       </c>
       <c r="C12">
         <v>23313</v>
@@ -4917,16 +4963,16 @@
         <v>19</v>
       </c>
       <c r="F12">
-        <v>1.092402396314453</v>
+        <v>1.087601597859491</v>
       </c>
       <c r="G12">
-        <v>0.7937412534847694</v>
+        <v>0.7902529859780106</v>
       </c>
       <c r="H12">
-        <v>1.466499228681399</v>
+        <v>1.460054380835029</v>
       </c>
       <c r="I12" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -4934,7 +4980,7 @@
         <v>411110</v>
       </c>
       <c r="B13">
-        <v>10.61352899729195</v>
+        <v>10.65936448659817</v>
       </c>
       <c r="C13">
         <v>6228</v>
@@ -4946,16 +4992,16 @@
         <v>20</v>
       </c>
       <c r="F13">
-        <v>0.9421936853002909</v>
+        <v>0.9381422328294355</v>
       </c>
       <c r="G13">
-        <v>0.4518184948056375</v>
+        <v>0.4498756658674717</v>
       </c>
       <c r="H13">
-        <v>1.73272773332132</v>
+        <v>1.725276967978686</v>
       </c>
       <c r="I13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -4963,7 +5009,7 @@
         <v>411480</v>
       </c>
       <c r="B14">
-        <v>75.81634682008129</v>
+        <v>76.17178242564367</v>
       </c>
       <c r="C14">
         <v>44749</v>
@@ -4975,16 +5021,16 @@
         <v>22</v>
       </c>
       <c r="F14">
-        <v>0.8573348984256731</v>
+        <v>0.8533343704205795</v>
       </c>
       <c r="G14">
-        <v>0.6616729746723569</v>
+        <v>0.6585854516166045</v>
       </c>
       <c r="H14">
-        <v>1.092743706215186</v>
+        <v>1.087644704871451</v>
       </c>
       <c r="I14" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -4992,7 +5038,7 @@
         <v>410780</v>
       </c>
       <c r="B15">
-        <v>9.495864216988322</v>
+        <v>9.536135539506603</v>
       </c>
       <c r="C15">
         <v>4805</v>
@@ -5004,16 +5050,16 @@
         <v>21</v>
       </c>
       <c r="F15">
-        <v>0.7371630259283655</v>
+        <v>0.7340499692983787</v>
       </c>
       <c r="G15">
-        <v>0.2963777690170533</v>
+        <v>0.2951261587946642</v>
       </c>
       <c r="H15">
-        <v>1.518837573087858</v>
+        <v>1.512423486636874</v>
       </c>
       <c r="I15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -5021,28 +5067,28 @@
         <v>412625</v>
       </c>
       <c r="B16">
-        <v>203.9851658248778</v>
+        <v>205.0170708322734</v>
       </c>
       <c r="C16">
         <v>128106</v>
       </c>
       <c r="D16">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E16" t="s">
         <v>23</v>
       </c>
       <c r="F16">
-        <v>0.6863244169440763</v>
+        <v>0.6877476076875255</v>
       </c>
       <c r="G16">
-        <v>0.5773487045345095</v>
+        <v>0.5789168998976707</v>
       </c>
       <c r="H16">
-        <v>0.8098897276804955</v>
+        <v>0.8110930839475775</v>
       </c>
       <c r="I16" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -5050,7 +5096,7 @@
         <v>411810</v>
       </c>
       <c r="B17">
-        <v>15.88641562521915</v>
+        <v>15.95996617493859</v>
       </c>
       <c r="C17">
         <v>9549</v>
@@ -5062,16 +5108,16 @@
         <v>24</v>
       </c>
       <c r="F17">
-        <v>0.629468612424148</v>
+        <v>0.6265677439656901</v>
       </c>
       <c r="G17">
-        <v>0.3018546668588927</v>
+        <v>0.3004635876774271</v>
       </c>
       <c r="H17">
-        <v>1.157615189975498</v>
+        <v>1.152280389597288</v>
       </c>
       <c r="I17" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -5079,7 +5125,7 @@
         <v>410210</v>
       </c>
       <c r="B18">
-        <v>47.42039187706349</v>
+        <v>47.63556056736902</v>
       </c>
       <c r="C18">
         <v>26203</v>
@@ -5091,16 +5137,16 @@
         <v>26</v>
       </c>
       <c r="F18">
-        <v>0.4006715096167311</v>
+        <v>0.3988616859694362</v>
       </c>
       <c r="G18">
-        <v>0.2412304224314038</v>
+        <v>0.2401407903700153</v>
       </c>
       <c r="H18">
-        <v>0.6256981943233779</v>
+        <v>0.6228719305113105</v>
       </c>
       <c r="I18" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -5108,7 +5154,7 @@
         <v>411360</v>
       </c>
       <c r="B19">
-        <v>7.600136934499216</v>
+        <v>7.633285073459273</v>
       </c>
       <c r="C19">
         <v>4707</v>
@@ -5120,16 +5166,16 @@
         <v>27</v>
       </c>
       <c r="F19">
-        <v>0.3947297299844867</v>
+        <v>0.3930155851811324</v>
       </c>
       <c r="G19">
-        <v>0.0814027600065033</v>
+        <v>0.08104926213835609</v>
       </c>
       <c r="H19">
-        <v>1.153567777173216</v>
+        <v>1.148558318649188</v>
       </c>
       <c r="I19" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -5137,7 +5183,7 @@
         <v>411630</v>
       </c>
       <c r="B20">
-        <v>7.846553373876229</v>
+        <v>7.882784676284354</v>
       </c>
       <c r="C20">
         <v>4057</v>
@@ -5149,16 +5195,16 @@
         <v>25</v>
       </c>
       <c r="F20">
-        <v>0.3823334726796089</v>
+        <v>0.3805761698687026</v>
       </c>
       <c r="G20">
-        <v>0.07884635373224701</v>
+        <v>0.07848395564538241</v>
       </c>
       <c r="H20">
-        <v>1.117340652894999</v>
+        <v>1.112205068358519</v>
       </c>
       <c r="I20" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -5166,7 +5212,7 @@
         <v>410790</v>
       </c>
       <c r="B21">
-        <v>19.93317023758988</v>
+        <v>20.03494509019059</v>
       </c>
       <c r="C21">
         <v>11522</v>
@@ -5178,16 +5224,16 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>0.3511734418842935</v>
+        <v>0.3493895275723667</v>
       </c>
       <c r="G21">
-        <v>0.1411899370734592</v>
+        <v>0.1404727109982358</v>
       </c>
       <c r="H21">
-        <v>0.7235515068498317</v>
+        <v>0.7198759615649725</v>
       </c>
       <c r="I21" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -5195,7 +5241,7 @@
         <v>411410</v>
       </c>
       <c r="B22">
-        <v>58.9758919548884</v>
+        <v>59.27647461376149</v>
       </c>
       <c r="C22">
         <v>34521</v>
@@ -5207,16 +5253,16 @@
         <v>29</v>
       </c>
       <c r="F22">
-        <v>0.3052094576843108</v>
+        <v>0.303661783486381</v>
       </c>
       <c r="G22">
-        <v>0.1808864677885602</v>
+        <v>0.1799692179724009</v>
       </c>
       <c r="H22">
-        <v>0.4823625268658613</v>
+        <v>0.4799165343905864</v>
       </c>
       <c r="I22" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -5224,7 +5270,7 @@
         <v>411750</v>
       </c>
       <c r="B23">
-        <v>79.35135855529957</v>
+        <v>79.74180237038844</v>
       </c>
       <c r="C23">
         <v>48695</v>
@@ -5236,16 +5282,16 @@
         <v>30</v>
       </c>
       <c r="F23">
-        <v>0.3024522886180269</v>
+        <v>0.3009713761989437</v>
       </c>
       <c r="G23">
-        <v>0.1937868882732503</v>
+        <v>0.1928380397430883</v>
       </c>
       <c r="H23">
-        <v>0.4500250310001563</v>
+        <v>0.4478215507079371</v>
       </c>
       <c r="I23" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -5253,7 +5299,7 @@
         <v>412040</v>
       </c>
       <c r="B24">
-        <v>7.013238548555828</v>
+        <v>7.044833660150949</v>
       </c>
       <c r="C24">
         <v>4304</v>
@@ -5265,16 +5311,16 @@
         <v>31</v>
       </c>
       <c r="F24">
-        <v>0.2851749567839585</v>
+        <v>0.283895986261959</v>
       </c>
       <c r="G24">
-        <v>0.03453601027072448</v>
+        <v>0.03438112100701823</v>
       </c>
       <c r="H24">
-        <v>1.030149996710389</v>
+        <v>1.025529915431553</v>
       </c>
       <c r="I24" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -5282,7 +5328,7 @@
         <v>412340</v>
       </c>
       <c r="B25">
-        <v>20.37211620262686</v>
+        <v>20.46290725620743</v>
       </c>
       <c r="C25">
         <v>11730</v>
@@ -5294,16 +5340,16 @@
         <v>32</v>
       </c>
       <c r="F25">
-        <v>0.245433510700046</v>
+        <v>0.2443445565870533</v>
       </c>
       <c r="G25">
-        <v>0.07969159286010168</v>
+        <v>0.07933801242372027</v>
       </c>
       <c r="H25">
-        <v>0.5727599412484259</v>
+        <v>0.5702186856065173</v>
       </c>
       <c r="I25" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -5311,7 +5357,7 @@
         <v>411420</v>
       </c>
       <c r="B26">
-        <v>66.84912943328723</v>
+        <v>67.15768140095651</v>
       </c>
       <c r="C26">
         <v>38313</v>
@@ -5323,16 +5369,16 @@
         <v>33</v>
       </c>
       <c r="F26">
-        <v>0.2243858690032666</v>
+        <v>0.2233549414912701</v>
       </c>
       <c r="G26">
-        <v>0.1255870675348371</v>
+        <v>0.1250100652322958</v>
       </c>
       <c r="H26">
-        <v>0.370090367387291</v>
+        <v>0.3683900092347958</v>
       </c>
       <c r="I26" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -5340,7 +5386,7 @@
         <v>411000</v>
       </c>
       <c r="B27">
-        <v>9.364617544753736</v>
+        <v>9.409137117451714</v>
       </c>
       <c r="C27">
         <v>5693</v>
@@ -5352,16 +5398,16 @@
         <v>35</v>
       </c>
       <c r="F27">
-        <v>0.2135698538079052</v>
+        <v>0.2125593425873745</v>
       </c>
       <c r="G27">
-        <v>0.02586430010477639</v>
+        <v>0.02574192250793372</v>
       </c>
       <c r="H27">
-        <v>0.7714877445017908</v>
+        <v>0.7678374305252582</v>
       </c>
       <c r="I27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -5369,7 +5415,7 @@
         <v>410810</v>
       </c>
       <c r="B28">
-        <v>4.896886753566739</v>
+        <v>4.919571245722143</v>
       </c>
       <c r="C28">
         <v>2711</v>
@@ -5381,74 +5427,74 @@
         <v>34</v>
       </c>
       <c r="F28">
-        <v>0.2042113796631362</v>
+        <v>0.2032697464986525</v>
       </c>
       <c r="G28">
-        <v>0.005170184498518202</v>
+        <v>0.005146344410868163</v>
       </c>
       <c r="H28">
-        <v>1.137792983854627</v>
+        <v>1.132546539657043</v>
       </c>
       <c r="I28" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29">
-        <v>410730</v>
+        <v>410115</v>
       </c>
       <c r="B29">
-        <v>12.53112036852488</v>
+        <v>6.067772497579909</v>
       </c>
       <c r="C29">
-        <v>6517</v>
+        <v>3357</v>
       </c>
       <c r="D29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F29">
-        <v>0.1596026485407891</v>
+        <v>0.1648051241866506</v>
       </c>
       <c r="G29">
-        <v>0.01932862117838526</v>
+        <v>0.004172504488984667</v>
       </c>
       <c r="H29">
-        <v>0.57653964332436</v>
+        <v>0.9182353809674164</v>
       </c>
       <c r="I29" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30">
-        <v>410115</v>
+        <v>410730</v>
       </c>
       <c r="B30">
-        <v>6.039275026784384</v>
+        <v>12.58712092416635</v>
       </c>
       <c r="C30">
-        <v>3357</v>
+        <v>6517</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E30" t="s">
+        <v>36</v>
+      </c>
+      <c r="F30">
+        <v>0.1588925705925449</v>
+      </c>
+      <c r="G30">
+        <v>0.01924262744460815</v>
+      </c>
+      <c r="H30">
+        <v>0.5739745976264586</v>
+      </c>
+      <c r="I30" t="s">
         <v>265</v>
-      </c>
-      <c r="F30">
-        <v>0</v>
-      </c>
-      <c r="G30">
-        <v>0</v>
-      </c>
-      <c r="H30">
-        <v>0.6108149467864328</v>
-      </c>
-      <c r="I30" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -5456,7 +5502,7 @@
         <v>411160</v>
       </c>
       <c r="B31">
-        <v>4.798574750665755</v>
+        <v>4.81867844685021</v>
       </c>
       <c r="C31">
         <v>2685</v>
@@ -5474,10 +5520,10 @@
         <v>0</v>
       </c>
       <c r="H31">
-        <v>0.7687448139892246</v>
+        <v>0.7655375835516101</v>
       </c>
       <c r="I31" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -5492,167 +5538,167 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B2">
-        <v>59.9</v>
+        <v>60</v>
       </c>
       <c r="C2">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B3">
-        <v>60.4</v>
+        <v>60.5</v>
       </c>
       <c r="C3">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4">
-        <v>60.4</v>
+        <v>60.5</v>
       </c>
       <c r="C4">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B5">
-        <v>60.5</v>
+        <v>60.6</v>
       </c>
       <c r="C5">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B6">
-        <v>92.09999999999999</v>
+        <v>92.8</v>
       </c>
       <c r="C6">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B7">
-        <v>95.5</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="C7">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8">
-        <v>98.7</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="C8">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9">
-        <v>98.7</v>
+        <v>98.8</v>
       </c>
       <c r="C9">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10">
         <v>99.09999999999999</v>
       </c>
       <c r="C10">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11">
         <v>99.90000000000001</v>
       </c>
       <c r="C11">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12">
         <v>100</v>
       </c>
       <c r="C12">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B13">
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B14">
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B15">
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1514</v>
+        <v>1521</v>
       </c>
     </row>
   </sheetData>
@@ -5667,13 +5713,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -5681,10 +5727,10 @@
         <v>267</v>
       </c>
       <c r="B2">
-        <v>1467</v>
+        <v>1473</v>
       </c>
       <c r="C2">
-        <v>96.90000000000001</v>
+        <v>96.8</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5692,10 +5738,10 @@
         <v>268</v>
       </c>
       <c r="B3">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5738,13 +5784,13 @@
         <v>272</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -5786,7 +5832,7 @@
         <v>273</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -5800,7 +5846,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B5" t="s">
         <v>274</v>
@@ -5817,7 +5863,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
         <v>275</v>
@@ -5834,10 +5880,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -5864,15 +5910,15 @@
         <v>276</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -5886,10 +5932,10 @@
         <v>275</v>
       </c>
       <c r="B3">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="C3">
-        <v>41.8</v>
+        <v>41.9</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5897,10 +5943,10 @@
         <v>274</v>
       </c>
       <c r="B4">
-        <v>879</v>
+        <v>882</v>
       </c>
       <c r="C4">
-        <v>58.1</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -5915,54 +5961,54 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C2">
-        <v>30.1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B3">
         <v>228</v>
       </c>
       <c r="C3">
-        <v>15.1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B4">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C4">
-        <v>12.6</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B5">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C5">
         <v>11.8</v>
@@ -5970,10 +6016,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B6">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C6">
         <v>10.8</v>
@@ -5981,18 +6027,18 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B7">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8">
         <v>38</v>
@@ -6003,7 +6049,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9">
         <v>29</v>
@@ -6014,7 +6060,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B10">
         <v>16</v>
@@ -6025,7 +6071,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -6046,7 +6092,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -6055,7 +6101,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>7</v>
@@ -6063,13 +6109,13 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2">
         <v>148</v>
       </c>
       <c r="C2">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -6080,13 +6126,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B3">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C3">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -6097,7 +6143,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B4">
         <v>34</v>
@@ -6114,7 +6160,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <v>9</v>
@@ -6131,7 +6177,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B6">
         <v>21</v>
@@ -6148,7 +6194,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7">
         <v>32</v>
@@ -6165,30 +6211,30 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8">
         <v>49</v>
       </c>
       <c r="C8">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D8">
         <v>2</v>
       </c>
       <c r="E8">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B9">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C9">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -6199,7 +6245,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B10">
         <v>84</v>
@@ -6216,10 +6262,10 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C11">
         <v>119</v>
@@ -6233,19 +6279,19 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="C12">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="D12">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E12">
-        <v>15.2</v>
+        <v>15.5</v>
       </c>
     </row>
   </sheetData>
@@ -6260,7 +6306,7 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -6274,7 +6320,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2">
         <v>148</v>
@@ -6288,10 +6334,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B3">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C3">
         <v>58</v>
@@ -6302,7 +6348,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B4">
         <v>34</v>
@@ -6316,7 +6362,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <v>9</v>
@@ -6330,7 +6376,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B6">
         <v>21</v>
@@ -6344,7 +6390,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7">
         <v>32</v>
@@ -6358,7 +6404,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B8">
         <v>49</v>
@@ -6372,21 +6418,21 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B9">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C9">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D9">
-        <v>24.2</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B10">
         <v>84</v>
@@ -6400,30 +6446,30 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B11">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C11">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11">
-        <v>25.2</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="C12">
         <v>189</v>
       </c>
       <c r="D12">
-        <v>29.4</v>
+        <v>29.3</v>
       </c>
     </row>
   </sheetData>
@@ -6438,46 +6484,46 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B2">
-        <v>858</v>
+        <v>877</v>
       </c>
       <c r="C2">
-        <v>98.59999999999999</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B4">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C4">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -6492,32 +6538,32 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B2">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B3">
-        <v>1120</v>
+        <v>1126</v>
       </c>
       <c r="C3">
         <v>74</v>
@@ -6525,13 +6571,13 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4">
         <v>374</v>
       </c>
       <c r="C4">
-        <v>24.7</v>
+        <v>24.6</v>
       </c>
     </row>
   </sheetData>
@@ -6546,18 +6592,18 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -6568,7 +6614,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B3">
         <v>94</v>
@@ -6579,7 +6625,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4">
         <v>277</v>
@@ -6600,33 +6646,33 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B2">
         <v>57</v>
@@ -6652,7 +6698,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B3">
         <v>291</v>

</xml_diff>

<commit_message>
Atualização de dados — 18/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -529,7 +529,7 @@
     <t xml:space="preserve"> 99,7% (944)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 92,6% (910)</t>
+    <t xml:space="preserve"> 92,6% (911)</t>
   </si>
   <si>
     <t xml:space="preserve"> 25,0% (8)</t>
@@ -1455,7 +1455,7 @@
         <v>949</v>
       </c>
       <c r="C9">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="D9">
         <v>80</v>
@@ -1470,7 +1470,7 @@
         <v>18.6</v>
       </c>
       <c r="H9">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="I9">
         <v>29.6</v>
@@ -2164,10 +2164,10 @@
         <v>101</v>
       </c>
       <c r="B6">
-        <v>1444</v>
+        <v>1445</v>
       </c>
       <c r="C6">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="D6">
         <v>94.09999999999999</v>
@@ -3178,7 +3178,7 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -3201,7 +3201,7 @@
         <v>100</v>
       </c>
       <c r="E3">
-        <v>1345</v>
+        <v>1350</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -3224,7 +3224,7 @@
         <v>98.5</v>
       </c>
       <c r="E4">
-        <v>1437</v>
+        <v>1438</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -3247,7 +3247,7 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1537</v>
+        <v>1538</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -3270,7 +3270,7 @@
         <v>99.8</v>
       </c>
       <c r="E6">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
@@ -3424,7 +3424,7 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -3433,7 +3433,7 @@
         <v>5</v>
       </c>
       <c r="F5">
-        <v>41.6</v>
+        <v>41.8</v>
       </c>
       <c r="G5">
         <v>97.7</v>
@@ -3554,7 +3554,7 @@
         <v>16</v>
       </c>
       <c r="C10">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -3563,10 +3563,10 @@
         <v>5</v>
       </c>
       <c r="F10">
-        <v>69.40000000000001</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="G10">
-        <v>97.2</v>
+        <v>97.3</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -3580,7 +3580,7 @@
         <v>19</v>
       </c>
       <c r="C11">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -3589,7 +3589,7 @@
         <v>2</v>
       </c>
       <c r="F11">
-        <v>71.40000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="G11">
         <v>99</v>
@@ -3658,7 +3658,7 @@
         <v>16</v>
       </c>
       <c r="C14">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -3667,10 +3667,10 @@
         <v>4</v>
       </c>
       <c r="F14">
-        <v>88</v>
+        <v>88.5</v>
       </c>
       <c r="G14">
-        <v>90</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="H14">
         <v>4</v>
@@ -3684,7 +3684,7 @@
         <v>16</v>
       </c>
       <c r="C15">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -4031,16 +4031,16 @@
         <v>46266</v>
       </c>
       <c r="B10">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>68.5</v>
+        <v>71.7</v>
       </c>
       <c r="F10">
         <v>100</v>
@@ -4148,7 +4148,7 @@
         <v>248</v>
       </c>
       <c r="B2">
-        <v>1495</v>
+        <v>1496</v>
       </c>
       <c r="C2">
         <v>16</v>
@@ -4176,7 +4176,7 @@
         <v>250</v>
       </c>
       <c r="B4">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -4190,7 +4190,7 @@
         <v>251</v>
       </c>
       <c r="B5">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -4204,7 +4204,7 @@
         <v>252</v>
       </c>
       <c r="B6">
-        <v>1421</v>
+        <v>1422</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -4218,7 +4218,7 @@
         <v>253</v>
       </c>
       <c r="B7">
-        <v>1432</v>
+        <v>1433</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -4279,19 +4279,19 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E3">
-        <v>6.8</v>
+        <v>5.1</v>
       </c>
       <c r="F3" t="s">
         <v>248</v>
@@ -4299,19 +4299,19 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4">
-        <v>101</v>
+        <v>44</v>
       </c>
       <c r="D4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="F4" t="s">
         <v>248</v>
@@ -4319,19 +4319,19 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
       </c>
       <c r="C5">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="F5" t="s">
         <v>248</v>
@@ -5596,7 +5596,7 @@
         <v>45</v>
       </c>
       <c r="B6">
-        <v>92.8</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="C6">
         <v>1521</v>
@@ -5801,13 +5801,13 @@
         <v>274</v>
       </c>
       <c r="C2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D2">
         <v>373</v>
       </c>
       <c r="E2">
-        <v>40.2</v>
+        <v>40.5</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -5818,13 +5818,13 @@
         <v>275</v>
       </c>
       <c r="C3">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D3">
         <v>373</v>
       </c>
       <c r="E3">
-        <v>59.2</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -5932,10 +5932,10 @@
         <v>275</v>
       </c>
       <c r="B3">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="C3">
-        <v>41.9</v>
+        <v>41.8</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5943,10 +5943,10 @@
         <v>274</v>
       </c>
       <c r="B4">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="C4">
-        <v>58</v>
+        <v>58.1</v>
       </c>
     </row>
   </sheetData>
@@ -6115,13 +6115,13 @@
         <v>148</v>
       </c>
       <c r="C2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D2">
         <v>4</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="3" spans="1:5">

</xml_diff>

<commit_message>
Atualização de dados — 25/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="278">
   <si>
     <t>municipio</t>
   </si>
@@ -100,27 +100,27 @@
     <t>Itambe</t>
   </si>
   <si>
+    <t>Marialva</t>
+  </si>
+  <si>
     <t>Florai</t>
   </si>
   <si>
-    <t>Marialva</t>
+    <t>Paranacity</t>
   </si>
   <si>
     <t>Sarandi</t>
   </si>
   <si>
-    <t>Paranacity</t>
+    <t>Lobato</t>
+  </si>
+  <si>
+    <t>Astorga</t>
   </si>
   <si>
     <t>Munhoz De Melo</t>
   </si>
   <si>
-    <t>Astorga</t>
-  </si>
-  <si>
-    <t>Lobato</t>
-  </si>
-  <si>
     <t>Floresta</t>
   </si>
   <si>
@@ -178,12 +178,12 @@
     <t>Critério Confirmação</t>
   </si>
   <si>
+    <t>Raça/Cor</t>
+  </si>
+  <si>
     <t>Antiviral</t>
   </si>
   <si>
-    <t>Raça/Cor</t>
-  </si>
-  <si>
     <t>Data Internação</t>
   </si>
   <si>
@@ -397,13 +397,13 @@
     <t>—</t>
   </si>
   <si>
-    <t xml:space="preserve"> 47,4% (19)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 78,9% (19)</t>
-  </si>
-  <si>
-    <t>100,0% (19)</t>
+    <t xml:space="preserve"> 50,0% (20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 80,0% (20)</t>
+  </si>
+  <si>
+    <t>100,0% (20)</t>
   </si>
   <si>
     <t>100,0% (18)</t>
@@ -430,9 +430,6 @@
     <t>100,0% (42)</t>
   </si>
   <si>
-    <t>100,0% (41)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 50,0% (2)</t>
   </si>
   <si>
@@ -478,13 +475,16 @@
     <t>100,0% (8)</t>
   </si>
   <si>
+    <t xml:space="preserve"> 33,3% (3)</t>
+  </si>
+  <si>
     <t>100,0% (3)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 27,8% (18)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 66,7% (18)</t>
+    <t xml:space="preserve"> 25,0% (20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 60,0% (20)</t>
   </si>
   <si>
     <t xml:space="preserve"> 83,3% (18)</t>
@@ -502,34 +502,34 @@
     <t xml:space="preserve"> 92,9% (14)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 26,2% (65)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 56,9% (65)</t>
+    <t xml:space="preserve"> 25,8% (66)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 57,6% (66)</t>
   </si>
   <si>
     <t>100,0% (4)</t>
   </si>
   <si>
-    <t>100,0% (65)</t>
+    <t>100,0% (66)</t>
   </si>
   <si>
     <t>100,0% (64)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 30,2% (945)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 76,5% (942)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 98,0% (347)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 99,7% (944)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,6% (911)</t>
+    <t xml:space="preserve"> 30,1% (965)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 76,3% (962)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 97,7% (347)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 99,7% (962)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,9% (938)</t>
   </si>
   <si>
     <t xml:space="preserve"> 25,0% (8)</t>
@@ -538,31 +538,34 @@
     <t xml:space="preserve"> 87,5% (8)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 25,9% (116)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,2% (116)</t>
-  </si>
-  <si>
-    <t>100,0% (114)</t>
-  </si>
-  <si>
-    <t>100,0% (109)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 37,5% (24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 75,0% (24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 95,8% (24)</t>
+    <t xml:space="preserve"> 26,5% (117)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,3% (117)</t>
+  </si>
+  <si>
+    <t>100,0% (117)</t>
+  </si>
+  <si>
+    <t>100,0% (111)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 36,0% (25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 72,0% (25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 96,0% (25)</t>
   </si>
   <si>
     <t xml:space="preserve"> 82,6% (23)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 50,0% (10)</t>
+    <t xml:space="preserve"> 45,5% (11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 81,8% (11)</t>
   </si>
   <si>
     <t xml:space="preserve"> 20,0% (5)</t>
@@ -598,16 +601,16 @@
     <t>100,0% (12)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 25,0% (136)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 67,6% (136)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 99,3% (136)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 93,8% (130)</t>
+    <t xml:space="preserve"> 24,8% (141)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 68,1% (141)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 99,3% (141)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 94,0% (133)</t>
   </si>
   <si>
     <t xml:space="preserve">  0,0% (6)</t>
@@ -691,12 +694,12 @@
     <t>HOSPITAL REGIONAL CRISTO REI</t>
   </si>
   <si>
+    <t>HOSP MUN E REG SAGRADO CORACAO DE JESUS NOVA ESPERANCA</t>
+  </si>
+  <si>
     <t>HOSPITAL MEMORIAL UNINGA</t>
   </si>
   <si>
-    <t>HOSP MUN E REG SAGRADO CORACAO DE JESUS NOVA ESPERANCA</t>
-  </si>
-  <si>
     <t>HOSPITAL E MATERNIDADE SAO MARCOS</t>
   </si>
   <si>
@@ -781,16 +784,16 @@
     <t>inconsistentes</t>
   </si>
   <si>
+    <t>Antiviral informado sem data de início</t>
+  </si>
+  <si>
     <t>Classificação final informada sem data de encerramento</t>
   </si>
   <si>
-    <t>Antiviral informado sem data de início</t>
+    <t>Internação em UTI informada sem data de entrada</t>
   </si>
   <si>
     <t>Internação mais de 30 dias após o início dos sintomas</t>
-  </si>
-  <si>
-    <t>Internação em UTI informada sem data de entrada</t>
   </si>
   <si>
     <t>Evolução mais de 120 dias após a internação</t>
@@ -1249,28 +1252,28 @@
         <v>9</v>
       </c>
       <c r="B2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C2">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D2">
         <v>12</v>
       </c>
       <c r="E2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F2">
-        <v>427.4</v>
+        <v>431.1</v>
       </c>
       <c r="G2">
         <v>44.2</v>
       </c>
       <c r="H2">
-        <v>11</v>
+        <v>10.8</v>
       </c>
       <c r="I2">
-        <v>5.2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1452,28 +1455,28 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>949</v>
+        <v>967</v>
       </c>
       <c r="C9">
-        <v>875</v>
+        <v>877</v>
       </c>
       <c r="D9">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E9">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="F9">
-        <v>220.9</v>
+        <v>225.1</v>
       </c>
       <c r="G9">
-        <v>18.6</v>
+        <v>17.7</v>
       </c>
       <c r="H9">
-        <v>9.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I9">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1542,7 +1545,7 @@
         <v>44</v>
       </c>
       <c r="C12">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -1597,28 +1600,28 @@
         <v>21</v>
       </c>
       <c r="B14">
-        <v>7</v>
+        <v>66</v>
       </c>
       <c r="C14">
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F14">
-        <v>145.7</v>
+        <v>147.5</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="I14">
-        <v>28.6</v>
+        <v>45.5</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1626,28 +1629,28 @@
         <v>22</v>
       </c>
       <c r="B15">
-        <v>65</v>
+        <v>7</v>
       </c>
       <c r="C15">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
         <v>2</v>
       </c>
-      <c r="E15">
-        <v>30</v>
-      </c>
       <c r="F15">
-        <v>145.3</v>
+        <v>145.7</v>
       </c>
       <c r="G15">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>3.1</v>
+        <v>0</v>
       </c>
       <c r="I15">
-        <v>46.2</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1655,28 +1658,28 @@
         <v>23</v>
       </c>
       <c r="B16">
-        <v>141</v>
+        <v>11</v>
       </c>
       <c r="C16">
-        <v>133</v>
+        <v>10</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="F16">
-        <v>110.1</v>
+        <v>115.2</v>
       </c>
       <c r="G16">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>39.7</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1684,28 +1687,28 @@
         <v>24</v>
       </c>
       <c r="B17">
+        <v>145</v>
+      </c>
+      <c r="C17">
+        <v>136</v>
+      </c>
+      <c r="D17">
         <v>10</v>
       </c>
-      <c r="C17">
-        <v>10</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
       <c r="E17">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="F17">
-        <v>104.7</v>
+        <v>113.2</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="I17">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1713,7 +1716,7 @@
         <v>25</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18">
         <v>3</v>
@@ -1722,10 +1725,10 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18">
-        <v>73.90000000000001</v>
+        <v>85</v>
       </c>
       <c r="G18">
         <v>0</v>
@@ -1734,7 +1737,7 @@
         <v>0</v>
       </c>
       <c r="I18">
-        <v>33.3</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1742,7 +1745,7 @@
         <v>26</v>
       </c>
       <c r="B19">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C19">
         <v>18</v>
@@ -1754,7 +1757,7 @@
         <v>5</v>
       </c>
       <c r="F19">
-        <v>72.5</v>
+        <v>76.3</v>
       </c>
       <c r="G19">
         <v>3.8</v>
@@ -1763,7 +1766,7 @@
         <v>5.6</v>
       </c>
       <c r="I19">
-        <v>26.3</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1783,7 +1786,7 @@
         <v>1</v>
       </c>
       <c r="F20">
-        <v>63.7</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -1829,7 +1832,7 @@
         <v>29</v>
       </c>
       <c r="B22">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C22">
         <v>17</v>
@@ -1838,10 +1841,10 @@
         <v>1</v>
       </c>
       <c r="E22">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F22">
-        <v>52.1</v>
+        <v>57.9</v>
       </c>
       <c r="G22">
         <v>2.9</v>
@@ -1850,7 +1853,7 @@
         <v>5.9</v>
       </c>
       <c r="I22">
-        <v>44.4</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1858,7 +1861,7 @@
         <v>30</v>
       </c>
       <c r="B23">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C23">
         <v>24</v>
@@ -1867,10 +1870,10 @@
         <v>1</v>
       </c>
       <c r="E23">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F23">
-        <v>49.3</v>
+        <v>51.3</v>
       </c>
       <c r="G23">
         <v>2.1</v>
@@ -1879,7 +1882,7 @@
         <v>4.2</v>
       </c>
       <c r="I23">
-        <v>62.5</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1977,7 +1980,7 @@
         <v>1</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1989,6 +1992,9 @@
         <v>36.9</v>
       </c>
       <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
         <v>0</v>
       </c>
       <c r="I27">
@@ -2108,13 +2114,13 @@
         <v>97</v>
       </c>
       <c r="B2">
-        <v>1507</v>
+        <v>1540</v>
       </c>
       <c r="C2">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="D2">
-        <v>29.1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2122,13 +2128,13 @@
         <v>98</v>
       </c>
       <c r="B3">
-        <v>1504</v>
+        <v>1537</v>
       </c>
       <c r="C3">
-        <v>1151</v>
+        <v>1172</v>
       </c>
       <c r="D3">
-        <v>76.5</v>
+        <v>76.3</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2139,10 +2145,10 @@
         <v>370</v>
       </c>
       <c r="C4">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D4">
-        <v>97.8</v>
+        <v>97.59999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2150,10 +2156,10 @@
         <v>100</v>
       </c>
       <c r="B5">
-        <v>1502</v>
+        <v>1536</v>
       </c>
       <c r="C5">
-        <v>1494</v>
+        <v>1528</v>
       </c>
       <c r="D5">
         <v>99.5</v>
@@ -2164,13 +2170,13 @@
         <v>101</v>
       </c>
       <c r="B6">
-        <v>1445</v>
+        <v>1478</v>
       </c>
       <c r="C6">
-        <v>1360</v>
+        <v>1393</v>
       </c>
       <c r="D6">
-        <v>94.09999999999999</v>
+        <v>94.2</v>
       </c>
     </row>
   </sheetData>
@@ -2214,25 +2220,25 @@
         <v>105</v>
       </c>
       <c r="B2">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="E2">
         <v>10254</v>
       </c>
       <c r="F2">
-        <v>2750.1</v>
+        <v>2789.2</v>
       </c>
       <c r="G2">
         <v>39</v>
       </c>
       <c r="H2">
-        <v>946</v>
+        <v>994.7</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2240,7 +2246,7 @@
         <v>106</v>
       </c>
       <c r="B3">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -2252,7 +2258,7 @@
         <v>42663</v>
       </c>
       <c r="F3">
-        <v>628.2</v>
+        <v>637.6</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2266,25 +2272,25 @@
         <v>107</v>
       </c>
       <c r="B4">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4">
         <v>58201</v>
       </c>
       <c r="F4">
-        <v>168.4</v>
+        <v>182.1</v>
       </c>
       <c r="G4">
         <v>1.7</v>
       </c>
       <c r="H4">
-        <v>43</v>
+        <v>44.7</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2370,7 +2376,7 @@
         <v>111</v>
       </c>
       <c r="B8">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -2382,7 +2388,7 @@
         <v>139537</v>
       </c>
       <c r="F8">
-        <v>22.9</v>
+        <v>23.6</v>
       </c>
       <c r="G8">
         <v>0.7</v>
@@ -2396,25 +2402,25 @@
         <v>112</v>
       </c>
       <c r="B9">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C9">
         <v>2</v>
       </c>
       <c r="D9">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E9">
         <v>129814</v>
       </c>
       <c r="F9">
-        <v>37.7</v>
+        <v>39.3</v>
       </c>
       <c r="G9">
         <v>1.5</v>
       </c>
       <c r="H9">
-        <v>14.6</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2448,7 +2454,7 @@
         <v>114</v>
       </c>
       <c r="B11">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C11">
         <v>16</v>
@@ -2460,7 +2466,7 @@
         <v>91102</v>
       </c>
       <c r="F11">
-        <v>158.1</v>
+        <v>162.5</v>
       </c>
       <c r="G11">
         <v>17.6</v>
@@ -2474,25 +2480,25 @@
         <v>115</v>
       </c>
       <c r="B12">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C12">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D12">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E12">
         <v>53206</v>
       </c>
       <c r="F12">
-        <v>364.6</v>
+        <v>372.1</v>
       </c>
       <c r="G12">
-        <v>48.9</v>
+        <v>45.1</v>
       </c>
       <c r="H12">
-        <v>105.3</v>
+        <v>110.9</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -2500,25 +2506,25 @@
         <v>116</v>
       </c>
       <c r="B13">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C13">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D13">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E13">
         <v>23417</v>
       </c>
       <c r="F13">
-        <v>1306.7</v>
+        <v>1319.6</v>
       </c>
       <c r="G13">
-        <v>226.3</v>
+        <v>217.8</v>
       </c>
       <c r="H13">
-        <v>320.3</v>
+        <v>328.8</v>
       </c>
     </row>
   </sheetData>
@@ -2628,7 +2634,7 @@
         <v>130</v>
       </c>
       <c r="F5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2636,16 +2642,16 @@
         <v>36</v>
       </c>
       <c r="B6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6" t="s">
         <v>132</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>132</v>
-      </c>
-      <c r="D6" t="s">
-        <v>133</v>
-      </c>
-      <c r="E6" t="s">
-        <v>133</v>
       </c>
       <c r="F6" t="s">
         <v>117</v>
@@ -2653,22 +2659,22 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7" t="s">
         <v>134</v>
-      </c>
-      <c r="C7" t="s">
-        <v>135</v>
       </c>
       <c r="D7" t="s">
         <v>119</v>
       </c>
       <c r="E7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F7" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2676,19 +2682,19 @@
         <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C8" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" t="s">
         <v>137</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>138</v>
       </c>
-      <c r="E8" t="s">
-        <v>139</v>
-      </c>
       <c r="F8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2705,7 +2711,7 @@
         <v>117</v>
       </c>
       <c r="E9" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F9" t="s">
         <v>117</v>
@@ -2716,16 +2722,16 @@
         <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D10" t="s">
         <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F10" t="s">
         <v>117</v>
@@ -2736,16 +2742,16 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" t="s">
         <v>141</v>
-      </c>
-      <c r="C11" t="s">
-        <v>142</v>
       </c>
       <c r="D11" t="s">
         <v>119</v>
       </c>
       <c r="E11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F11" t="s">
         <v>127</v>
@@ -2756,36 +2762,36 @@
         <v>20</v>
       </c>
       <c r="B12" t="s">
+        <v>143</v>
+      </c>
+      <c r="C12" t="s">
         <v>144</v>
-      </c>
-      <c r="C12" t="s">
-        <v>145</v>
       </c>
       <c r="D12" t="s">
         <v>117</v>
       </c>
       <c r="E12" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="C13" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D13" t="s">
         <v>119</v>
       </c>
       <c r="E13" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="F13" t="s">
         <v>147</v>
@@ -2802,10 +2808,10 @@
         <v>149</v>
       </c>
       <c r="D14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F14" t="s">
         <v>150</v>
@@ -2833,7 +2839,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
         <v>155</v>
@@ -2873,22 +2879,22 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D18" t="s">
         <v>119</v>
       </c>
       <c r="E18" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2905,10 +2911,10 @@
         <v>119</v>
       </c>
       <c r="E19" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F19" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2945,7 +2951,7 @@
         <v>119</v>
       </c>
       <c r="E21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F21" t="s">
         <v>166</v>
@@ -2973,22 +2979,22 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" t="s">
         <v>175</v>
       </c>
       <c r="C23" t="s">
-        <v>142</v>
+        <v>176</v>
       </c>
       <c r="D23" t="s">
         <v>117</v>
       </c>
       <c r="E23" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="F23" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2996,19 +3002,19 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D24" t="s">
         <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -3016,19 +3022,19 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C25" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D25" t="s">
         <v>117</v>
       </c>
       <c r="E25" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F25" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -3036,7 +3042,7 @@
         <v>11</v>
       </c>
       <c r="B26" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C26" t="s">
         <v>157</v>
@@ -3048,7 +3054,7 @@
         <v>157</v>
       </c>
       <c r="F26" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -3056,19 +3062,19 @@
         <v>18</v>
       </c>
       <c r="B27" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C27" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D27" t="s">
         <v>119</v>
       </c>
       <c r="E27" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F27" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -3076,39 +3082,39 @@
         <v>15</v>
       </c>
       <c r="B28" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C28" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D28" t="s">
         <v>119</v>
       </c>
       <c r="E28" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F28" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B29" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C29" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D29" t="s">
         <v>157</v>
       </c>
       <c r="E29" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F29" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -3116,19 +3122,19 @@
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C30" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D30" t="s">
         <v>119</v>
       </c>
       <c r="E30" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F30" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -3146,30 +3152,30 @@
         <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>56</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -3178,21 +3184,21 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1529</v>
+        <v>1563</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C3">
         <v>90</v>
@@ -3201,44 +3207,44 @@
         <v>100</v>
       </c>
       <c r="E3">
-        <v>1350</v>
+        <v>1366</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B4" t="s">
         <v>203</v>
-      </c>
-      <c r="B4" t="s">
-        <v>202</v>
       </c>
       <c r="C4">
         <v>90</v>
       </c>
       <c r="D4">
-        <v>98.5</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="E4">
-        <v>1438</v>
+        <v>1470</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -3247,21 +3253,21 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1538</v>
+        <v>1569</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -3270,21 +3276,21 @@
         <v>99.8</v>
       </c>
       <c r="E6">
-        <v>476</v>
+        <v>488</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -3293,13 +3299,13 @@
         <v>100</v>
       </c>
       <c r="E7">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3314,7 +3320,7 @@
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3323,27 +3329,27 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C2">
         <v>9</v>
@@ -3366,13 +3372,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -3381,10 +3387,10 @@
         <v>5</v>
       </c>
       <c r="F3">
-        <v>36.3</v>
+        <v>36.1</v>
       </c>
       <c r="G3">
-        <v>98.2</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -3392,7 +3398,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
@@ -3418,13 +3424,13 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
       </c>
       <c r="C5">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -3433,10 +3439,10 @@
         <v>5</v>
       </c>
       <c r="F5">
-        <v>41.8</v>
+        <v>42.9</v>
       </c>
       <c r="G5">
-        <v>97.7</v>
+        <v>97.8</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -3444,22 +3450,22 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6">
         <v>4</v>
       </c>
       <c r="F6">
-        <v>45.5</v>
+        <v>57.1</v>
       </c>
       <c r="G6">
         <v>100</v>
@@ -3470,74 +3476,74 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C7">
-        <v>18</v>
+        <v>125</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7">
-        <v>138</v>
+        <v>4</v>
       </c>
       <c r="F7">
-        <v>55.6</v>
+        <v>57.6</v>
       </c>
       <c r="G7">
-        <v>66.7</v>
+        <v>99.2</v>
       </c>
       <c r="H7">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C8">
-        <v>122</v>
+        <v>19</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8">
-        <v>4</v>
+        <v>138</v>
       </c>
       <c r="F8">
-        <v>56.6</v>
+        <v>57.9</v>
       </c>
       <c r="G8">
-        <v>99.2</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B9" t="s">
         <v>16</v>
       </c>
       <c r="C9">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D9">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E9">
         <v>5</v>
       </c>
       <c r="F9">
-        <v>66.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="G9">
         <v>100</v>
@@ -3548,13 +3554,13 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B10" t="s">
         <v>16</v>
       </c>
       <c r="C10">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -3563,7 +3569,7 @@
         <v>5</v>
       </c>
       <c r="F10">
-        <v>69.90000000000001</v>
+        <v>70.7</v>
       </c>
       <c r="G10">
         <v>97.3</v>
@@ -3574,7 +3580,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
@@ -3600,22 +3606,22 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
       </c>
       <c r="C12">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12">
-        <v>80.7</v>
+        <v>81.3</v>
       </c>
       <c r="G12">
         <v>98.90000000000001</v>
@@ -3626,13 +3632,13 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
       </c>
       <c r="C13">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -3652,13 +3658,13 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
       </c>
       <c r="C14">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -3667,10 +3673,10 @@
         <v>4</v>
       </c>
       <c r="F14">
-        <v>88.5</v>
+        <v>89.3</v>
       </c>
       <c r="G14">
-        <v>90.40000000000001</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="H14">
         <v>4</v>
@@ -3678,13 +3684,13 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
       </c>
       <c r="C15">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -3704,7 +3710,7 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
@@ -3730,7 +3736,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -3756,7 +3762,7 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B18" t="s">
         <v>16</v>
@@ -3782,10 +3788,10 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B19" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -3821,25 +3827,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -4031,19 +4037,19 @@
         <v>46266</v>
       </c>
       <c r="B10">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10">
         <v>3</v>
       </c>
       <c r="E10">
-        <v>71.7</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="F10">
-        <v>100</v>
+        <v>98.8</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -4061,62 +4067,62 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
       <c r="C2">
-        <v>1515</v>
+        <v>1546</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B3">
-        <v>880</v>
+        <v>897</v>
       </c>
       <c r="C3">
-        <v>1521</v>
+        <v>1551</v>
       </c>
       <c r="D3">
-        <v>57.9</v>
+        <v>57.8</v>
       </c>
       <c r="E3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -4131,13 +4137,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>57</v>
@@ -4145,55 +4151,55 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B2">
-        <v>1496</v>
+        <v>385</v>
       </c>
       <c r="C2">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B3">
-        <v>385</v>
+        <v>1526</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B4">
-        <v>1529</v>
+        <v>488</v>
       </c>
       <c r="C4">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D4">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B5">
-        <v>476</v>
+        <v>1563</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D5">
         <v>0.4</v>
@@ -4201,10 +4207,10 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B6">
-        <v>1422</v>
+        <v>1426</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -4215,10 +4221,10 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B7">
-        <v>1433</v>
+        <v>1440</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -4239,27 +4245,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>57</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -4274,98 +4280,98 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
       <c r="C3">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3">
-        <v>5.1</v>
+        <v>4.3</v>
       </c>
       <c r="F3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="F4" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C5">
-        <v>101</v>
+        <v>298</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="F5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C6">
-        <v>295</v>
+        <v>101</v>
       </c>
       <c r="D6">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="C7">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -4374,78 +4380,78 @@
         <v>2.5</v>
       </c>
       <c r="F7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C8">
-        <v>64</v>
+        <v>137</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="F8" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C9">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B10" t="s">
         <v>19</v>
       </c>
       <c r="C10">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F10" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
       </c>
       <c r="C11">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -4454,18 +4460,18 @@
         <v>0.7</v>
       </c>
       <c r="F11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
       </c>
       <c r="C12">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -4479,13 +4485,13 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B13" t="s">
         <v>16</v>
       </c>
       <c r="C13">
-        <v>102</v>
+        <v>65</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -4499,13 +4505,13 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B14" t="s">
         <v>16</v>
       </c>
       <c r="C14">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -4519,13 +4525,13 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
       </c>
       <c r="C15">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -4539,7 +4545,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
@@ -4559,7 +4565,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B17" t="s">
         <v>16</v>
@@ -4579,10 +4585,10 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C18">
         <v>9</v>
@@ -4599,10 +4605,10 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B19" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -4614,7 +4620,7 @@
         <v>16.7</v>
       </c>
       <c r="F19" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -4629,31 +4635,31 @@
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>103</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -4661,28 +4667,28 @@
         <v>411690</v>
       </c>
       <c r="B2">
-        <v>47.38508409765746</v>
+        <v>48.30107492611468</v>
       </c>
       <c r="C2">
         <v>27142</v>
       </c>
       <c r="D2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>
       </c>
       <c r="F2">
-        <v>2.448027732966176</v>
+        <v>2.42230633953743</v>
       </c>
       <c r="G2">
-        <v>2.022852683006045</v>
+        <v>2.003313340069452</v>
       </c>
       <c r="H2">
-        <v>2.936176080041506</v>
+        <v>2.90307057176576</v>
       </c>
       <c r="I2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -4690,7 +4696,7 @@
         <v>410220</v>
       </c>
       <c r="B3">
-        <v>7.10530453020303</v>
+        <v>7.238728845986588</v>
       </c>
       <c r="C3">
         <v>4046</v>
@@ -4702,16 +4708,16 @@
         <v>10</v>
       </c>
       <c r="F3">
-        <v>1.829618976180396</v>
+        <v>1.795895422606922</v>
       </c>
       <c r="G3">
-        <v>0.9741950484430553</v>
+        <v>0.9562386764689467</v>
       </c>
       <c r="H3">
-        <v>3.128704170758977</v>
+        <v>3.071035867089317</v>
       </c>
       <c r="I3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -4719,7 +4725,7 @@
         <v>412360</v>
       </c>
       <c r="B4">
-        <v>3.10181828849193</v>
+        <v>3.162009756399614</v>
       </c>
       <c r="C4">
         <v>1745</v>
@@ -4731,16 +4737,16 @@
         <v>11</v>
       </c>
       <c r="F4">
-        <v>1.611957740577687</v>
+        <v>1.581272793317751</v>
       </c>
       <c r="G4">
-        <v>0.5233982906547829</v>
+        <v>0.5134349718031814</v>
       </c>
       <c r="H4">
-        <v>3.761771642979022</v>
+        <v>3.690163212085936</v>
       </c>
       <c r="I4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -4748,7 +4754,7 @@
         <v>412830</v>
       </c>
       <c r="B5">
-        <v>3.788441971696381</v>
+        <v>3.859117955902845</v>
       </c>
       <c r="C5">
         <v>2106</v>
@@ -4760,16 +4766,16 @@
         <v>12</v>
       </c>
       <c r="F5">
-        <v>1.583764525054433</v>
+        <v>1.554759421339401</v>
       </c>
       <c r="G5">
-        <v>0.5812136677666706</v>
+        <v>0.5705693059013313</v>
       </c>
       <c r="H5">
-        <v>3.447188612122503</v>
+        <v>3.384056712374682</v>
       </c>
       <c r="I5" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -4777,7 +4783,7 @@
         <v>411090</v>
       </c>
       <c r="B6">
-        <v>7.918213436783874</v>
+        <v>8.07658145790295</v>
       </c>
       <c r="C6">
         <v>4530</v>
@@ -4789,16 +4795,16 @@
         <v>14</v>
       </c>
       <c r="F6">
-        <v>1.389202259805193</v>
+        <v>1.361962367040387</v>
       </c>
       <c r="G6">
-        <v>0.6934847628289208</v>
+        <v>0.6798867065054767</v>
       </c>
       <c r="H6">
-        <v>2.485666580022901</v>
+        <v>2.436926887432435</v>
       </c>
       <c r="I6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -4806,7 +4812,7 @@
         <v>411740</v>
       </c>
       <c r="B7">
-        <v>5.827231889666747</v>
+        <v>5.936113581323124</v>
       </c>
       <c r="C7">
         <v>3193</v>
@@ -4818,16 +4824,16 @@
         <v>13</v>
       </c>
       <c r="F7">
-        <v>1.372864535249774</v>
+        <v>1.347683107878952</v>
       </c>
       <c r="G7">
-        <v>0.5927054632703183</v>
+        <v>0.581833910256593</v>
       </c>
       <c r="H7">
-        <v>2.705090430354367</v>
+        <v>2.655472979794264</v>
       </c>
       <c r="I7" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -4835,28 +4841,28 @@
         <v>411520</v>
       </c>
       <c r="B8">
-        <v>705.9502798612566</v>
+        <v>719.6529728771376</v>
       </c>
       <c r="C8">
         <v>429660</v>
       </c>
       <c r="D8">
-        <v>949</v>
+        <v>967</v>
       </c>
       <c r="E8" t="s">
         <v>16</v>
       </c>
       <c r="F8">
-        <v>1.344287306163418</v>
+        <v>1.343703196464236</v>
       </c>
       <c r="G8">
-        <v>1.260109023961197</v>
+        <v>1.260335721703425</v>
       </c>
       <c r="H8">
-        <v>1.432610311569867</v>
+        <v>1.431136066593093</v>
       </c>
       <c r="I8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -4864,7 +4870,7 @@
         <v>411640</v>
       </c>
       <c r="B9">
-        <v>6.040577057625908</v>
+        <v>6.162928197530854</v>
       </c>
       <c r="C9">
         <v>3669</v>
@@ -4876,16 +4882,16 @@
         <v>17</v>
       </c>
       <c r="F9">
-        <v>1.324376781171995</v>
+        <v>1.298084245603439</v>
       </c>
       <c r="G9">
-        <v>0.5717718926188056</v>
+        <v>0.5604206419494328</v>
       </c>
       <c r="H9">
-        <v>2.609550225055589</v>
+        <v>2.557743448399862</v>
       </c>
       <c r="I9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -4893,7 +4899,7 @@
         <v>412530</v>
       </c>
       <c r="B10">
-        <v>9.760875835952792</v>
+        <v>9.939154525720845</v>
       </c>
       <c r="C10">
         <v>5170</v>
@@ -4905,16 +4911,16 @@
         <v>15</v>
       </c>
       <c r="F10">
-        <v>1.229397873887476</v>
+        <v>1.207346154941654</v>
       </c>
       <c r="G10">
-        <v>0.6352478212952247</v>
+        <v>0.623853376328558</v>
       </c>
       <c r="H10">
-        <v>2.147510674295021</v>
+        <v>2.108990759116576</v>
       </c>
       <c r="I10" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -4922,7 +4928,7 @@
         <v>412450</v>
       </c>
       <c r="B11">
-        <v>11.64930804914038</v>
+        <v>11.88145064901948</v>
       </c>
       <c r="C11">
         <v>6463</v>
@@ -4934,16 +4940,16 @@
         <v>18</v>
       </c>
       <c r="F11">
-        <v>1.201788118310863</v>
+        <v>1.178307297110674</v>
       </c>
       <c r="G11">
-        <v>0.6570287474598454</v>
+        <v>0.6441915640100934</v>
       </c>
       <c r="H11">
-        <v>2.016396254846134</v>
+        <v>1.976999426730276</v>
       </c>
       <c r="I11" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -4951,7 +4957,7 @@
         <v>410590</v>
       </c>
       <c r="B12">
-        <v>40.455990582026</v>
+        <v>41.23722755044143</v>
       </c>
       <c r="C12">
         <v>23313</v>
@@ -4963,16 +4969,16 @@
         <v>19</v>
       </c>
       <c r="F12">
-        <v>1.087601597859491</v>
+        <v>1.066997046447391</v>
       </c>
       <c r="G12">
-        <v>0.7902529859780106</v>
+        <v>0.7752816873791529</v>
       </c>
       <c r="H12">
-        <v>1.460054380835029</v>
+        <v>1.432393732290944</v>
       </c>
       <c r="I12" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -4980,7 +4986,7 @@
         <v>411110</v>
       </c>
       <c r="B13">
-        <v>10.65936448659817</v>
+        <v>10.86470264763838</v>
       </c>
       <c r="C13">
         <v>6228</v>
@@ -4992,16 +4998,16 @@
         <v>20</v>
       </c>
       <c r="F13">
-        <v>0.9381422328294355</v>
+        <v>0.9204117521038336</v>
       </c>
       <c r="G13">
-        <v>0.4498756658674717</v>
+        <v>0.4413732111826171</v>
       </c>
       <c r="H13">
-        <v>1.725276967978686</v>
+        <v>1.692669982644691</v>
       </c>
       <c r="I13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -5009,28 +5015,28 @@
         <v>411480</v>
       </c>
       <c r="B14">
-        <v>76.17178242564367</v>
+        <v>77.69069147927273</v>
       </c>
       <c r="C14">
         <v>44749</v>
       </c>
       <c r="D14">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F14">
-        <v>0.8533343704205795</v>
+        <v>0.8495226228950258</v>
       </c>
       <c r="G14">
-        <v>0.6585854516166045</v>
+        <v>0.6570207350034915</v>
       </c>
       <c r="H14">
-        <v>1.087644704871451</v>
+        <v>1.080801069519492</v>
       </c>
       <c r="I14" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -5038,7 +5044,7 @@
         <v>410780</v>
       </c>
       <c r="B15">
-        <v>9.536135539506603</v>
+        <v>9.713536080847046</v>
       </c>
       <c r="C15">
         <v>4805</v>
@@ -5047,19 +5053,19 @@
         <v>7</v>
       </c>
       <c r="E15" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F15">
-        <v>0.7340499692983787</v>
+        <v>0.7206438460451553</v>
       </c>
       <c r="G15">
-        <v>0.2951261587946642</v>
+        <v>0.2897362019449509</v>
       </c>
       <c r="H15">
-        <v>1.512423486636874</v>
+        <v>1.484801748988272</v>
       </c>
       <c r="I15" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -5067,28 +5073,28 @@
         <v>412625</v>
       </c>
       <c r="B16">
-        <v>205.0170708322734</v>
+        <v>209.2850121326406</v>
       </c>
       <c r="C16">
         <v>128106</v>
       </c>
       <c r="D16">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="E16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F16">
-        <v>0.6877476076875255</v>
+        <v>0.6928350889651953</v>
       </c>
       <c r="G16">
-        <v>0.5789168998976707</v>
+        <v>0.5846565411413399</v>
       </c>
       <c r="H16">
-        <v>0.8110930839475775</v>
+        <v>0.8152270746461704</v>
       </c>
       <c r="I16" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -5096,54 +5102,54 @@
         <v>411810</v>
       </c>
       <c r="B17">
-        <v>15.95996617493859</v>
+        <v>16.27266485298788</v>
       </c>
       <c r="C17">
         <v>9549</v>
       </c>
       <c r="D17">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F17">
-        <v>0.6265677439656901</v>
+        <v>0.6759802465900506</v>
       </c>
       <c r="G17">
-        <v>0.3004635876774271</v>
+        <v>0.3374469035554792</v>
       </c>
       <c r="H17">
-        <v>1.152280389597288</v>
+        <v>1.209515386146975</v>
       </c>
       <c r="I17" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18">
-        <v>410210</v>
+        <v>411360</v>
       </c>
       <c r="B18">
-        <v>47.63556056736902</v>
+        <v>7.783986307734082</v>
       </c>
       <c r="C18">
-        <v>26203</v>
+        <v>4707</v>
       </c>
       <c r="D18">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F18">
-        <v>0.3988616859694362</v>
+        <v>0.5138755185149343</v>
       </c>
       <c r="G18">
-        <v>0.2401407903700153</v>
+        <v>0.1400137834959251</v>
       </c>
       <c r="H18">
-        <v>0.6228719305113105</v>
+        <v>1.315725422747438</v>
       </c>
       <c r="I18" t="s">
         <v>265</v>
@@ -5151,31 +5157,31 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19">
-        <v>411360</v>
+        <v>410210</v>
       </c>
       <c r="B19">
-        <v>7.633285073459273</v>
+        <v>48.55566975652325</v>
       </c>
       <c r="C19">
-        <v>4707</v>
+        <v>26203</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F19">
-        <v>0.3930155851811324</v>
+        <v>0.4118983447306498</v>
       </c>
       <c r="G19">
-        <v>0.08104926213835609</v>
+        <v>0.2515982097798724</v>
       </c>
       <c r="H19">
-        <v>1.148558318649188</v>
+        <v>0.6361435864763223</v>
       </c>
       <c r="I19" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -5183,7 +5189,7 @@
         <v>411630</v>
       </c>
       <c r="B20">
-        <v>7.882784676284354</v>
+        <v>8.031181483295246</v>
       </c>
       <c r="C20">
         <v>4057</v>
@@ -5192,19 +5198,19 @@
         <v>3</v>
       </c>
       <c r="E20" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F20">
-        <v>0.3805761698687026</v>
+        <v>0.3735440428335434</v>
       </c>
       <c r="G20">
-        <v>0.07848395564538241</v>
+        <v>0.07703376199161124</v>
       </c>
       <c r="H20">
-        <v>1.112205068358519</v>
+        <v>1.091654209032399</v>
       </c>
       <c r="I20" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -5212,7 +5218,7 @@
         <v>410790</v>
       </c>
       <c r="B21">
-        <v>20.03494509019059</v>
+        <v>20.44186950941049</v>
       </c>
       <c r="C21">
         <v>11522</v>
@@ -5224,16 +5230,16 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>0.3493895275723667</v>
+        <v>0.3424344332487556</v>
       </c>
       <c r="G21">
-        <v>0.1404727109982358</v>
+        <v>0.1376764023576348</v>
       </c>
       <c r="H21">
-        <v>0.7198759615649725</v>
+        <v>0.7055458090593349</v>
       </c>
       <c r="I21" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -5241,28 +5247,28 @@
         <v>411410</v>
       </c>
       <c r="B22">
-        <v>59.27647461376149</v>
+        <v>60.47964065424704</v>
       </c>
       <c r="C22">
         <v>34521</v>
       </c>
       <c r="D22">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E22" t="s">
         <v>29</v>
       </c>
       <c r="F22">
-        <v>0.303661783486381</v>
+        <v>0.3306897955022084</v>
       </c>
       <c r="G22">
-        <v>0.1799692179724009</v>
+        <v>0.2019939181722976</v>
       </c>
       <c r="H22">
-        <v>0.4799165343905864</v>
+        <v>0.5107235686015197</v>
       </c>
       <c r="I22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -5270,28 +5276,28 @@
         <v>411750</v>
       </c>
       <c r="B23">
-        <v>79.74180237038844</v>
+        <v>81.38211863861062</v>
       </c>
       <c r="C23">
         <v>48695</v>
       </c>
       <c r="D23">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E23" t="s">
         <v>30</v>
       </c>
       <c r="F23">
-        <v>0.3009713761989437</v>
+        <v>0.3071927890083104</v>
       </c>
       <c r="G23">
-        <v>0.1928380397430883</v>
+        <v>0.1987989759725127</v>
       </c>
       <c r="H23">
-        <v>0.4478215507079371</v>
+        <v>0.4534771558530221</v>
       </c>
       <c r="I23" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -5299,7 +5305,7 @@
         <v>412040</v>
       </c>
       <c r="B24">
-        <v>7.044833660150949</v>
+        <v>7.185789935959376</v>
       </c>
       <c r="C24">
         <v>4304</v>
@@ -5311,16 +5317,16 @@
         <v>31</v>
       </c>
       <c r="F24">
-        <v>0.283895986261959</v>
+        <v>0.2783270896901023</v>
       </c>
       <c r="G24">
-        <v>0.03438112100701823</v>
+        <v>0.03370670179654055</v>
       </c>
       <c r="H24">
-        <v>1.025529915431553</v>
+        <v>1.005413146238791</v>
       </c>
       <c r="I24" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -5328,7 +5334,7 @@
         <v>412340</v>
       </c>
       <c r="B25">
-        <v>20.46290725620743</v>
+        <v>20.85835781950359</v>
       </c>
       <c r="C25">
         <v>11730</v>
@@ -5340,16 +5346,16 @@
         <v>32</v>
       </c>
       <c r="F25">
-        <v>0.2443445565870533</v>
+        <v>0.239712063781203</v>
       </c>
       <c r="G25">
-        <v>0.07933801242372027</v>
+        <v>0.07783385461919638</v>
       </c>
       <c r="H25">
-        <v>0.5702186856065173</v>
+        <v>0.5594079927237705</v>
       </c>
       <c r="I25" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -5357,7 +5363,7 @@
         <v>411420</v>
       </c>
       <c r="B26">
-        <v>67.15768140095651</v>
+        <v>68.47329253981592</v>
       </c>
       <c r="C26">
         <v>38313</v>
@@ -5369,16 +5375,16 @@
         <v>33</v>
       </c>
       <c r="F26">
-        <v>0.2233549414912701</v>
+        <v>0.2190635128474038</v>
       </c>
       <c r="G26">
-        <v>0.1250100652322958</v>
+        <v>0.1226081851971929</v>
       </c>
       <c r="H26">
-        <v>0.3683900092347958</v>
+        <v>0.3613119503067546</v>
       </c>
       <c r="I26" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -5386,7 +5392,7 @@
         <v>411000</v>
       </c>
       <c r="B27">
-        <v>9.409137117451714</v>
+        <v>9.600329276281888</v>
       </c>
       <c r="C27">
         <v>5693</v>
@@ -5398,16 +5404,16 @@
         <v>35</v>
       </c>
       <c r="F27">
-        <v>0.2125593425873745</v>
+        <v>0.2083261878257763</v>
       </c>
       <c r="G27">
-        <v>0.02574192250793372</v>
+        <v>0.0252292678275479</v>
       </c>
       <c r="H27">
-        <v>0.7678374305252582</v>
+        <v>0.7525458200244156</v>
       </c>
       <c r="I27" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -5415,7 +5421,7 @@
         <v>410810</v>
       </c>
       <c r="B28">
-        <v>4.919571245722143</v>
+        <v>5.015891852603958</v>
       </c>
       <c r="C28">
         <v>2711</v>
@@ -5427,16 +5433,16 @@
         <v>34</v>
       </c>
       <c r="F28">
-        <v>0.2032697464986525</v>
+        <v>0.199366339902416</v>
       </c>
       <c r="G28">
-        <v>0.005146344410868163</v>
+        <v>0.005047518712180038</v>
       </c>
       <c r="H28">
-        <v>1.132546539657043</v>
+        <v>1.110798150092974</v>
       </c>
       <c r="I28" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -5444,7 +5450,7 @@
         <v>410115</v>
       </c>
       <c r="B29">
-        <v>6.067772497579909</v>
+        <v>6.187232173738672</v>
       </c>
       <c r="C29">
         <v>3357</v>
@@ -5456,16 +5462,16 @@
         <v>37</v>
       </c>
       <c r="F29">
-        <v>0.1648051241866506</v>
+        <v>0.1616231574829919</v>
       </c>
       <c r="G29">
-        <v>0.004172504488984667</v>
+        <v>0.004091944066969034</v>
       </c>
       <c r="H29">
-        <v>0.9182353809674164</v>
+        <v>0.9005065972127889</v>
       </c>
       <c r="I29" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -5473,7 +5479,7 @@
         <v>410730</v>
       </c>
       <c r="B30">
-        <v>12.58712092416635</v>
+        <v>12.82194342279607</v>
       </c>
       <c r="C30">
         <v>6517</v>
@@ -5485,16 +5491,16 @@
         <v>36</v>
       </c>
       <c r="F30">
-        <v>0.1588925705925449</v>
+        <v>0.1559825943736586</v>
       </c>
       <c r="G30">
-        <v>0.01924262744460815</v>
+        <v>0.01889021582432988</v>
       </c>
       <c r="H30">
-        <v>0.5739745976264586</v>
+        <v>0.5634627629754799</v>
       </c>
       <c r="I30" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -5502,7 +5508,7 @@
         <v>411160</v>
       </c>
       <c r="B31">
-        <v>4.81867844685021</v>
+        <v>4.908729112613215</v>
       </c>
       <c r="C31">
         <v>2685</v>
@@ -5511,19 +5517,19 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
+        <v>267</v>
+      </c>
+      <c r="F31">
+        <v>0</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+      <c r="H31">
+        <v>0.7514937918727645</v>
+      </c>
+      <c r="I31" t="s">
         <v>266</v>
-      </c>
-      <c r="F31">
-        <v>0</v>
-      </c>
-      <c r="G31">
-        <v>0</v>
-      </c>
-      <c r="H31">
-        <v>0.7655375835516101</v>
-      </c>
-      <c r="I31" t="s">
-        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -5552,10 +5558,10 @@
         <v>41</v>
       </c>
       <c r="B2">
-        <v>60</v>
+        <v>59.7</v>
       </c>
       <c r="C2">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5563,10 +5569,10 @@
         <v>42</v>
       </c>
       <c r="B3">
-        <v>60.5</v>
+        <v>60.2</v>
       </c>
       <c r="C3">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5574,10 +5580,10 @@
         <v>43</v>
       </c>
       <c r="B4">
-        <v>60.5</v>
+        <v>60.2</v>
       </c>
       <c r="C4">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5585,10 +5591,10 @@
         <v>44</v>
       </c>
       <c r="B5">
-        <v>60.6</v>
+        <v>60.3</v>
       </c>
       <c r="C5">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -5596,10 +5602,10 @@
         <v>45</v>
       </c>
       <c r="B6">
-        <v>92.90000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="C6">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5610,7 +5616,7 @@
         <v>96.59999999999999</v>
       </c>
       <c r="C7">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5618,10 +5624,10 @@
         <v>47</v>
       </c>
       <c r="B8">
-        <v>98.59999999999999</v>
+        <v>98.7</v>
       </c>
       <c r="C8">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -5632,7 +5638,7 @@
         <v>98.8</v>
       </c>
       <c r="C9">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -5640,10 +5646,10 @@
         <v>49</v>
       </c>
       <c r="B10">
-        <v>99.09999999999999</v>
+        <v>99.3</v>
       </c>
       <c r="C10">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -5651,10 +5657,10 @@
         <v>50</v>
       </c>
       <c r="B11">
-        <v>99.90000000000001</v>
+        <v>99.8</v>
       </c>
       <c r="C11">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -5665,7 +5671,7 @@
         <v>100</v>
       </c>
       <c r="C12">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -5676,7 +5682,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -5687,7 +5693,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -5698,7 +5704,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1521</v>
+        <v>1551</v>
       </c>
     </row>
   </sheetData>
@@ -5713,7 +5719,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -5724,29 +5730,29 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B2">
-        <v>1473</v>
+        <v>1505</v>
       </c>
       <c r="C2">
-        <v>96.8</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B3">
         <v>24</v>
       </c>
       <c r="C3">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B4">
         <v>9</v>
@@ -5757,13 +5763,13 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B5">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -5778,10 +5784,10 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>56</v>
@@ -5795,41 +5801,41 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C2">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D2">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E2">
-        <v>40.5</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C3">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D3">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E3">
-        <v>59</v>
+        <v>59.2</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B4" t="s">
         <v>83</v>
@@ -5838,7 +5844,7 @@
         <v>2</v>
       </c>
       <c r="D4">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E4">
         <v>0.5</v>
@@ -5849,16 +5855,16 @@
         <v>93</v>
       </c>
       <c r="B5" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C5">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D5">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E5">
-        <v>52.6</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -5866,16 +5872,16 @@
         <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C6">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D6">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E6">
-        <v>47.4</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -5889,7 +5895,7 @@
         <v>0</v>
       </c>
       <c r="D7">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -5907,7 +5913,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>78</v>
@@ -5921,29 +5927,29 @@
         <v>83</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B3">
-        <v>636</v>
+        <v>647</v>
       </c>
       <c r="C3">
-        <v>41.8</v>
+        <v>41.7</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B4">
-        <v>883</v>
+        <v>901</v>
       </c>
       <c r="C4">
         <v>58.1</v>
@@ -5975,10 +5981,10 @@
         <v>44</v>
       </c>
       <c r="B2">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C2">
-        <v>30</v>
+        <v>29.7</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5986,10 +5992,10 @@
         <v>42</v>
       </c>
       <c r="B3">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5997,10 +6003,10 @@
         <v>58</v>
       </c>
       <c r="B4">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C4">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -6008,7 +6014,7 @@
         <v>59</v>
       </c>
       <c r="B5">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="C5">
         <v>11.8</v>
@@ -6019,10 +6025,10 @@
         <v>60</v>
       </c>
       <c r="B6">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="C6">
-        <v>10.8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -6033,7 +6039,7 @@
         <v>59</v>
       </c>
       <c r="C7">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -6063,7 +6069,7 @@
         <v>62</v>
       </c>
       <c r="B10">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10">
         <v>1.1</v>
@@ -6077,7 +6083,7 @@
         <v>10</v>
       </c>
       <c r="C11">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -6129,10 +6135,10 @@
         <v>67</v>
       </c>
       <c r="B3">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C3">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -6149,7 +6155,7 @@
         <v>34</v>
       </c>
       <c r="C4">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -6197,7 +6203,7 @@
         <v>71</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>32</v>
@@ -6214,7 +6220,7 @@
         <v>72</v>
       </c>
       <c r="B8">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C8">
         <v>48</v>
@@ -6231,10 +6237,10 @@
         <v>73</v>
       </c>
       <c r="B9">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C9">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -6265,10 +6271,10 @@
         <v>75</v>
       </c>
       <c r="B11">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C11">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -6282,16 +6288,16 @@
         <v>76</v>
       </c>
       <c r="B12">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="C12">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="D12">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E12">
-        <v>15.5</v>
+        <v>14.7</v>
       </c>
     </row>
   </sheetData>
@@ -6326,10 +6332,10 @@
         <v>148</v>
       </c>
       <c r="C2">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D2">
-        <v>43.9</v>
+        <v>45.3</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -6337,13 +6343,13 @@
         <v>67</v>
       </c>
       <c r="B3">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C3">
         <v>58</v>
       </c>
       <c r="D3">
-        <v>21.6</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -6393,13 +6399,13 @@
         <v>71</v>
       </c>
       <c r="B7">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>13</v>
       </c>
       <c r="D7">
-        <v>40.6</v>
+        <v>39.4</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -6407,13 +6413,13 @@
         <v>72</v>
       </c>
       <c r="B8">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C8">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D8">
-        <v>38.8</v>
+        <v>39.2</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -6421,13 +6427,13 @@
         <v>73</v>
       </c>
       <c r="B9">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C9">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D9">
-        <v>25.5</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -6449,13 +6455,13 @@
         <v>75</v>
       </c>
       <c r="B11">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C11">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D11">
-        <v>23.9</v>
+        <v>25.4</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -6463,13 +6469,13 @@
         <v>76</v>
       </c>
       <c r="B12">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="C12">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="D12">
-        <v>29.3</v>
+        <v>29.6</v>
       </c>
     </row>
   </sheetData>
@@ -6498,10 +6504,10 @@
         <v>79</v>
       </c>
       <c r="B2">
-        <v>877</v>
+        <v>891</v>
       </c>
       <c r="C2">
-        <v>99.40000000000001</v>
+        <v>99.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6509,10 +6515,10 @@
         <v>80</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6552,10 +6558,10 @@
         <v>83</v>
       </c>
       <c r="B2">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C2">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6563,10 +6569,10 @@
         <v>84</v>
       </c>
       <c r="B3">
-        <v>1126</v>
+        <v>1159</v>
       </c>
       <c r="C3">
-        <v>74</v>
+        <v>74.7</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6577,7 +6583,7 @@
         <v>374</v>
       </c>
       <c r="C4">
-        <v>24.6</v>
+        <v>24.1</v>
       </c>
     </row>
   </sheetData>
@@ -6617,10 +6623,10 @@
         <v>84</v>
       </c>
       <c r="B3">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C3">
-        <v>25.2</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6628,10 +6634,10 @@
         <v>85</v>
       </c>
       <c r="B4">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="C4">
-        <v>74.3</v>
+        <v>73.8</v>
       </c>
     </row>
   </sheetData>
@@ -6675,25 +6681,25 @@
         <v>93</v>
       </c>
       <c r="B2">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="C2">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D2">
-        <v>77.2</v>
+        <v>73.5</v>
       </c>
       <c r="E2">
         <v>13</v>
       </c>
       <c r="F2">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G2">
-        <v>52.3</v>
+        <v>50</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -6701,19 +6707,19 @@
         <v>94</v>
       </c>
       <c r="B3">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C3">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D3">
-        <v>73.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="E3">
         <v>75</v>
       </c>
       <c r="F3">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G3">
         <v>50.5</v>

</xml_diff>

<commit_message>
Atualização de dados — 28/10/2026
</commit_message>
<xml_diff>
--- a/tabelas/descritiva_15rs_2026.xlsx
+++ b/tabelas/descritiva_15rs_2026.xlsx
@@ -82,6 +82,9 @@
     <t>Itaguaje</t>
   </si>
   <si>
+    <t>Santo Inacio</t>
+  </si>
+  <si>
     <t>Sao Jorge Do Ivai</t>
   </si>
   <si>
@@ -91,9 +94,6 @@
     <t>Nossa Senhora Das Gracas</t>
   </si>
   <si>
-    <t>Santo Inacio</t>
-  </si>
-  <si>
     <t>Colorado</t>
   </si>
   <si>
@@ -163,15 +163,15 @@
     <t>Obesidade</t>
   </si>
   <si>
+    <t>Cardiopatia</t>
+  </si>
+  <si>
     <t>Diabetes</t>
   </si>
   <si>
     <t>Imunodepressão</t>
   </si>
   <si>
-    <t>Cardiopatia</t>
-  </si>
-  <si>
     <t>Evolução (Desfecho)</t>
   </si>
   <si>
@@ -514,22 +514,22 @@
     <t>100,0% (66)</t>
   </si>
   <si>
-    <t>100,0% (64)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 30,1% (965)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 76,3% (962)</t>
+    <t>100,0% (65)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 30,0% (977)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 76,2% (974)</t>
   </si>
   <si>
     <t xml:space="preserve"> 97,7% (347)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 99,7% (962)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,9% (938)</t>
+    <t xml:space="preserve"> 99,7% (972)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,6% (937)</t>
   </si>
   <si>
     <t xml:space="preserve"> 25,0% (8)</t>
@@ -583,10 +583,10 @@
     <t xml:space="preserve"> 25,0% (4)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 14,3% (14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 85,7% (14)</t>
+    <t xml:space="preserve"> 13,3% (15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 86,7% (15)</t>
   </si>
   <si>
     <t>100,0% (14)</t>
@@ -601,16 +601,16 @@
     <t>100,0% (12)</t>
   </si>
   <si>
-    <t xml:space="preserve"> 24,8% (141)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 68,1% (141)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 99,3% (141)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 94,0% (133)</t>
+    <t xml:space="preserve"> 24,5% (143)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 67,8% (143)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 99,3% (143)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 93,4% (137)</t>
   </si>
   <si>
     <t xml:space="preserve">  0,0% (6)</t>
@@ -1426,10 +1426,10 @@
         <v>15</v>
       </c>
       <c r="B8">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C8">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1455,28 +1455,28 @@
         <v>16</v>
       </c>
       <c r="B9">
-        <v>967</v>
+        <v>12</v>
       </c>
       <c r="C9">
-        <v>877</v>
+        <v>12</v>
       </c>
       <c r="D9">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>285</v>
+        <v>3</v>
       </c>
       <c r="F9">
-        <v>225.1</v>
+        <v>232.1</v>
       </c>
       <c r="G9">
-        <v>17.7</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>8.699999999999999</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>29.5</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1484,28 +1484,28 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>8</v>
+        <v>977</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>878</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>289</v>
       </c>
       <c r="F10">
-        <v>218</v>
+        <v>227.4</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>17.7</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I10">
-        <v>37.5</v>
+        <v>29.6</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1513,10 +1513,10 @@
         <v>18</v>
       </c>
       <c r="B11">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C11">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -1525,7 +1525,7 @@
         <v>3</v>
       </c>
       <c r="F11">
-        <v>216.6</v>
+        <v>218</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1534,7 +1534,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>21.4</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1603,7 +1603,7 @@
         <v>66</v>
       </c>
       <c r="C14">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D14">
         <v>2</v>
@@ -1687,10 +1687,10 @@
         <v>24</v>
       </c>
       <c r="B17">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C17">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D17">
         <v>10</v>
@@ -1699,16 +1699,16 @@
         <v>58</v>
       </c>
       <c r="F17">
-        <v>113.2</v>
+        <v>114</v>
       </c>
       <c r="G17">
         <v>7.8</v>
       </c>
       <c r="H17">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="I17">
-        <v>40</v>
+        <v>39.7</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -2038,7 +2038,7 @@
         <v>2</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -2114,13 +2114,13 @@
         <v>97</v>
       </c>
       <c r="B2">
-        <v>1540</v>
+        <v>1555</v>
       </c>
       <c r="C2">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="D2">
-        <v>29</v>
+        <v>28.9</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2128,13 +2128,13 @@
         <v>98</v>
       </c>
       <c r="B3">
-        <v>1537</v>
+        <v>1552</v>
       </c>
       <c r="C3">
-        <v>1172</v>
+        <v>1182</v>
       </c>
       <c r="D3">
-        <v>76.3</v>
+        <v>76.2</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2156,10 +2156,10 @@
         <v>100</v>
       </c>
       <c r="B5">
-        <v>1536</v>
+        <v>1548</v>
       </c>
       <c r="C5">
-        <v>1528</v>
+        <v>1540</v>
       </c>
       <c r="D5">
         <v>99.5</v>
@@ -2170,13 +2170,13 @@
         <v>101</v>
       </c>
       <c r="B6">
-        <v>1478</v>
+        <v>1483</v>
       </c>
       <c r="C6">
-        <v>1393</v>
+        <v>1394</v>
       </c>
       <c r="D6">
-        <v>94.2</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2220,25 +2220,25 @@
         <v>105</v>
       </c>
       <c r="B2">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C2">
         <v>4</v>
       </c>
       <c r="D2">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E2">
         <v>10254</v>
       </c>
       <c r="F2">
-        <v>2789.2</v>
+        <v>2818.4</v>
       </c>
       <c r="G2">
         <v>39</v>
       </c>
       <c r="H2">
-        <v>994.7</v>
+        <v>1014.2</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2246,25 +2246,25 @@
         <v>106</v>
       </c>
       <c r="B3">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E3">
         <v>42663</v>
       </c>
       <c r="F3">
-        <v>637.6</v>
+        <v>644.6</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
-        <v>135.9</v>
+        <v>140.6</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2298,7 +2298,7 @@
         <v>108</v>
       </c>
       <c r="B5">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -2310,7 +2310,7 @@
         <v>57229</v>
       </c>
       <c r="F5">
-        <v>59.4</v>
+        <v>57.7</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -2402,7 +2402,7 @@
         <v>112</v>
       </c>
       <c r="B9">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -2414,7 +2414,7 @@
         <v>129814</v>
       </c>
       <c r="F9">
-        <v>39.3</v>
+        <v>38.5</v>
       </c>
       <c r="G9">
         <v>1.5</v>
@@ -2428,7 +2428,7 @@
         <v>113</v>
       </c>
       <c r="B10">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C10">
         <v>6</v>
@@ -2440,7 +2440,7 @@
         <v>114639</v>
       </c>
       <c r="F10">
-        <v>73.3</v>
+        <v>75</v>
       </c>
       <c r="G10">
         <v>5.2</v>
@@ -2454,7 +2454,7 @@
         <v>114</v>
       </c>
       <c r="B11">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C11">
         <v>16</v>
@@ -2466,7 +2466,7 @@
         <v>91102</v>
       </c>
       <c r="F11">
-        <v>162.5</v>
+        <v>164.7</v>
       </c>
       <c r="G11">
         <v>17.6</v>
@@ -2480,7 +2480,7 @@
         <v>115</v>
       </c>
       <c r="B12">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C12">
         <v>24</v>
@@ -2492,7 +2492,7 @@
         <v>53206</v>
       </c>
       <c r="F12">
-        <v>372.1</v>
+        <v>377.8</v>
       </c>
       <c r="G12">
         <v>45.1</v>
@@ -2506,7 +2506,7 @@
         <v>116</v>
       </c>
       <c r="B13">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C13">
         <v>51</v>
@@ -2518,7 +2518,7 @@
         <v>23417</v>
       </c>
       <c r="F13">
-        <v>1319.6</v>
+        <v>1323.8</v>
       </c>
       <c r="G13">
         <v>217.8</v>
@@ -2654,7 +2654,7 @@
         <v>132</v>
       </c>
       <c r="F6" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2859,7 +2859,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>160</v>
@@ -2899,7 +2899,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
         <v>165</v>
@@ -3059,7 +3059,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B27" t="s">
         <v>182</v>
@@ -3079,7 +3079,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B28" t="s">
         <v>185</v>
@@ -3184,7 +3184,7 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1563</v>
+        <v>1578</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -3207,7 +3207,7 @@
         <v>100</v>
       </c>
       <c r="E3">
-        <v>1366</v>
+        <v>1387</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -3227,10 +3227,10 @@
         <v>90</v>
       </c>
       <c r="D4">
-        <v>98.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="E4">
-        <v>1470</v>
+        <v>1484</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -3253,7 +3253,7 @@
         <v>0</v>
       </c>
       <c r="E5">
-        <v>1569</v>
+        <v>1578</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -3273,10 +3273,10 @@
         <v>100</v>
       </c>
       <c r="D6">
-        <v>99.8</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E6">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="F6" t="b">
         <v>0</v>
@@ -3378,7 +3378,7 @@
         <v>24</v>
       </c>
       <c r="C3">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -3387,7 +3387,7 @@
         <v>5</v>
       </c>
       <c r="F3">
-        <v>36.1</v>
+        <v>36.7</v>
       </c>
       <c r="G3">
         <v>97.90000000000001</v>
@@ -3401,7 +3401,7 @@
         <v>216</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>101</v>
@@ -3427,10 +3427,10 @@
         <v>217</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -3439,7 +3439,7 @@
         <v>5</v>
       </c>
       <c r="F5">
-        <v>42.9</v>
+        <v>44.2</v>
       </c>
       <c r="G5">
         <v>97.8</v>
@@ -3456,7 +3456,7 @@
         <v>26</v>
       </c>
       <c r="C6">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -3465,7 +3465,7 @@
         <v>4</v>
       </c>
       <c r="F6">
-        <v>57.1</v>
+        <v>53.3</v>
       </c>
       <c r="G6">
         <v>100</v>
@@ -3482,7 +3482,7 @@
         <v>9</v>
       </c>
       <c r="C7">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -3491,7 +3491,7 @@
         <v>4</v>
       </c>
       <c r="F7">
-        <v>57.6</v>
+        <v>56.2</v>
       </c>
       <c r="G7">
         <v>99.2</v>
@@ -3505,10 +3505,10 @@
         <v>220</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C8">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -3517,13 +3517,13 @@
         <v>138</v>
       </c>
       <c r="F8">
-        <v>57.9</v>
+        <v>61.1</v>
       </c>
       <c r="G8">
-        <v>68.40000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="H8">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3531,7 +3531,7 @@
         <v>221</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <v>17</v>
@@ -3557,10 +3557,10 @@
         <v>222</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -3569,10 +3569,10 @@
         <v>5</v>
       </c>
       <c r="F10">
-        <v>70.7</v>
+        <v>71.8</v>
       </c>
       <c r="G10">
-        <v>97.3</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -3586,7 +3586,7 @@
         <v>19</v>
       </c>
       <c r="C11">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -3595,7 +3595,7 @@
         <v>2</v>
       </c>
       <c r="F11">
-        <v>71.7</v>
+        <v>72</v>
       </c>
       <c r="G11">
         <v>99</v>
@@ -3609,10 +3609,10 @@
         <v>224</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -3621,10 +3621,10 @@
         <v>3</v>
       </c>
       <c r="F12">
-        <v>81.3</v>
+        <v>82.3</v>
       </c>
       <c r="G12">
-        <v>98.90000000000001</v>
+        <v>99</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -3635,10 +3635,10 @@
         <v>225</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -3647,7 +3647,7 @@
         <v>2</v>
       </c>
       <c r="F13">
-        <v>86.8</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="G13">
         <v>99.3</v>
@@ -3661,10 +3661,10 @@
         <v>226</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -3673,10 +3673,10 @@
         <v>4</v>
       </c>
       <c r="F14">
-        <v>89.3</v>
+        <v>89.8</v>
       </c>
       <c r="G14">
-        <v>91.09999999999999</v>
+        <v>91.5</v>
       </c>
       <c r="H14">
         <v>4</v>
@@ -3687,7 +3687,7 @@
         <v>227</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C15">
         <v>60</v>
@@ -3713,7 +3713,7 @@
         <v>228</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C16">
         <v>40</v>
@@ -3739,7 +3739,7 @@
         <v>229</v>
       </c>
       <c r="B17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C17">
         <v>14</v>
@@ -3765,7 +3765,7 @@
         <v>230</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C18">
         <v>13</v>
@@ -3968,7 +3968,7 @@
         <v>46174</v>
       </c>
       <c r="B7">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -3977,13 +3977,13 @@
         <v>5</v>
       </c>
       <c r="E7">
-        <v>59.3</v>
+        <v>59.6</v>
       </c>
       <c r="F7">
-        <v>97</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -3991,7 +3991,7 @@
         <v>46204</v>
       </c>
       <c r="B8">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -4000,10 +4000,10 @@
         <v>4</v>
       </c>
       <c r="E8">
-        <v>65.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F8">
-        <v>95.3</v>
+        <v>95.2</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -4037,7 +4037,7 @@
         <v>46266</v>
       </c>
       <c r="B10">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -4046,10 +4046,10 @@
         <v>3</v>
       </c>
       <c r="E10">
-        <v>77.90000000000001</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="F10">
-        <v>98.8</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -4093,7 +4093,7 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>1546</v>
+        <v>1555</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -4110,13 +4110,13 @@
         <v>243</v>
       </c>
       <c r="B3">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="C3">
-        <v>1551</v>
+        <v>1563</v>
       </c>
       <c r="D3">
-        <v>57.8</v>
+        <v>57.6</v>
       </c>
       <c r="E3" t="s">
         <v>244</v>
@@ -4168,7 +4168,7 @@
         <v>250</v>
       </c>
       <c r="B3">
-        <v>1526</v>
+        <v>1532</v>
       </c>
       <c r="C3">
         <v>14</v>
@@ -4182,7 +4182,7 @@
         <v>251</v>
       </c>
       <c r="B4">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -4196,7 +4196,7 @@
         <v>252</v>
       </c>
       <c r="B5">
-        <v>1563</v>
+        <v>1578</v>
       </c>
       <c r="C5">
         <v>7</v>
@@ -4210,7 +4210,7 @@
         <v>253</v>
       </c>
       <c r="B6">
-        <v>1426</v>
+        <v>1438</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -4224,7 +4224,7 @@
         <v>254</v>
       </c>
       <c r="B7">
-        <v>1440</v>
+        <v>1448</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -4268,19 +4268,19 @@
         <v>220</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>5.3</v>
       </c>
       <c r="F2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -4288,16 +4288,16 @@
         <v>228</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D3">
         <v>2</v>
       </c>
       <c r="E3">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="F3" t="s">
         <v>250</v>
@@ -4308,10 +4308,10 @@
         <v>226</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D4">
         <v>3</v>
@@ -4331,13 +4331,13 @@
         <v>24</v>
       </c>
       <c r="C5">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="F5" t="s">
         <v>249</v>
@@ -4348,7 +4348,7 @@
         <v>224</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6">
         <v>101</v>
@@ -4368,7 +4368,7 @@
         <v>222</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>81</v>
@@ -4405,19 +4405,19 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C9">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="F9" t="s">
         <v>250</v>
@@ -4425,10 +4425,10 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C10">
         <v>106</v>
@@ -4448,10 +4448,10 @@
         <v>217</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -4468,10 +4468,10 @@
         <v>225</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C12">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -4488,7 +4488,7 @@
         <v>227</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13">
         <v>65</v>
@@ -4508,7 +4508,7 @@
         <v>221</v>
       </c>
       <c r="B14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14">
         <v>17</v>
@@ -4548,7 +4548,7 @@
         <v>229</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C16">
         <v>14</v>
@@ -4568,7 +4568,7 @@
         <v>230</v>
       </c>
       <c r="B17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C17">
         <v>13</v>
@@ -4667,7 +4667,7 @@
         <v>411690</v>
       </c>
       <c r="B2">
-        <v>48.30107492611468</v>
+        <v>48.68164099146575</v>
       </c>
       <c r="C2">
         <v>27142</v>
@@ -4679,13 +4679,13 @@
         <v>9</v>
       </c>
       <c r="F2">
-        <v>2.42230633953743</v>
+        <v>2.403370092238899</v>
       </c>
       <c r="G2">
-        <v>2.003313340069452</v>
+        <v>1.987652547623504</v>
       </c>
       <c r="H2">
-        <v>2.90307057176576</v>
+        <v>2.8803759763817</v>
       </c>
       <c r="I2" t="s">
         <v>264</v>
@@ -4696,7 +4696,7 @@
         <v>410220</v>
       </c>
       <c r="B3">
-        <v>7.238728845986588</v>
+        <v>7.296072727773727</v>
       </c>
       <c r="C3">
         <v>4046</v>
@@ -4708,13 +4708,13 @@
         <v>10</v>
       </c>
       <c r="F3">
-        <v>1.795895422606922</v>
+        <v>1.781780484521942</v>
       </c>
       <c r="G3">
-        <v>0.9562386764689467</v>
+        <v>0.9487230664045091</v>
       </c>
       <c r="H3">
-        <v>3.071035867089317</v>
+        <v>3.046898893090133</v>
       </c>
       <c r="I3" t="s">
         <v>265</v>
@@ -4725,7 +4725,7 @@
         <v>412360</v>
       </c>
       <c r="B4">
-        <v>3.162009756399614</v>
+        <v>3.18825911295674</v>
       </c>
       <c r="C4">
         <v>1745</v>
@@ -4737,13 +4737,13 @@
         <v>11</v>
       </c>
       <c r="F4">
-        <v>1.581272793317751</v>
+        <v>1.568253966461051</v>
       </c>
       <c r="G4">
-        <v>0.5134349718031814</v>
+        <v>0.5092077941597493</v>
       </c>
       <c r="H4">
-        <v>3.690163212085936</v>
+        <v>3.659781613076499</v>
       </c>
       <c r="I4" t="s">
         <v>265</v>
@@ -4754,7 +4754,7 @@
         <v>412830</v>
       </c>
       <c r="B5">
-        <v>3.859117955902845</v>
+        <v>3.88876220296837</v>
       </c>
       <c r="C5">
         <v>2106</v>
@@ -4766,13 +4766,13 @@
         <v>12</v>
       </c>
       <c r="F5">
-        <v>1.554759421339401</v>
+        <v>1.542907405194403</v>
       </c>
       <c r="G5">
-        <v>0.5705693059013313</v>
+        <v>0.5662198248610061</v>
       </c>
       <c r="H5">
-        <v>3.384056712374682</v>
+        <v>3.358259862881337</v>
       </c>
       <c r="I5" t="s">
         <v>265</v>
@@ -4783,7 +4783,7 @@
         <v>411090</v>
       </c>
       <c r="B6">
-        <v>8.07658145790295</v>
+        <v>8.140656609503422</v>
       </c>
       <c r="C6">
         <v>4530</v>
@@ -4795,13 +4795,13 @@
         <v>14</v>
       </c>
       <c r="F6">
-        <v>1.361962367040387</v>
+        <v>1.3512423539839</v>
       </c>
       <c r="G6">
-        <v>0.6798867065054767</v>
+        <v>0.6745353146116548</v>
       </c>
       <c r="H6">
-        <v>2.436926887432435</v>
+        <v>2.417745822901447</v>
       </c>
       <c r="I6" t="s">
         <v>265</v>
@@ -4809,60 +4809,60 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7">
-        <v>411740</v>
+        <v>411520</v>
       </c>
       <c r="B7">
-        <v>5.936113581323124</v>
+        <v>725.2132960602268</v>
       </c>
       <c r="C7">
-        <v>3193</v>
+        <v>429660</v>
       </c>
       <c r="D7">
-        <v>8</v>
+        <v>977</v>
       </c>
       <c r="E7" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F7">
-        <v>1.347683107878952</v>
+        <v>1.347189861669143</v>
       </c>
       <c r="G7">
-        <v>0.581833910256593</v>
+        <v>1.26402810853362</v>
       </c>
       <c r="H7">
-        <v>2.655472979794264</v>
+        <v>1.434385619291172</v>
       </c>
       <c r="I7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8">
-        <v>411520</v>
+        <v>411740</v>
       </c>
       <c r="B8">
-        <v>719.6529728771376</v>
+        <v>5.98090565434091</v>
       </c>
       <c r="C8">
-        <v>429660</v>
+        <v>3193</v>
       </c>
       <c r="D8">
-        <v>967</v>
+        <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>1.343703196464236</v>
+        <v>1.337590067850952</v>
       </c>
       <c r="G8">
-        <v>1.260335721703425</v>
+        <v>0.5774764519553536</v>
       </c>
       <c r="H8">
-        <v>1.431136066593093</v>
+        <v>2.635585667323221</v>
       </c>
       <c r="I8" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -4870,7 +4870,7 @@
         <v>411640</v>
       </c>
       <c r="B9">
-        <v>6.162928197530854</v>
+        <v>6.212217174396419</v>
       </c>
       <c r="C9">
         <v>3669</v>
@@ -4879,16 +4879,16 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F9">
-        <v>1.298084245603439</v>
+        <v>1.28778498487978</v>
       </c>
       <c r="G9">
-        <v>0.5604206419494328</v>
+        <v>0.5559741521889207</v>
       </c>
       <c r="H9">
-        <v>2.557743448399862</v>
+        <v>2.537449798947969</v>
       </c>
       <c r="I9" t="s">
         <v>265</v>
@@ -4896,28 +4896,28 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10">
-        <v>412530</v>
+        <v>412450</v>
       </c>
       <c r="B10">
-        <v>9.939154525720845</v>
+        <v>11.97479580014789</v>
       </c>
       <c r="C10">
-        <v>5170</v>
+        <v>6463</v>
       </c>
       <c r="D10">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E10" t="s">
         <v>15</v>
       </c>
       <c r="F10">
-        <v>1.207346154941654</v>
+        <v>1.2526309634286</v>
       </c>
       <c r="G10">
-        <v>0.623853376328558</v>
+        <v>0.7010880413242314</v>
       </c>
       <c r="H10">
-        <v>2.108990759116576</v>
+        <v>2.06602428002825</v>
       </c>
       <c r="I10" t="s">
         <v>265</v>
@@ -4925,28 +4925,28 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11">
-        <v>412450</v>
+        <v>412530</v>
       </c>
       <c r="B11">
-        <v>11.88145064901948</v>
+        <v>10.0166756028254</v>
       </c>
       <c r="C11">
-        <v>6463</v>
+        <v>5170</v>
       </c>
       <c r="D11">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F11">
-        <v>1.178307297110674</v>
+        <v>1.198002259014474</v>
       </c>
       <c r="G11">
-        <v>0.6441915640100934</v>
+        <v>0.6190252489531777</v>
       </c>
       <c r="H11">
-        <v>1.976999426730276</v>
+        <v>2.092668853353334</v>
       </c>
       <c r="I11" t="s">
         <v>265</v>
@@ -4957,7 +4957,7 @@
         <v>410590</v>
       </c>
       <c r="B12">
-        <v>41.23722755044143</v>
+        <v>41.56425601710328</v>
       </c>
       <c r="C12">
         <v>23313</v>
@@ -4969,13 +4969,13 @@
         <v>19</v>
       </c>
       <c r="F12">
-        <v>1.066997046447391</v>
+        <v>1.058601890573825</v>
       </c>
       <c r="G12">
-        <v>0.7752816873791529</v>
+        <v>0.7691817542695532</v>
       </c>
       <c r="H12">
-        <v>1.432393732290944</v>
+        <v>1.421123627378339</v>
       </c>
       <c r="I12" t="s">
         <v>265</v>
@@ -4986,7 +4986,7 @@
         <v>411110</v>
       </c>
       <c r="B13">
-        <v>10.86470264763838</v>
+        <v>10.95255273804457</v>
       </c>
       <c r="C13">
         <v>6228</v>
@@ -4998,13 +4998,13 @@
         <v>20</v>
       </c>
       <c r="F13">
-        <v>0.9204117521038336</v>
+        <v>0.9130291576012411</v>
       </c>
       <c r="G13">
-        <v>0.4413732111826171</v>
+        <v>0.437832970160031</v>
       </c>
       <c r="H13">
-        <v>1.692669982644691</v>
+        <v>1.679093128503039</v>
       </c>
       <c r="I13" t="s">
         <v>265</v>
@@ -5015,7 +5015,7 @@
         <v>411480</v>
       </c>
       <c r="B14">
-        <v>77.69069147927273</v>
+        <v>78.29012495858673</v>
       </c>
       <c r="C14">
         <v>44749</v>
@@ -5027,13 +5027,13 @@
         <v>21</v>
       </c>
       <c r="F14">
-        <v>0.8495226228950258</v>
+        <v>0.8430181971853046</v>
       </c>
       <c r="G14">
-        <v>0.6570207350034915</v>
+        <v>0.6519902126308051</v>
       </c>
       <c r="H14">
-        <v>1.080801069519492</v>
+        <v>1.072525845206195</v>
       </c>
       <c r="I14" t="s">
         <v>265</v>
@@ -5044,7 +5044,7 @@
         <v>410780</v>
       </c>
       <c r="B15">
-        <v>9.713536080847046</v>
+        <v>9.790665115021525</v>
       </c>
       <c r="C15">
         <v>4805</v>
@@ -5056,13 +5056,13 @@
         <v>22</v>
       </c>
       <c r="F15">
-        <v>0.7206438460451553</v>
+        <v>0.7149667481997836</v>
       </c>
       <c r="G15">
-        <v>0.2897362019449509</v>
+        <v>0.2874537141712541</v>
       </c>
       <c r="H15">
-        <v>1.484801748988272</v>
+        <v>1.47310475767107</v>
       </c>
       <c r="I15" t="s">
         <v>265</v>
@@ -5073,25 +5073,25 @@
         <v>412625</v>
       </c>
       <c r="B16">
-        <v>209.2850121326406</v>
+        <v>210.8844048395926</v>
       </c>
       <c r="C16">
         <v>128106</v>
       </c>
       <c r="D16">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E16" t="s">
         <v>24</v>
       </c>
       <c r="F16">
-        <v>0.6928350889651953</v>
+        <v>0.6923224128927581</v>
       </c>
       <c r="G16">
-        <v>0.5846565411413399</v>
+        <v>0.5845788483251614</v>
       </c>
       <c r="H16">
-        <v>0.8152270746461704</v>
+        <v>0.8141703285310481</v>
       </c>
       <c r="I16" t="s">
         <v>266</v>
@@ -5102,7 +5102,7 @@
         <v>411810</v>
       </c>
       <c r="B17">
-        <v>16.27266485298788</v>
+        <v>16.39742250540482</v>
       </c>
       <c r="C17">
         <v>9549</v>
@@ -5114,13 +5114,13 @@
         <v>23</v>
       </c>
       <c r="F17">
-        <v>0.6759802465900506</v>
+        <v>0.6708371389695086</v>
       </c>
       <c r="G17">
-        <v>0.3374469035554792</v>
+        <v>0.3348794827618106</v>
       </c>
       <c r="H17">
-        <v>1.209515386146975</v>
+        <v>1.200312945941015</v>
       </c>
       <c r="I17" t="s">
         <v>265</v>
@@ -5131,7 +5131,7 @@
         <v>411360</v>
       </c>
       <c r="B18">
-        <v>7.783986307734082</v>
+        <v>7.843956877400136</v>
       </c>
       <c r="C18">
         <v>4707</v>
@@ -5143,13 +5143,13 @@
         <v>25</v>
       </c>
       <c r="F18">
-        <v>0.5138755185149343</v>
+        <v>0.5099467096160009</v>
       </c>
       <c r="G18">
-        <v>0.1400137834959251</v>
+        <v>0.1389433153012894</v>
       </c>
       <c r="H18">
-        <v>1.315725422747438</v>
+        <v>1.305666111565653</v>
       </c>
       <c r="I18" t="s">
         <v>265</v>
@@ -5160,7 +5160,7 @@
         <v>410210</v>
       </c>
       <c r="B19">
-        <v>48.55566975652325</v>
+        <v>48.93654898009187</v>
       </c>
       <c r="C19">
         <v>26203</v>
@@ -5172,13 +5172,13 @@
         <v>26</v>
       </c>
       <c r="F19">
-        <v>0.4118983447306498</v>
+        <v>0.4086924888826203</v>
       </c>
       <c r="G19">
-        <v>0.2515982097798724</v>
+        <v>0.2496399897421007</v>
       </c>
       <c r="H19">
-        <v>0.6361435864763223</v>
+        <v>0.6311924021295505</v>
       </c>
       <c r="I19" t="s">
         <v>266</v>
@@ -5189,7 +5189,7 @@
         <v>411630</v>
       </c>
       <c r="B20">
-        <v>8.031181483295246</v>
+        <v>8.093864286948808</v>
       </c>
       <c r="C20">
         <v>4057</v>
@@ -5201,13 +5201,13 @@
         <v>27</v>
       </c>
       <c r="F20">
-        <v>0.3735440428335434</v>
+        <v>0.3706511369158288</v>
       </c>
       <c r="G20">
-        <v>0.07703376199161124</v>
+        <v>0.07643717524312801</v>
       </c>
       <c r="H20">
-        <v>1.091654209032399</v>
+        <v>1.083199910317174</v>
       </c>
       <c r="I20" t="s">
         <v>265</v>
@@ -5218,7 +5218,7 @@
         <v>410790</v>
       </c>
       <c r="B21">
-        <v>20.44186950941049</v>
+        <v>20.59523462491628</v>
       </c>
       <c r="C21">
         <v>11522</v>
@@ -5230,13 +5230,13 @@
         <v>28</v>
       </c>
       <c r="F21">
-        <v>0.3424344332487556</v>
+        <v>0.339884450334513</v>
       </c>
       <c r="G21">
-        <v>0.1376764023576348</v>
+        <v>0.1366511769725132</v>
       </c>
       <c r="H21">
-        <v>0.7055458090593349</v>
+        <v>0.7002918696664766</v>
       </c>
       <c r="I21" t="s">
         <v>266</v>
@@ -5247,7 +5247,7 @@
         <v>411410</v>
       </c>
       <c r="B22">
-        <v>60.47964065424704</v>
+        <v>60.94675503204042</v>
       </c>
       <c r="C22">
         <v>34521</v>
@@ -5259,13 +5259,13 @@
         <v>29</v>
       </c>
       <c r="F22">
-        <v>0.3306897955022084</v>
+        <v>0.32815528881703</v>
       </c>
       <c r="G22">
-        <v>0.2019939181722976</v>
+        <v>0.2004457756443567</v>
       </c>
       <c r="H22">
-        <v>0.5107235686015197</v>
+        <v>0.5068092285870874</v>
       </c>
       <c r="I22" t="s">
         <v>266</v>
@@ -5276,7 +5276,7 @@
         <v>411750</v>
       </c>
       <c r="B23">
-        <v>81.38211863861062</v>
+        <v>82.00622491399278</v>
       </c>
       <c r="C23">
         <v>48695</v>
@@ -5288,13 +5288,13 @@
         <v>30</v>
       </c>
       <c r="F23">
-        <v>0.3071927890083104</v>
+        <v>0.3048549061515723</v>
       </c>
       <c r="G23">
-        <v>0.1987989759725127</v>
+        <v>0.1972860214550463</v>
       </c>
       <c r="H23">
-        <v>0.4534771558530221</v>
+        <v>0.4500259795672322</v>
       </c>
       <c r="I23" t="s">
         <v>266</v>
@@ -5305,7 +5305,7 @@
         <v>412040</v>
       </c>
       <c r="B24">
-        <v>7.185789935959376</v>
+        <v>7.24417855660043</v>
       </c>
       <c r="C24">
         <v>4304</v>
@@ -5317,16 +5317,16 @@
         <v>31</v>
       </c>
       <c r="F24">
-        <v>0.2783270896901023</v>
+        <v>0.2760837525433065</v>
       </c>
       <c r="G24">
-        <v>0.03370670179654055</v>
+        <v>0.03343502326061239</v>
       </c>
       <c r="H24">
-        <v>1.005413146238791</v>
+        <v>0.9973094411292897</v>
       </c>
       <c r="I24" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -5334,7 +5334,7 @@
         <v>412340</v>
       </c>
       <c r="B25">
-        <v>20.85835781950359</v>
+        <v>21.01882739615039</v>
       </c>
       <c r="C25">
         <v>11730</v>
@@ -5346,13 +5346,13 @@
         <v>32</v>
       </c>
       <c r="F25">
-        <v>0.239712063781203</v>
+        <v>0.237881966760703</v>
       </c>
       <c r="G25">
-        <v>0.07783385461919638</v>
+        <v>0.07723962709812078</v>
       </c>
       <c r="H25">
-        <v>0.5594079927237705</v>
+        <v>0.5551371567692559</v>
       </c>
       <c r="I25" t="s">
         <v>266</v>
@@ -5363,7 +5363,7 @@
         <v>411420</v>
       </c>
       <c r="B26">
-        <v>68.47329253981592</v>
+        <v>69.00689703929753</v>
       </c>
       <c r="C26">
         <v>38313</v>
@@ -5375,13 +5375,13 @@
         <v>33</v>
       </c>
       <c r="F26">
-        <v>0.2190635128474038</v>
+        <v>0.2173695767172072</v>
       </c>
       <c r="G26">
-        <v>0.1226081851971929</v>
+        <v>0.1216601020040413</v>
       </c>
       <c r="H26">
-        <v>0.3613119503067546</v>
+        <v>0.3585180602657292</v>
       </c>
       <c r="I26" t="s">
         <v>266</v>
@@ -5392,7 +5392,7 @@
         <v>411000</v>
       </c>
       <c r="B27">
-        <v>9.600329276281888</v>
+        <v>9.673871629905946</v>
       </c>
       <c r="C27">
         <v>5693</v>
@@ -5404,13 +5404,13 @@
         <v>35</v>
       </c>
       <c r="F27">
-        <v>0.2083261878257763</v>
+        <v>0.2067424580885662</v>
       </c>
       <c r="G27">
-        <v>0.0252292678275479</v>
+        <v>0.02503747080901876</v>
       </c>
       <c r="H27">
-        <v>0.7525458200244156</v>
+        <v>0.7468248436737008</v>
       </c>
       <c r="I27" t="s">
         <v>266</v>
@@ -5421,7 +5421,7 @@
         <v>410810</v>
       </c>
       <c r="B28">
-        <v>5.015891852603958</v>
+        <v>5.056021608135453</v>
       </c>
       <c r="C28">
         <v>2711</v>
@@ -5433,13 +5433,13 @@
         <v>34</v>
       </c>
       <c r="F28">
-        <v>0.199366339902416</v>
+        <v>0.1977839648451933</v>
       </c>
       <c r="G28">
-        <v>0.005047518712180038</v>
+        <v>0.005007456444322143</v>
       </c>
       <c r="H28">
-        <v>1.110798150092974</v>
+        <v>1.101981720563413</v>
       </c>
       <c r="I28" t="s">
         <v>265</v>
@@ -5450,7 +5450,7 @@
         <v>410115</v>
       </c>
       <c r="B29">
-        <v>6.187232173738672</v>
+        <v>6.235441077188169</v>
       </c>
       <c r="C29">
         <v>3357</v>
@@ -5462,13 +5462,13 @@
         <v>37</v>
       </c>
       <c r="F29">
-        <v>0.1616231574829919</v>
+        <v>0.1603735786484159</v>
       </c>
       <c r="G29">
-        <v>0.004091944066969034</v>
+        <v>0.004060307469974004</v>
       </c>
       <c r="H29">
-        <v>0.9005065972127889</v>
+        <v>0.8935443895576661</v>
       </c>
       <c r="I29" t="s">
         <v>266</v>
@@ -5479,7 +5479,7 @@
         <v>410730</v>
       </c>
       <c r="B30">
-        <v>12.82194342279607</v>
+        <v>12.92312217950379</v>
       </c>
       <c r="C30">
         <v>6517</v>
@@ -5491,13 +5491,13 @@
         <v>36</v>
       </c>
       <c r="F30">
-        <v>0.1559825943736586</v>
+        <v>0.1547613627898699</v>
       </c>
       <c r="G30">
-        <v>0.01889021582432988</v>
+        <v>0.0187423190139076</v>
       </c>
       <c r="H30">
-        <v>0.5634627629754799</v>
+        <v>0.5590512545940631</v>
       </c>
       <c r="I30" t="s">
         <v>266</v>
@@ -5508,7 +5508,7 @@
         <v>411160</v>
       </c>
       <c r="B31">
-        <v>4.908729112613215</v>
+        <v>4.946347687469058</v>
       </c>
       <c r="C31">
         <v>2685</v>
@@ -5526,7 +5526,7 @@
         <v>0</v>
       </c>
       <c r="H31">
-        <v>0.7514937918727645</v>
+        <v>0.7457784383938966</v>
       </c>
       <c r="I31" t="s">
         <v>266</v>
@@ -5558,10 +5558,10 @@
         <v>41</v>
       </c>
       <c r="B2">
-        <v>59.7</v>
+        <v>59.8</v>
       </c>
       <c r="C2">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5569,10 +5569,10 @@
         <v>42</v>
       </c>
       <c r="B3">
-        <v>60.2</v>
+        <v>60.3</v>
       </c>
       <c r="C3">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -5580,10 +5580,10 @@
         <v>43</v>
       </c>
       <c r="B4">
-        <v>60.2</v>
+        <v>60.3</v>
       </c>
       <c r="C4">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -5594,7 +5594,7 @@
         <v>60.3</v>
       </c>
       <c r="C5">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -5602,10 +5602,10 @@
         <v>45</v>
       </c>
       <c r="B6">
-        <v>91.7</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="C6">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -5613,10 +5613,10 @@
         <v>46</v>
       </c>
       <c r="B7">
-        <v>96.59999999999999</v>
+        <v>96.2</v>
       </c>
       <c r="C7">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -5624,10 +5624,10 @@
         <v>47</v>
       </c>
       <c r="B8">
-        <v>98.7</v>
+        <v>98.8</v>
       </c>
       <c r="C8">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -5635,10 +5635,10 @@
         <v>48</v>
       </c>
       <c r="B9">
-        <v>98.8</v>
+        <v>99</v>
       </c>
       <c r="C9">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -5646,10 +5646,10 @@
         <v>49</v>
       </c>
       <c r="B10">
-        <v>99.3</v>
+        <v>99.5</v>
       </c>
       <c r="C10">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -5660,7 +5660,7 @@
         <v>99.8</v>
       </c>
       <c r="C11">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -5671,7 +5671,7 @@
         <v>100</v>
       </c>
       <c r="C12">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -5682,7 +5682,7 @@
         <v>100</v>
       </c>
       <c r="C13">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -5693,7 +5693,7 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -5704,7 +5704,7 @@
         <v>100</v>
       </c>
       <c r="C15">
-        <v>1551</v>
+        <v>1563</v>
       </c>
     </row>
   </sheetData>
@@ -5733,10 +5733,10 @@
         <v>268</v>
       </c>
       <c r="B2">
-        <v>1505</v>
+        <v>1519</v>
       </c>
       <c r="C2">
-        <v>97</v>
+        <v>97.2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -5766,10 +5766,10 @@
         <v>271</v>
       </c>
       <c r="B5">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>
@@ -5810,10 +5810,10 @@
         <v>149</v>
       </c>
       <c r="D2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E2">
-        <v>40.3</v>
+        <v>40.4</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -5824,13 +5824,13 @@
         <v>276</v>
       </c>
       <c r="C3">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D3">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E3">
-        <v>59.2</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -5844,7 +5844,7 @@
         <v>2</v>
       </c>
       <c r="D4">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E4">
         <v>0.5</v>
@@ -5938,7 +5938,7 @@
         <v>276</v>
       </c>
       <c r="B3">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="C3">
         <v>41.7</v>
@@ -5949,10 +5949,10 @@
         <v>275</v>
       </c>
       <c r="B4">
-        <v>901</v>
+        <v>909</v>
       </c>
       <c r="C4">
-        <v>58.1</v>
+        <v>58.2</v>
       </c>
     </row>
   </sheetData>
@@ -5978,21 +5978,21 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2">
-        <v>461</v>
+        <v>466</v>
       </c>
       <c r="C2">
-        <v>29.7</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B3">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C3">
         <v>14.9</v>
@@ -6006,7 +6006,7 @@
         <v>199</v>
       </c>
       <c r="C4">
-        <v>12.8</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -6014,7 +6014,7 @@
         <v>59</v>
       </c>
       <c r="B5">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C5">
         <v>11.8</v>
@@ -6025,10 +6025,10 @@
         <v>60</v>
       </c>
       <c r="B6">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -6050,15 +6050,15 @@
         <v>38</v>
       </c>
       <c r="C8">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B9">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C9">
         <v>1.9</v>
@@ -6118,7 +6118,7 @@
         <v>66</v>
       </c>
       <c r="B2">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C2">
         <v>136</v>
@@ -6135,7 +6135,7 @@
         <v>67</v>
       </c>
       <c r="B3">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C3">
         <v>237</v>
@@ -6152,7 +6152,7 @@
         <v>68</v>
       </c>
       <c r="B4">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4">
         <v>31</v>
@@ -6189,7 +6189,7 @@
         <v>21</v>
       </c>
       <c r="C6">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -6220,7 +6220,7 @@
         <v>72</v>
       </c>
       <c r="B8">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8">
         <v>48</v>
@@ -6240,7 +6240,7 @@
         <v>106</v>
       </c>
       <c r="C9">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -6254,7 +6254,7 @@
         <v>74</v>
       </c>
       <c r="B10">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C10">
         <v>79</v>
@@ -6274,7 +6274,7 @@
         <v>138</v>
       </c>
       <c r="C11">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -6288,16 +6288,16 @@
         <v>76</v>
       </c>
       <c r="B12">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="C12">
-        <v>617</v>
+        <v>622</v>
       </c>
       <c r="D12">
         <v>91</v>
       </c>
       <c r="E12">
-        <v>14.7</v>
+        <v>14.6</v>
       </c>
     </row>
   </sheetData>
@@ -6329,13 +6329,13 @@
         <v>66</v>
       </c>
       <c r="B2">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C2">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2">
-        <v>45.3</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -6343,13 +6343,13 @@
         <v>67</v>
       </c>
       <c r="B3">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C3">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D3">
-        <v>21.3</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -6357,13 +6357,13 @@
         <v>68</v>
       </c>
       <c r="B4">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4">
         <v>7</v>
       </c>
       <c r="D4">
-        <v>20.6</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -6413,13 +6413,13 @@
         <v>72</v>
       </c>
       <c r="B8">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8">
         <v>20</v>
       </c>
       <c r="D8">
-        <v>39.2</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -6441,13 +6441,13 @@
         <v>74</v>
       </c>
       <c r="B10">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C10">
         <v>28</v>
       </c>
       <c r="D10">
-        <v>33.3</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -6469,13 +6469,13 @@
         <v>76</v>
       </c>
       <c r="B12">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="C12">
         <v>194</v>
       </c>
       <c r="D12">
-        <v>29.6</v>
+        <v>29.3</v>
       </c>
     </row>
   </sheetData>
@@ -6504,10 +6504,10 @@
         <v>79</v>
       </c>
       <c r="B2">
-        <v>891</v>
+        <v>897</v>
       </c>
       <c r="C2">
-        <v>99.2</v>
+        <v>99.40000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6515,10 +6515,10 @@
         <v>80</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6558,10 +6558,10 @@
         <v>83</v>
       </c>
       <c r="B2">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C2">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6569,10 +6569,10 @@
         <v>84</v>
       </c>
       <c r="B3">
-        <v>1159</v>
+        <v>1174</v>
       </c>
       <c r="C3">
-        <v>74.7</v>
+        <v>75.09999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6583,7 +6583,7 @@
         <v>374</v>
       </c>
       <c r="C4">
-        <v>24.1</v>
+        <v>23.9</v>
       </c>
     </row>
   </sheetData>
@@ -6612,10 +6612,10 @@
         <v>83</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -6623,10 +6623,10 @@
         <v>84</v>
       </c>
       <c r="B3">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C3">
-        <v>25.7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -6634,10 +6634,10 @@
         <v>85</v>
       </c>
       <c r="B4">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C4">
-        <v>73.8</v>
+        <v>73.7</v>
       </c>
     </row>
   </sheetData>
@@ -6716,7 +6716,7 @@
         <v>73.40000000000001</v>
       </c>
       <c r="E3">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F3">
         <v>106</v>

</xml_diff>